<commit_message>
Replaced "values for my sanity" with "coefficients." Cleaner.
</commit_message>
<xml_diff>
--- a/examples/F-16A B Block 10 and 15/Operator/F-16A Block 50.xlsx
+++ b/examples/F-16A B Block 10 and 15/Operator/F-16A Block 50.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\John Freeman\Desktop\Academics\VRMastersProgram\Tasks\Spring_2026\MATLAB\Design_Comparison\Operator\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\John Freeman\Desktop\Academics\VRMastersProgram\code\air-vehicle-design\examples\F-16A B Block 10 and 15\Operator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC03F7CC-F4D9-4BC1-9467-F3C88A03AFC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F20AAFCA-B61D-4A44-8428-FDB3206F7B4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="24480" yWindow="1488" windowWidth="21600" windowHeight="11508" activeTab="2" xr2:uid="{5F5D00AF-8D4A-4BC4-9FDA-F17071C88D94}"/>
+    <workbookView xWindow="22932" yWindow="384" windowWidth="23256" windowHeight="12720" activeTab="5" xr2:uid="{5F5D00AF-8D4A-4BC4-9FDA-F17071C88D94}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -181,9 +181,6 @@
     <t>Fw (ft)</t>
   </si>
   <si>
-    <t>Values for my sanity</t>
-  </si>
-  <si>
     <t>Bw</t>
   </si>
   <si>
@@ -503,6 +500,9 @@
   </si>
   <si>
     <t>Area (side) (ft^2)</t>
+  </si>
+  <si>
+    <t>Coefficients</t>
   </si>
 </sst>
 </file>
@@ -2290,7 +2290,7 @@
     </row>
     <row r="33" spans="2:14" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B33" s="5" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C33" s="12">
         <f>(1/6)*((1+2*C18)/(1+C18))</f>
@@ -2319,7 +2319,7 @@
     </row>
     <row r="34" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B34" s="5" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C34" s="12">
         <f>C33*C14</f>
@@ -2438,13 +2438,13 @@
     <row r="13" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B13" s="1"/>
       <c r="C13" s="6" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D13" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="F13" s="7"/>
       <c r="G13" s="7"/>
@@ -2540,7 +2540,7 @@
     </row>
     <row r="18" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B18" s="4" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C18" s="12"/>
       <c r="D18" s="12"/>
@@ -2557,7 +2557,7 @@
     </row>
     <row r="19" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B19" s="5" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C19" s="12"/>
       <c r="D19" s="12">
@@ -2580,7 +2580,7 @@
     </row>
     <row r="20" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B20" s="5" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C20" s="12"/>
       <c r="D20" s="12">
@@ -2910,7 +2910,7 @@
         <v>42</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="H13" s="7"/>
       <c r="I13" s="7"/>
@@ -3005,7 +3005,7 @@
     </row>
     <row r="19" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B19" s="5" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C19" s="12"/>
       <c r="D19" s="12"/>
@@ -3321,10 +3321,10 @@
         <v>34</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>46</v>
+        <v>153</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="F3" s="7"/>
       <c r="G3" s="7"/>
@@ -3395,7 +3395,7 @@
     </row>
     <row r="7" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B7" s="4" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C7" s="12"/>
       <c r="D7" s="12">
@@ -3414,7 +3414,7 @@
     </row>
     <row r="8" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B8" s="4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C8" s="12"/>
       <c r="D8" s="12">
@@ -3433,7 +3433,7 @@
     </row>
     <row r="9" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B9" s="4" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C9" s="12"/>
       <c r="D9" s="12">
@@ -3452,7 +3452,7 @@
     </row>
     <row r="10" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B10" s="4" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C10" s="12"/>
       <c r="D10" s="12">
@@ -3472,7 +3472,7 @@
     </row>
     <row r="11" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B11" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C11" s="12"/>
       <c r="D11" s="12">
@@ -3492,7 +3492,7 @@
     </row>
     <row r="12" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B12" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C12" s="12"/>
       <c r="D12" s="12">
@@ -3511,7 +3511,7 @@
     </row>
     <row r="13" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B13" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C13" s="12"/>
       <c r="D13" s="12">
@@ -3530,7 +3530,7 @@
     </row>
     <row r="14" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B14" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C14" s="12"/>
       <c r="D14" s="12">
@@ -3549,7 +3549,7 @@
     </row>
     <row r="15" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B15" s="5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C15" s="12"/>
       <c r="D15" s="12">
@@ -3569,7 +3569,7 @@
     </row>
     <row r="16" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B16" s="5" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C16" s="12"/>
       <c r="D16" s="12">
@@ -3589,7 +3589,7 @@
     </row>
     <row r="17" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B17" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C17" s="12"/>
       <c r="D17" s="12">
@@ -3609,7 +3609,7 @@
     </row>
     <row r="18" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B18" s="5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C18" s="12"/>
       <c r="D18" s="12">
@@ -3629,7 +3629,7 @@
     </row>
     <row r="19" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B19" s="5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C19" s="12"/>
       <c r="D19" s="12">
@@ -3648,7 +3648,7 @@
     </row>
     <row r="20" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B20" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C20" s="12"/>
       <c r="D20" s="12">
@@ -3667,7 +3667,7 @@
     </row>
     <row r="21" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B21" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C21" s="12"/>
       <c r="D21" s="12">
@@ -3686,7 +3686,7 @@
     </row>
     <row r="22" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B22" s="5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C22" s="12"/>
       <c r="D22" s="12">
@@ -3705,7 +3705,7 @@
     </row>
     <row r="23" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B23" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C23" s="12"/>
       <c r="D23" s="12">
@@ -3724,7 +3724,7 @@
     </row>
     <row r="24" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B24" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C24" s="12"/>
       <c r="D24" s="12">
@@ -3743,7 +3743,7 @@
     </row>
     <row r="25" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B25" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C25" s="12"/>
       <c r="D25" s="10">
@@ -3762,7 +3762,7 @@
     </row>
     <row r="26" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B26" s="5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C26" s="12"/>
       <c r="D26" s="10">
@@ -3781,7 +3781,7 @@
     </row>
     <row r="27" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B27" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C27" s="12"/>
       <c r="D27" s="10">
@@ -3800,7 +3800,7 @@
     </row>
     <row r="28" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B28" s="5" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C28" s="12"/>
       <c r="D28" s="10">
@@ -3819,7 +3819,7 @@
     </row>
     <row r="29" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B29" s="5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C29" s="12"/>
       <c r="D29" s="10">
@@ -3838,7 +3838,7 @@
     </row>
     <row r="30" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B30" s="5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C30" s="12"/>
       <c r="D30" s="10">
@@ -3857,7 +3857,7 @@
     </row>
     <row r="31" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B31" s="5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C31" s="12"/>
       <c r="D31" s="10">
@@ -3876,7 +3876,7 @@
     </row>
     <row r="32" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B32" s="17" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C32" s="12"/>
       <c r="D32" s="10">
@@ -3895,7 +3895,7 @@
     </row>
     <row r="33" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B33" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C33" s="12"/>
       <c r="D33" s="10">
@@ -3914,7 +3914,7 @@
     </row>
     <row r="34" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B34" s="4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C34" s="12"/>
       <c r="D34" s="10">
@@ -3933,7 +3933,7 @@
     </row>
     <row r="35" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B35" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C35" s="12"/>
       <c r="D35" s="10">
@@ -3952,7 +3952,7 @@
     </row>
     <row r="36" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B36" s="4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C36" s="12"/>
       <c r="D36" s="10">
@@ -3971,7 +3971,7 @@
     </row>
     <row r="37" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B37" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C37" s="12"/>
       <c r="D37" s="10">
@@ -3990,7 +3990,7 @@
     </row>
     <row r="38" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B38" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C38" s="12"/>
       <c r="D38" s="10">
@@ -4009,7 +4009,7 @@
     </row>
     <row r="39" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B39" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C39" s="12"/>
       <c r="D39" s="10">
@@ -4028,7 +4028,7 @@
     </row>
     <row r="40" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B40" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C40" s="12"/>
       <c r="D40" s="10">
@@ -4048,7 +4048,7 @@
     </row>
     <row r="41" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B41" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C41" s="12"/>
       <c r="D41" s="10">
@@ -4068,7 +4068,7 @@
     </row>
     <row r="42" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B42" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C42" s="12"/>
       <c r="D42" s="10">
@@ -4088,7 +4088,7 @@
     </row>
     <row r="43" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B43" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C43" s="12"/>
       <c r="D43" s="10">
@@ -4108,7 +4108,7 @@
     </row>
     <row r="44" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B44" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C44" s="12"/>
       <c r="D44" s="10">
@@ -4128,7 +4128,7 @@
     </row>
     <row r="45" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B45" s="4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C45" s="12"/>
       <c r="D45" s="10">
@@ -4147,7 +4147,7 @@
     </row>
     <row r="46" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B46" s="4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C46" s="12"/>
       <c r="D46" s="10">
@@ -4166,7 +4166,7 @@
     </row>
     <row r="47" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B47" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C47" s="12"/>
       <c r="D47" s="10">
@@ -4186,7 +4186,7 @@
     </row>
     <row r="48" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B48" s="4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C48" s="12"/>
       <c r="D48" s="10">
@@ -4206,7 +4206,7 @@
     </row>
     <row r="49" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B49" s="4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C49" s="12"/>
       <c r="D49" s="10">
@@ -4226,7 +4226,7 @@
     </row>
     <row r="50" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B50" s="4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C50" s="12"/>
       <c r="D50" s="10">
@@ -4246,7 +4246,7 @@
     </row>
     <row r="51" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B51" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C51" s="12"/>
       <c r="D51" s="10">
@@ -4265,7 +4265,7 @@
     </row>
     <row r="52" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B52" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C52" s="12"/>
       <c r="D52" s="10">
@@ -4285,7 +4285,7 @@
     </row>
     <row r="53" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B53" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C53" s="12"/>
       <c r="D53" s="10">
@@ -4305,7 +4305,7 @@
     </row>
     <row r="54" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B54" s="4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C54" s="12"/>
       <c r="D54" s="10">
@@ -4324,7 +4324,7 @@
     </row>
     <row r="55" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B55" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C55" s="12"/>
       <c r="D55" s="10">
@@ -4343,7 +4343,7 @@
     </row>
     <row r="56" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B56" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C56" s="12"/>
       <c r="D56" s="10">
@@ -4362,7 +4362,7 @@
     </row>
     <row r="57" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B57" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C57" s="12"/>
       <c r="D57" s="10">
@@ -4381,7 +4381,7 @@
     </row>
     <row r="58" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B58" s="4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C58" s="12"/>
       <c r="D58" s="10">
@@ -4400,7 +4400,7 @@
     </row>
     <row r="59" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B59" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C59" s="12"/>
       <c r="D59" s="10">
@@ -4419,7 +4419,7 @@
     </row>
     <row r="60" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B60" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C60" s="12"/>
       <c r="D60" s="10">
@@ -4438,7 +4438,7 @@
     </row>
     <row r="61" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B61" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C61" s="12"/>
       <c r="D61" s="10">
@@ -4458,7 +4458,7 @@
     </row>
     <row r="62" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B62" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C62" s="12"/>
       <c r="D62" s="10">
@@ -4477,7 +4477,7 @@
     </row>
     <row r="63" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B63" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C63" s="12"/>
       <c r="D63" s="10">
@@ -4496,7 +4496,7 @@
     </row>
     <row r="64" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B64" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C64" s="12"/>
       <c r="D64" s="10">
@@ -4515,7 +4515,7 @@
     </row>
     <row r="65" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B65" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C65" s="12"/>
       <c r="D65" s="10">
@@ -4534,7 +4534,7 @@
     </row>
     <row r="66" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B66" s="4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C66" s="12"/>
       <c r="D66" s="10">
@@ -4553,7 +4553,7 @@
     </row>
     <row r="67" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B67" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C67" s="12"/>
       <c r="D67" s="10">
@@ -4572,7 +4572,7 @@
     </row>
     <row r="68" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B68" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C68" s="12"/>
       <c r="D68" s="10">
@@ -4591,7 +4591,7 @@
     </row>
     <row r="69" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B69" s="4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C69" s="12"/>
       <c r="D69" s="10">
@@ -4610,7 +4610,7 @@
     </row>
     <row r="70" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B70" s="4" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C70" s="12"/>
       <c r="D70" s="10">
@@ -4629,7 +4629,7 @@
     </row>
     <row r="71" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B71" s="4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C71" s="12"/>
       <c r="D71" s="10">
@@ -4649,7 +4649,7 @@
     </row>
     <row r="72" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B72" s="4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C72" s="12"/>
       <c r="D72" s="10">
@@ -4669,7 +4669,7 @@
     </row>
     <row r="73" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B73" s="4" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C73" s="12"/>
       <c r="D73" s="10">
@@ -4688,7 +4688,7 @@
     </row>
     <row r="74" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B74" s="4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C74" s="12"/>
       <c r="D74" s="10">
@@ -4708,7 +4708,7 @@
     </row>
     <row r="75" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B75" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C75" s="12"/>
       <c r="D75" s="10">
@@ -4728,7 +4728,7 @@
     </row>
     <row r="76" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B76" s="4" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C76" s="12"/>
       <c r="D76" s="10">
@@ -4747,7 +4747,7 @@
     </row>
     <row r="77" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B77" s="4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C77" s="12"/>
       <c r="D77" s="10">
@@ -4766,7 +4766,7 @@
     </row>
     <row r="78" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B78" s="4" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C78" s="12"/>
       <c r="D78" s="10">
@@ -4785,7 +4785,7 @@
     </row>
     <row r="79" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B79" s="4" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C79" s="12"/>
       <c r="D79" s="10">
@@ -4805,7 +4805,7 @@
     </row>
     <row r="80" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B80" s="4" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C80" s="12"/>
       <c r="D80" s="10">
@@ -4824,7 +4824,7 @@
     </row>
     <row r="81" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B81" s="4" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C81" s="12"/>
       <c r="D81" s="10">
@@ -4843,7 +4843,7 @@
     </row>
     <row r="82" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B82" s="4" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C82" s="12"/>
       <c r="D82" s="10">
@@ -4862,7 +4862,7 @@
     </row>
     <row r="83" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B83" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C83" s="12"/>
       <c r="D83" s="10">
@@ -4881,7 +4881,7 @@
     </row>
     <row r="84" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B84" s="4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C84" s="12"/>
       <c r="D84" s="10">
@@ -4900,7 +4900,7 @@
     </row>
     <row r="85" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B85" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C85" s="12"/>
       <c r="D85" s="10">
@@ -4920,7 +4920,7 @@
     </row>
     <row r="86" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B86" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C86" s="12"/>
       <c r="D86" s="10">
@@ -4939,7 +4939,7 @@
     </row>
     <row r="87" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B87" s="4" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C87" s="12"/>
       <c r="D87" s="10">
@@ -4978,7 +4978,7 @@
     </row>
     <row r="89" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B89" s="4" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C89" s="12"/>
       <c r="D89" s="10">
@@ -4998,7 +4998,7 @@
     </row>
     <row r="90" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B90" s="4" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C90" s="12"/>
       <c r="D90" s="10">
@@ -5017,7 +5017,7 @@
     </row>
     <row r="91" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B91" s="4" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C91" s="12"/>
       <c r="D91" s="10">
@@ -5036,7 +5036,7 @@
     </row>
     <row r="92" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B92" s="4" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C92" s="12"/>
       <c r="D92" s="10">
@@ -5056,7 +5056,7 @@
     </row>
     <row r="93" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B93" s="4" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C93" s="12"/>
       <c r="D93" s="10">
@@ -5076,7 +5076,7 @@
     </row>
     <row r="94" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B94" s="4" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C94" s="12"/>
       <c r="D94" s="10">
@@ -5095,7 +5095,7 @@
     </row>
     <row r="95" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B95" s="4" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C95" s="12"/>
       <c r="D95" s="10">
@@ -5115,7 +5115,7 @@
     </row>
     <row r="96" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B96" s="4" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C96" s="12"/>
       <c r="D96" s="10">
@@ -5135,7 +5135,7 @@
     </row>
     <row r="97" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B97" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C97" s="12"/>
       <c r="D97" s="10">
@@ -5154,7 +5154,7 @@
     </row>
     <row r="98" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B98" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C98" s="12"/>
       <c r="D98" s="10">
@@ -5174,7 +5174,7 @@
     </row>
     <row r="99" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B99" s="4" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C99" s="12"/>
       <c r="D99" s="10">
@@ -5194,7 +5194,7 @@
     </row>
     <row r="100" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B100" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C100" s="12"/>
       <c r="D100" s="10">
@@ -5214,7 +5214,7 @@
     </row>
     <row r="101" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B101" s="4" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C101" s="12"/>
       <c r="D101" s="10">
@@ -5234,7 +5234,7 @@
     </row>
     <row r="102" spans="2:14" ht="30" x14ac:dyDescent="0.25">
       <c r="B102" s="4" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C102" s="12"/>
       <c r="D102" s="10">
@@ -5254,7 +5254,7 @@
     </row>
     <row r="103" spans="2:14" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B103" s="5" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C103" s="12"/>
       <c r="D103" s="10">
@@ -5274,7 +5274,7 @@
     </row>
     <row r="104" spans="2:14" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B104" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C104" s="12"/>
       <c r="D104" s="10">
@@ -5294,7 +5294,7 @@
     </row>
     <row r="105" spans="2:14" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B105" s="5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C105" s="12"/>
       <c r="D105" s="10">
@@ -5314,7 +5314,7 @@
     </row>
     <row r="106" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B106" s="5" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C106" s="12"/>
       <c r="D106" s="10"/>

</xml_diff>

<commit_message>
Missionanalysis now correctly uses GeometryStuff's "size_tail" and "get_S_wet" functions. Both those now produce acceptable values.
</commit_message>
<xml_diff>
--- a/examples/F-16A B Block 10 and 15/Operator/F-16A Block 50.xlsx
+++ b/examples/F-16A B Block 10 and 15/Operator/F-16A Block 50.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\John Freeman\Desktop\Academics\VRMastersProgram\code\air-vehicle-design\examples\F-16A B Block 10 and 15\Operator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F20AAFCA-B61D-4A44-8428-FDB3206F7B4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B742EA6-20FA-4369-BF7A-058D0E98EA44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="384" windowWidth="23256" windowHeight="12720" activeTab="5" xr2:uid="{5F5D00AF-8D4A-4BC4-9FDA-F17071C88D94}"/>
+    <workbookView xWindow="22932" yWindow="384" windowWidth="23256" windowHeight="12720" activeTab="4" xr2:uid="{5F5D00AF-8D4A-4BC4-9FDA-F17071C88D94}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Removed old "get_drag" function. Added "get_CD0" function (works).
</commit_message>
<xml_diff>
--- a/examples/F-16A B Block 10 and 15/Operator/F-16A Block 50.xlsx
+++ b/examples/F-16A B Block 10 and 15/Operator/F-16A Block 50.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\John Freeman\Desktop\Academics\VRMastersProgram\code\air-vehicle-design\examples\F-16A B Block 10 and 15\Operator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B742EA6-20FA-4369-BF7A-058D0E98EA44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC94930B-E524-4053-BC56-089E35F94CB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="384" windowWidth="23256" windowHeight="12720" activeTab="4" xr2:uid="{5F5D00AF-8D4A-4BC4-9FDA-F17071C88D94}"/>
+    <workbookView xWindow="22932" yWindow="384" windowWidth="23256" windowHeight="12720" activeTab="2" xr2:uid="{5F5D00AF-8D4A-4BC4-9FDA-F17071C88D94}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="155">
   <si>
     <t>THIS IS FOR THE END USER</t>
   </si>
@@ -503,6 +503,9 @@
   </si>
   <si>
     <t>Coefficients</t>
+  </si>
+  <si>
+    <t>x/c</t>
   </si>
 </sst>
 </file>
@@ -912,74 +915,6 @@
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -996,10 +931,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="0A0A0A"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FAFAFA"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="0E2841"/>
@@ -2347,10 +2282,18 @@
       <c r="N34" s="10"/>
     </row>
     <row r="35" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="5"/>
-      <c r="C35" s="12"/>
-      <c r="D35" s="10"/>
-      <c r="E35" s="10"/>
+      <c r="B35" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="C35" s="12">
+        <v>0.5</v>
+      </c>
+      <c r="D35" s="10">
+        <v>0.04</v>
+      </c>
+      <c r="E35" s="10">
+        <v>0.04</v>
+      </c>
       <c r="F35" s="10"/>
       <c r="G35" s="10"/>
       <c r="H35" s="10"/>

</xml_diff>

<commit_message>
Refactored some code. Simplified. Reorganized. Compute CD0 subsonic done.
</commit_message>
<xml_diff>
--- a/examples/F-16A B Block 10 and 15/Operator/F-16A Block 50.xlsx
+++ b/examples/F-16A B Block 10 and 15/Operator/F-16A Block 50.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\John Freeman\Desktop\Academics\VRMastersProgram\code\air-vehicle-design\examples\F-16A B Block 10 and 15\Operator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC94930B-E524-4053-BC56-089E35F94CB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4134956E-C43D-4079-B6CB-CAFF0D9292AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="384" windowWidth="23256" windowHeight="12720" activeTab="2" xr2:uid="{5F5D00AF-8D4A-4BC4-9FDA-F17071C88D94}"/>
+    <workbookView xWindow="22932" yWindow="384" windowWidth="23256" windowHeight="12720" activeTab="6" xr2:uid="{5F5D00AF-8D4A-4BC4-9FDA-F17071C88D94}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,8 @@
     <sheet name="Fuselage" sheetId="5" r:id="rId4"/>
     <sheet name="Propulsion" sheetId="7" r:id="rId5"/>
     <sheet name="Weights" sheetId="8" r:id="rId6"/>
+    <sheet name="Protuberances" sheetId="9" r:id="rId7"/>
+    <sheet name="Skin roughness" sheetId="10" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="176">
   <si>
     <t>THIS IS FOR THE END USER</t>
   </si>
@@ -506,6 +508,69 @@
   </si>
   <si>
     <t>x/c</t>
+  </si>
+  <si>
+    <t>Q</t>
+  </si>
+  <si>
+    <t>Y/N</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>Arresting hook</t>
+  </si>
+  <si>
+    <t>USAF</t>
+  </si>
+  <si>
+    <t>USAF/USN</t>
+  </si>
+  <si>
+    <t>Cannon port</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>k (m)</t>
+  </si>
+  <si>
+    <t>k (ft)</t>
+  </si>
+  <si>
+    <t>Camo paint on aluminum</t>
+  </si>
+  <si>
+    <t>Smooth paint</t>
+  </si>
+  <si>
+    <t>Production sheet metal</t>
+  </si>
+  <si>
+    <t>Polished sheet metal</t>
+  </si>
+  <si>
+    <t>Smooth molded composite</t>
+  </si>
+  <si>
+    <t>Exposed pilot - seated</t>
+  </si>
+  <si>
+    <t>Exposed pilot - spread eagle</t>
+  </si>
+  <si>
+    <t>Machine gun ports</t>
+  </si>
+  <si>
+    <t>D/q (ft^2)</t>
+  </si>
+  <si>
+    <t>D/q (m^2)</t>
+  </si>
+  <si>
+    <t>Exposed  pilot - prone</t>
   </si>
 </sst>
 </file>
@@ -767,7 +832,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -810,11 +875,54 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="14">
+  <dxfs count="20">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -1674,15 +1782,15 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="C14:N37">
-    <cfRule type="expression" dxfId="13" priority="2">
+    <cfRule type="expression" dxfId="19" priority="2">
       <formula>_xlfn.ISFORMULA(C14)</formula>
     </cfRule>
-    <cfRule type="containsBlanks" dxfId="12" priority="3">
+    <cfRule type="containsBlanks" dxfId="18" priority="3">
       <formula>LEN(TRIM(C14))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F23">
-    <cfRule type="expression" dxfId="11" priority="1">
+    <cfRule type="expression" dxfId="17" priority="1">
       <formula>ISNOTFORMULA(C14)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2305,11 +2413,21 @@
       <c r="N35" s="10"/>
     </row>
     <row r="36" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B36" s="5"/>
-      <c r="C36" s="12"/>
-      <c r="D36" s="10"/>
-      <c r="E36" s="10"/>
-      <c r="F36" s="10"/>
+      <c r="B36" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="C36" s="12">
+        <v>1</v>
+      </c>
+      <c r="D36" s="10">
+        <v>1</v>
+      </c>
+      <c r="E36" s="10">
+        <v>1</v>
+      </c>
+      <c r="F36" s="10">
+        <v>1</v>
+      </c>
       <c r="G36" s="10"/>
       <c r="H36" s="10"/>
       <c r="I36" s="10"/>
@@ -2336,13 +2454,13 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="C14:N37">
-    <cfRule type="expression" dxfId="10" priority="1">
+    <cfRule type="expression" dxfId="16" priority="1">
       <formula>ISNOTFORMULA(C14)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="9" priority="2">
+    <cfRule type="expression" dxfId="15" priority="2">
       <formula>_xlfn.ISFORMULA(C14)</formula>
     </cfRule>
-    <cfRule type="containsBlanks" dxfId="8" priority="3">
+    <cfRule type="containsBlanks" dxfId="14" priority="3">
       <formula>LEN(TRIM(C14))=0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2545,10 +2663,16 @@
       <c r="N20" s="10"/>
     </row>
     <row r="21" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="5"/>
+      <c r="B21" s="5" t="s">
+        <v>155</v>
+      </c>
       <c r="C21" s="12"/>
-      <c r="D21" s="12"/>
-      <c r="E21" s="12"/>
+      <c r="D21" s="12">
+        <v>1</v>
+      </c>
+      <c r="E21" s="12">
+        <v>1</v>
+      </c>
       <c r="F21" s="12"/>
       <c r="G21" s="10"/>
       <c r="H21" s="10"/>
@@ -2801,13 +2925,13 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="C14:N37">
-    <cfRule type="expression" dxfId="7" priority="1">
+    <cfRule type="expression" dxfId="13" priority="1">
       <formula>ISNOTFORMULA(C14)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="2">
+    <cfRule type="expression" dxfId="12" priority="2">
       <formula>_xlfn.ISFORMULA(C14)</formula>
     </cfRule>
-    <cfRule type="containsBlanks" dxfId="5" priority="3">
+    <cfRule type="containsBlanks" dxfId="11" priority="3">
       <formula>LEN(TRIM(C14))=0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3237,10 +3361,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="C14:N37">
-    <cfRule type="expression" dxfId="4" priority="2">
+    <cfRule type="expression" dxfId="10" priority="2">
       <formula>_xlfn.ISFORMULA(C14)</formula>
     </cfRule>
-    <cfRule type="containsBlanks" dxfId="3" priority="3">
+    <cfRule type="containsBlanks" dxfId="9" priority="3">
       <formula>LEN(TRIM(C14))=0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5277,18 +5401,919 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="C4:N106">
-    <cfRule type="expression" dxfId="2" priority="2">
+    <cfRule type="expression" dxfId="8" priority="2">
       <formula>_xlfn.ISFORMULA(C4)</formula>
     </cfRule>
-    <cfRule type="containsBlanks" dxfId="1" priority="3">
+    <cfRule type="containsBlanks" dxfId="7" priority="3">
       <formula>LEN(TRIM(C4))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F16:F17">
-    <cfRule type="expression" dxfId="0" priority="1">
+    <cfRule type="expression" dxfId="6" priority="1">
       <formula>ISNOTFORMULA(C3)</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{41AFF542-1B93-43EB-9BE7-8E21B1D3B06C}">
+  <dimension ref="D5:P34"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="5" spans="4:16" x14ac:dyDescent="0.25">
+      <c r="F5" s="14"/>
+    </row>
+    <row r="6" spans="4:16" x14ac:dyDescent="0.25">
+      <c r="F6" s="15"/>
+    </row>
+    <row r="7" spans="4:16" ht="31.5" x14ac:dyDescent="0.5">
+      <c r="D7" s="18"/>
+      <c r="F7" s="3"/>
+    </row>
+    <row r="8" spans="4:16" x14ac:dyDescent="0.25">
+      <c r="F8" s="16"/>
+    </row>
+    <row r="9" spans="4:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="10" spans="4:16" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D10" s="1"/>
+      <c r="E10" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="G10" s="7" t="s">
+        <v>173</v>
+      </c>
+      <c r="H10" s="7" t="s">
+        <v>174</v>
+      </c>
+      <c r="I10" s="7"/>
+      <c r="J10" s="7"/>
+      <c r="K10" s="7"/>
+      <c r="L10" s="7"/>
+      <c r="M10" s="7"/>
+      <c r="N10" s="7"/>
+      <c r="O10" s="7"/>
+      <c r="P10" s="8"/>
+    </row>
+    <row r="11" spans="4:16" ht="30" x14ac:dyDescent="0.25">
+      <c r="D11" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>157</v>
+      </c>
+      <c r="F11" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="G11" s="9">
+        <v>0.1</v>
+      </c>
+      <c r="H11" s="9">
+        <v>8.9999999999999993E-3</v>
+      </c>
+      <c r="I11" s="11"/>
+      <c r="J11" s="11"/>
+      <c r="K11" s="11"/>
+      <c r="L11" s="11"/>
+      <c r="M11" s="11"/>
+      <c r="N11" s="11"/>
+      <c r="O11" s="10"/>
+      <c r="P11" s="10"/>
+    </row>
+    <row r="12" spans="4:16" ht="45" x14ac:dyDescent="0.25">
+      <c r="D12" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="E12" s="12" t="s">
+        <v>162</v>
+      </c>
+      <c r="F12" s="12"/>
+      <c r="G12" s="12"/>
+      <c r="H12" s="12"/>
+      <c r="I12" s="12"/>
+      <c r="J12" s="12"/>
+      <c r="K12" s="12"/>
+      <c r="L12" s="10"/>
+      <c r="M12" s="10"/>
+      <c r="N12" s="10"/>
+      <c r="O12" s="10"/>
+      <c r="P12" s="10"/>
+    </row>
+    <row r="13" spans="4:16" ht="30" x14ac:dyDescent="0.25">
+      <c r="D13" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="E13" s="12" t="s">
+        <v>157</v>
+      </c>
+      <c r="F13" s="12"/>
+      <c r="G13" s="12">
+        <v>0.2</v>
+      </c>
+      <c r="H13" s="12">
+        <v>1.9E-2</v>
+      </c>
+      <c r="I13" s="12"/>
+      <c r="J13" s="12"/>
+      <c r="K13" s="12"/>
+      <c r="L13" s="10"/>
+      <c r="M13" s="10"/>
+      <c r="N13" s="10"/>
+      <c r="O13" s="10"/>
+      <c r="P13" s="10"/>
+    </row>
+    <row r="14" spans="4:16" ht="45" x14ac:dyDescent="0.25">
+      <c r="D14" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="E14" s="12" t="s">
+        <v>162</v>
+      </c>
+      <c r="F14" s="12"/>
+      <c r="G14" s="12"/>
+      <c r="H14" s="12"/>
+      <c r="I14" s="10"/>
+      <c r="J14" s="10"/>
+      <c r="K14" s="10"/>
+      <c r="L14" s="10"/>
+      <c r="M14" s="10"/>
+      <c r="N14" s="10"/>
+      <c r="O14" s="10"/>
+      <c r="P14" s="10"/>
+    </row>
+    <row r="15" spans="4:16" ht="45" x14ac:dyDescent="0.25">
+      <c r="D15" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="E15" s="12" t="s">
+        <v>162</v>
+      </c>
+      <c r="F15" s="12"/>
+      <c r="G15" s="12"/>
+      <c r="H15" s="12"/>
+      <c r="I15" s="10"/>
+      <c r="J15" s="10"/>
+      <c r="K15" s="10"/>
+      <c r="L15" s="10"/>
+      <c r="M15" s="10"/>
+      <c r="N15" s="10"/>
+      <c r="O15" s="10"/>
+      <c r="P15" s="10"/>
+    </row>
+    <row r="16" spans="4:16" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D16" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="E16" s="12" t="s">
+        <v>162</v>
+      </c>
+      <c r="F16" s="12"/>
+      <c r="G16" s="12"/>
+      <c r="H16" s="12"/>
+      <c r="I16" s="10"/>
+      <c r="J16" s="10"/>
+      <c r="K16" s="10"/>
+      <c r="L16" s="10"/>
+      <c r="M16" s="10"/>
+      <c r="N16" s="10"/>
+      <c r="O16" s="10"/>
+      <c r="P16" s="10"/>
+    </row>
+    <row r="17" spans="4:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D17" s="5"/>
+      <c r="E17" s="12"/>
+      <c r="F17" s="12"/>
+      <c r="G17" s="12"/>
+      <c r="H17" s="12"/>
+      <c r="I17" s="10"/>
+      <c r="J17" s="10"/>
+      <c r="K17" s="10"/>
+      <c r="L17" s="10"/>
+      <c r="M17" s="10"/>
+      <c r="N17" s="10"/>
+      <c r="O17" s="10"/>
+      <c r="P17" s="10"/>
+    </row>
+    <row r="18" spans="4:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D18" s="5"/>
+      <c r="E18" s="12"/>
+      <c r="F18" s="12"/>
+      <c r="G18" s="12"/>
+      <c r="H18" s="12"/>
+      <c r="I18" s="10"/>
+      <c r="J18" s="10"/>
+      <c r="K18" s="10"/>
+      <c r="L18" s="10"/>
+      <c r="M18" s="10"/>
+      <c r="N18" s="10"/>
+      <c r="O18" s="10"/>
+      <c r="P18" s="10"/>
+    </row>
+    <row r="19" spans="4:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D19" s="5"/>
+      <c r="E19" s="12"/>
+      <c r="F19" s="12"/>
+      <c r="G19" s="12"/>
+      <c r="H19" s="12"/>
+      <c r="I19" s="10"/>
+      <c r="J19" s="10"/>
+      <c r="K19" s="10"/>
+      <c r="L19" s="10"/>
+      <c r="M19" s="10"/>
+      <c r="N19" s="10"/>
+      <c r="O19" s="10"/>
+      <c r="P19" s="10"/>
+    </row>
+    <row r="20" spans="4:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D20" s="5"/>
+      <c r="E20" s="12"/>
+      <c r="F20" s="12"/>
+      <c r="G20" s="12"/>
+      <c r="H20" s="12"/>
+      <c r="I20" s="10"/>
+      <c r="J20" s="10"/>
+      <c r="K20" s="10"/>
+      <c r="L20" s="10"/>
+      <c r="M20" s="10"/>
+      <c r="N20" s="10"/>
+      <c r="O20" s="10"/>
+      <c r="P20" s="10"/>
+    </row>
+    <row r="21" spans="4:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D21" s="5"/>
+      <c r="E21" s="12"/>
+      <c r="F21" s="12"/>
+      <c r="G21" s="12"/>
+      <c r="H21" s="12"/>
+      <c r="I21" s="10"/>
+      <c r="J21" s="10"/>
+      <c r="K21" s="10"/>
+      <c r="L21" s="10"/>
+      <c r="M21" s="10"/>
+      <c r="N21" s="10"/>
+      <c r="O21" s="10"/>
+      <c r="P21" s="10"/>
+    </row>
+    <row r="22" spans="4:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D22" s="5"/>
+      <c r="E22" s="12"/>
+      <c r="F22" s="12"/>
+      <c r="G22" s="12"/>
+      <c r="H22" s="12"/>
+      <c r="I22" s="10"/>
+      <c r="J22" s="10"/>
+      <c r="K22" s="10"/>
+      <c r="L22" s="10"/>
+      <c r="M22" s="10"/>
+      <c r="N22" s="10"/>
+      <c r="O22" s="10"/>
+      <c r="P22" s="10"/>
+    </row>
+    <row r="23" spans="4:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D23" s="5"/>
+      <c r="E23" s="12"/>
+      <c r="F23" s="12"/>
+      <c r="G23" s="12"/>
+      <c r="H23" s="12"/>
+      <c r="I23" s="10"/>
+      <c r="J23" s="10"/>
+      <c r="K23" s="10"/>
+      <c r="L23" s="10"/>
+      <c r="M23" s="10"/>
+      <c r="N23" s="10"/>
+      <c r="O23" s="10"/>
+      <c r="P23" s="10"/>
+    </row>
+    <row r="24" spans="4:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D24" s="5"/>
+      <c r="E24" s="12"/>
+      <c r="F24" s="12"/>
+      <c r="G24" s="12"/>
+      <c r="H24" s="12"/>
+      <c r="I24" s="10"/>
+      <c r="J24" s="10"/>
+      <c r="K24" s="10"/>
+      <c r="L24" s="10"/>
+      <c r="M24" s="10"/>
+      <c r="N24" s="10"/>
+      <c r="O24" s="10"/>
+      <c r="P24" s="10"/>
+    </row>
+    <row r="25" spans="4:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D25" s="5"/>
+      <c r="E25" s="12"/>
+      <c r="F25" s="12"/>
+      <c r="G25" s="12"/>
+      <c r="H25" s="12"/>
+      <c r="I25" s="10"/>
+      <c r="J25" s="10"/>
+      <c r="K25" s="10"/>
+      <c r="L25" s="10"/>
+      <c r="M25" s="10"/>
+      <c r="N25" s="10"/>
+      <c r="O25" s="10"/>
+      <c r="P25" s="10"/>
+    </row>
+    <row r="26" spans="4:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D26" s="5"/>
+      <c r="E26" s="12"/>
+      <c r="F26" s="12"/>
+      <c r="G26" s="12"/>
+      <c r="H26" s="12"/>
+      <c r="I26" s="10"/>
+      <c r="J26" s="10"/>
+      <c r="K26" s="10"/>
+      <c r="L26" s="10"/>
+      <c r="M26" s="10"/>
+      <c r="N26" s="10"/>
+      <c r="O26" s="10"/>
+      <c r="P26" s="10"/>
+    </row>
+    <row r="27" spans="4:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D27" s="5"/>
+      <c r="E27" s="12"/>
+      <c r="F27" s="10"/>
+      <c r="G27" s="10"/>
+      <c r="H27" s="10"/>
+      <c r="I27" s="10"/>
+      <c r="J27" s="10"/>
+      <c r="K27" s="10"/>
+      <c r="L27" s="10"/>
+      <c r="M27" s="10"/>
+      <c r="N27" s="10"/>
+      <c r="O27" s="10"/>
+      <c r="P27" s="10"/>
+    </row>
+    <row r="28" spans="4:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D28" s="5"/>
+      <c r="E28" s="12"/>
+      <c r="F28" s="10"/>
+      <c r="G28" s="10"/>
+      <c r="H28" s="10"/>
+      <c r="I28" s="10"/>
+      <c r="J28" s="10"/>
+      <c r="K28" s="10"/>
+      <c r="L28" s="10"/>
+      <c r="M28" s="10"/>
+      <c r="N28" s="10"/>
+      <c r="O28" s="10"/>
+      <c r="P28" s="10"/>
+    </row>
+    <row r="29" spans="4:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D29" s="5"/>
+      <c r="E29" s="12"/>
+      <c r="F29" s="10"/>
+      <c r="G29" s="10"/>
+      <c r="H29" s="10"/>
+      <c r="I29" s="10"/>
+      <c r="J29" s="10"/>
+      <c r="K29" s="10"/>
+      <c r="L29" s="10"/>
+      <c r="M29" s="10"/>
+      <c r="N29" s="10"/>
+      <c r="O29" s="10"/>
+      <c r="P29" s="10"/>
+    </row>
+    <row r="30" spans="4:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D30" s="5"/>
+      <c r="E30" s="12"/>
+      <c r="F30" s="10"/>
+      <c r="G30" s="10"/>
+      <c r="H30" s="10"/>
+      <c r="I30" s="10"/>
+      <c r="J30" s="10"/>
+      <c r="K30" s="10"/>
+      <c r="L30" s="10"/>
+      <c r="M30" s="10"/>
+      <c r="N30" s="10"/>
+      <c r="O30" s="10"/>
+      <c r="P30" s="10"/>
+    </row>
+    <row r="31" spans="4:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D31" s="5"/>
+      <c r="E31" s="12"/>
+      <c r="F31" s="10"/>
+      <c r="G31" s="10"/>
+      <c r="H31" s="10"/>
+      <c r="I31" s="10"/>
+      <c r="J31" s="10"/>
+      <c r="K31" s="10"/>
+      <c r="L31" s="10"/>
+      <c r="M31" s="10"/>
+      <c r="N31" s="10"/>
+      <c r="O31" s="10"/>
+      <c r="P31" s="10"/>
+    </row>
+    <row r="32" spans="4:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D32" s="5"/>
+      <c r="E32" s="12"/>
+      <c r="F32" s="10"/>
+      <c r="G32" s="10"/>
+      <c r="H32" s="10"/>
+      <c r="I32" s="10"/>
+      <c r="J32" s="10"/>
+      <c r="K32" s="10"/>
+      <c r="L32" s="10"/>
+      <c r="M32" s="10"/>
+      <c r="N32" s="10"/>
+      <c r="O32" s="10"/>
+      <c r="P32" s="10"/>
+    </row>
+    <row r="33" spans="4:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D33" s="5"/>
+      <c r="E33" s="12"/>
+      <c r="F33" s="10"/>
+      <c r="G33" s="10"/>
+      <c r="H33" s="10"/>
+      <c r="I33" s="10"/>
+      <c r="J33" s="10"/>
+      <c r="K33" s="10"/>
+      <c r="L33" s="10"/>
+      <c r="M33" s="10"/>
+      <c r="N33" s="10"/>
+      <c r="O33" s="10"/>
+      <c r="P33" s="10"/>
+    </row>
+    <row r="34" spans="4:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D34" s="5"/>
+      <c r="E34" s="12"/>
+      <c r="F34" s="10"/>
+      <c r="G34" s="10"/>
+      <c r="H34" s="10"/>
+      <c r="I34" s="10"/>
+      <c r="J34" s="10"/>
+      <c r="K34" s="10"/>
+      <c r="L34" s="10"/>
+      <c r="M34" s="10"/>
+      <c r="N34" s="10"/>
+      <c r="O34" s="10"/>
+      <c r="P34" s="10"/>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="E11:P34">
+    <cfRule type="expression" dxfId="5" priority="2">
+      <formula>_xlfn.ISFORMULA(E11)</formula>
+    </cfRule>
+    <cfRule type="containsBlanks" dxfId="4" priority="3">
+      <formula>LEN(TRIM(E11))=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H20">
+    <cfRule type="expression" dxfId="3" priority="1">
+      <formula>ISNOTFORMULA(E11)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B886CA18-31EA-4ECA-BF44-35433BB56EEA}">
+  <dimension ref="C5:O30"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="4" max="4" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="5" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="6" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C6" s="1"/>
+      <c r="D6" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>163</v>
+      </c>
+      <c r="F6" s="7"/>
+      <c r="G6" s="7"/>
+      <c r="H6" s="7"/>
+      <c r="I6" s="7"/>
+      <c r="J6" s="7"/>
+      <c r="K6" s="7"/>
+      <c r="L6" s="7"/>
+      <c r="M6" s="7"/>
+      <c r="N6" s="7"/>
+      <c r="O6" s="8"/>
+    </row>
+    <row r="7" spans="3:15" ht="60" x14ac:dyDescent="0.25">
+      <c r="C7" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="D7" s="9">
+        <f>3.33*10^(-5)</f>
+        <v>3.3300000000000003E-5</v>
+      </c>
+      <c r="E7" s="9">
+        <f>1.015*10^(-5)</f>
+        <v>1.0149999999999999E-5</v>
+      </c>
+      <c r="F7" s="9"/>
+      <c r="G7" s="9"/>
+      <c r="H7" s="11"/>
+      <c r="I7" s="11"/>
+      <c r="J7" s="11"/>
+      <c r="K7" s="11"/>
+      <c r="L7" s="11"/>
+      <c r="M7" s="11"/>
+      <c r="N7" s="10"/>
+      <c r="O7" s="10"/>
+    </row>
+    <row r="8" spans="3:15" ht="30" x14ac:dyDescent="0.25">
+      <c r="C8" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="D8" s="12">
+        <f>2.08*10^(-5)</f>
+        <v>2.0800000000000001E-5</v>
+      </c>
+      <c r="E8" s="12">
+        <f>0.634*10^(-5)</f>
+        <v>6.3400000000000003E-6</v>
+      </c>
+      <c r="F8" s="12"/>
+      <c r="G8" s="12"/>
+      <c r="H8" s="12"/>
+      <c r="I8" s="12"/>
+      <c r="J8" s="12"/>
+      <c r="K8" s="10"/>
+      <c r="L8" s="10"/>
+      <c r="M8" s="10"/>
+      <c r="N8" s="10"/>
+      <c r="O8" s="10"/>
+    </row>
+    <row r="9" spans="3:15" ht="45" x14ac:dyDescent="0.25">
+      <c r="C9" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="D9" s="12">
+        <f>1.33*10^(-5)</f>
+        <v>1.3300000000000001E-5</v>
+      </c>
+      <c r="E9" s="12">
+        <f>0.405*10^(-5)</f>
+        <v>4.0500000000000002E-6</v>
+      </c>
+      <c r="F9" s="12"/>
+      <c r="G9" s="12"/>
+      <c r="H9" s="12"/>
+      <c r="I9" s="12"/>
+      <c r="J9" s="12"/>
+      <c r="K9" s="10"/>
+      <c r="L9" s="10"/>
+      <c r="M9" s="10"/>
+      <c r="N9" s="10"/>
+      <c r="O9" s="10"/>
+    </row>
+    <row r="10" spans="3:15" ht="45" x14ac:dyDescent="0.25">
+      <c r="C10" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="D10" s="12">
+        <f>0.5*10^(-5)</f>
+        <v>5.0000000000000004E-6</v>
+      </c>
+      <c r="E10" s="12">
+        <f>0.152*10^(-5)</f>
+        <v>1.5200000000000001E-6</v>
+      </c>
+      <c r="F10" s="12"/>
+      <c r="G10" s="12"/>
+      <c r="H10" s="10"/>
+      <c r="I10" s="10"/>
+      <c r="J10" s="10"/>
+      <c r="K10" s="10"/>
+      <c r="L10" s="10"/>
+      <c r="M10" s="10"/>
+      <c r="N10" s="10"/>
+      <c r="O10" s="10"/>
+    </row>
+    <row r="11" spans="3:15" ht="60" x14ac:dyDescent="0.25">
+      <c r="C11" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="D11" s="12">
+        <f>0.7*10^(-5)</f>
+        <v>6.9999999999999999E-6</v>
+      </c>
+      <c r="E11" s="12">
+        <f>0.052*10^(-5)</f>
+        <v>5.2E-7</v>
+      </c>
+      <c r="F11" s="12"/>
+      <c r="G11" s="12"/>
+      <c r="H11" s="10"/>
+      <c r="I11" s="10"/>
+      <c r="J11" s="10"/>
+      <c r="K11" s="10"/>
+      <c r="L11" s="10"/>
+      <c r="M11" s="10"/>
+      <c r="N11" s="10"/>
+      <c r="O11" s="10"/>
+    </row>
+    <row r="12" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C12" s="5"/>
+      <c r="D12" s="12"/>
+      <c r="E12" s="12"/>
+      <c r="F12" s="12"/>
+      <c r="G12" s="12"/>
+      <c r="H12" s="10"/>
+      <c r="I12" s="10"/>
+      <c r="J12" s="10"/>
+      <c r="K12" s="10"/>
+      <c r="L12" s="10"/>
+      <c r="M12" s="10"/>
+      <c r="N12" s="10"/>
+      <c r="O12" s="10"/>
+    </row>
+    <row r="13" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C13" s="5"/>
+      <c r="D13" s="12"/>
+      <c r="E13" s="12"/>
+      <c r="F13" s="12"/>
+      <c r="G13" s="12"/>
+      <c r="H13" s="10"/>
+      <c r="I13" s="10"/>
+      <c r="J13" s="10"/>
+      <c r="K13" s="10"/>
+      <c r="L13" s="10"/>
+      <c r="M13" s="10"/>
+      <c r="N13" s="10"/>
+      <c r="O13" s="10"/>
+    </row>
+    <row r="14" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C14" s="5"/>
+      <c r="D14" s="12"/>
+      <c r="E14" s="12"/>
+      <c r="F14" s="12"/>
+      <c r="G14" s="12"/>
+      <c r="H14" s="10"/>
+      <c r="I14" s="10"/>
+      <c r="J14" s="10"/>
+      <c r="K14" s="10"/>
+      <c r="L14" s="10"/>
+      <c r="M14" s="10"/>
+      <c r="N14" s="10"/>
+      <c r="O14" s="10"/>
+    </row>
+    <row r="15" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C15" s="5"/>
+      <c r="D15" s="12"/>
+      <c r="E15" s="12"/>
+      <c r="F15" s="12"/>
+      <c r="G15" s="12"/>
+      <c r="H15" s="10"/>
+      <c r="I15" s="10"/>
+      <c r="J15" s="10"/>
+      <c r="K15" s="10"/>
+      <c r="L15" s="10"/>
+      <c r="M15" s="10"/>
+      <c r="N15" s="10"/>
+      <c r="O15" s="10"/>
+    </row>
+    <row r="16" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C16" s="5"/>
+      <c r="D16" s="12"/>
+      <c r="E16" s="12"/>
+      <c r="F16" s="12"/>
+      <c r="G16" s="12"/>
+      <c r="H16" s="10"/>
+      <c r="I16" s="10"/>
+      <c r="J16" s="10"/>
+      <c r="K16" s="10"/>
+      <c r="L16" s="10"/>
+      <c r="M16" s="10"/>
+      <c r="N16" s="10"/>
+      <c r="O16" s="10"/>
+    </row>
+    <row r="17" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C17" s="5"/>
+      <c r="D17" s="12"/>
+      <c r="E17" s="12"/>
+      <c r="F17" s="12"/>
+      <c r="G17" s="12"/>
+      <c r="H17" s="10"/>
+      <c r="I17" s="10"/>
+      <c r="J17" s="10"/>
+      <c r="K17" s="10"/>
+      <c r="L17" s="10"/>
+      <c r="M17" s="10"/>
+      <c r="N17" s="10"/>
+      <c r="O17" s="10"/>
+    </row>
+    <row r="18" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C18" s="5"/>
+      <c r="D18" s="12"/>
+      <c r="E18" s="12"/>
+      <c r="F18" s="12"/>
+      <c r="G18" s="12"/>
+      <c r="H18" s="10"/>
+      <c r="I18" s="10"/>
+      <c r="J18" s="10"/>
+      <c r="K18" s="10"/>
+      <c r="L18" s="10"/>
+      <c r="M18" s="10"/>
+      <c r="N18" s="10"/>
+      <c r="O18" s="10"/>
+    </row>
+    <row r="19" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C19" s="5"/>
+      <c r="D19" s="12"/>
+      <c r="E19" s="12"/>
+      <c r="F19" s="12"/>
+      <c r="G19" s="12"/>
+      <c r="H19" s="10"/>
+      <c r="I19" s="10"/>
+      <c r="J19" s="10"/>
+      <c r="K19" s="10"/>
+      <c r="L19" s="10"/>
+      <c r="M19" s="10"/>
+      <c r="N19" s="10"/>
+      <c r="O19" s="10"/>
+    </row>
+    <row r="20" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C20" s="5"/>
+      <c r="D20" s="12"/>
+      <c r="E20" s="12"/>
+      <c r="F20" s="12"/>
+      <c r="G20" s="12"/>
+      <c r="H20" s="10"/>
+      <c r="I20" s="10"/>
+      <c r="J20" s="10"/>
+      <c r="K20" s="10"/>
+      <c r="L20" s="10"/>
+      <c r="M20" s="10"/>
+      <c r="N20" s="10"/>
+      <c r="O20" s="10"/>
+    </row>
+    <row r="21" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C21" s="5"/>
+      <c r="D21" s="12"/>
+      <c r="E21" s="12"/>
+      <c r="F21" s="12"/>
+      <c r="G21" s="12"/>
+      <c r="H21" s="10"/>
+      <c r="I21" s="10"/>
+      <c r="J21" s="10"/>
+      <c r="K21" s="10"/>
+      <c r="L21" s="10"/>
+      <c r="M21" s="10"/>
+      <c r="N21" s="10"/>
+      <c r="O21" s="10"/>
+    </row>
+    <row r="22" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C22" s="5"/>
+      <c r="D22" s="12"/>
+      <c r="E22" s="12"/>
+      <c r="F22" s="12"/>
+      <c r="G22" s="12"/>
+      <c r="H22" s="10"/>
+      <c r="I22" s="10"/>
+      <c r="J22" s="10"/>
+      <c r="K22" s="10"/>
+      <c r="L22" s="10"/>
+      <c r="M22" s="10"/>
+      <c r="N22" s="10"/>
+      <c r="O22" s="10"/>
+    </row>
+    <row r="23" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C23" s="5"/>
+      <c r="D23" s="12"/>
+      <c r="E23" s="10"/>
+      <c r="F23" s="10"/>
+      <c r="G23" s="10"/>
+      <c r="H23" s="10"/>
+      <c r="I23" s="10"/>
+      <c r="J23" s="10"/>
+      <c r="K23" s="10"/>
+      <c r="L23" s="10"/>
+      <c r="M23" s="10"/>
+      <c r="N23" s="10"/>
+      <c r="O23" s="10"/>
+    </row>
+    <row r="24" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C24" s="5"/>
+      <c r="D24" s="12"/>
+      <c r="E24" s="10"/>
+      <c r="F24" s="10"/>
+      <c r="G24" s="10"/>
+      <c r="H24" s="10"/>
+      <c r="I24" s="10"/>
+      <c r="J24" s="10"/>
+      <c r="K24" s="10"/>
+      <c r="L24" s="10"/>
+      <c r="M24" s="10"/>
+      <c r="N24" s="10"/>
+      <c r="O24" s="10"/>
+    </row>
+    <row r="25" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C25" s="5"/>
+      <c r="D25" s="12"/>
+      <c r="E25" s="10"/>
+      <c r="F25" s="10"/>
+      <c r="G25" s="10"/>
+      <c r="H25" s="10"/>
+      <c r="I25" s="10"/>
+      <c r="J25" s="10"/>
+      <c r="K25" s="10"/>
+      <c r="L25" s="10"/>
+      <c r="M25" s="10"/>
+      <c r="N25" s="10"/>
+      <c r="O25" s="10"/>
+    </row>
+    <row r="26" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C26" s="5"/>
+      <c r="D26" s="12"/>
+      <c r="E26" s="10"/>
+      <c r="F26" s="10"/>
+      <c r="G26" s="10"/>
+      <c r="H26" s="10"/>
+      <c r="I26" s="10"/>
+      <c r="J26" s="10"/>
+      <c r="K26" s="10"/>
+      <c r="L26" s="10"/>
+      <c r="M26" s="10"/>
+      <c r="N26" s="10"/>
+      <c r="O26" s="10"/>
+    </row>
+    <row r="27" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C27" s="5"/>
+      <c r="D27" s="12"/>
+      <c r="E27" s="10"/>
+      <c r="F27" s="10"/>
+      <c r="G27" s="10"/>
+      <c r="H27" s="10"/>
+      <c r="I27" s="10"/>
+      <c r="J27" s="10"/>
+      <c r="K27" s="10"/>
+      <c r="L27" s="10"/>
+      <c r="M27" s="10"/>
+      <c r="N27" s="10"/>
+      <c r="O27" s="10"/>
+    </row>
+    <row r="28" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C28" s="5"/>
+      <c r="D28" s="12"/>
+      <c r="E28" s="10"/>
+      <c r="F28" s="10"/>
+      <c r="G28" s="10"/>
+      <c r="H28" s="10"/>
+      <c r="I28" s="10"/>
+      <c r="J28" s="10"/>
+      <c r="K28" s="10"/>
+      <c r="L28" s="10"/>
+      <c r="M28" s="10"/>
+      <c r="N28" s="10"/>
+      <c r="O28" s="10"/>
+    </row>
+    <row r="29" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C29" s="5"/>
+      <c r="D29" s="12"/>
+      <c r="E29" s="10"/>
+      <c r="F29" s="10"/>
+      <c r="G29" s="10"/>
+      <c r="H29" s="10"/>
+      <c r="I29" s="10"/>
+      <c r="J29" s="10"/>
+      <c r="K29" s="10"/>
+      <c r="L29" s="10"/>
+      <c r="M29" s="10"/>
+      <c r="N29" s="10"/>
+      <c r="O29" s="10"/>
+    </row>
+    <row r="30" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C30" s="5"/>
+      <c r="D30" s="12"/>
+      <c r="E30" s="10"/>
+      <c r="F30" s="10"/>
+      <c r="G30" s="10"/>
+      <c r="H30" s="10"/>
+      <c r="I30" s="10"/>
+      <c r="J30" s="10"/>
+      <c r="K30" s="10"/>
+      <c r="L30" s="10"/>
+      <c r="M30" s="10"/>
+      <c r="N30" s="10"/>
+      <c r="O30" s="10"/>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="D7:O30">
+    <cfRule type="expression" dxfId="2" priority="2">
+      <formula>_xlfn.ISFORMULA(D7)</formula>
+    </cfRule>
+    <cfRule type="containsBlanks" dxfId="1" priority="3">
+      <formula>LEN(TRIM(D7))=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G16">
+    <cfRule type="expression" dxfId="0" priority="1">
+      <formula>ISNOTFORMULA(D7)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Completed drag results, CD, CDi, CL_minD, CL_alpha functions. Added "S_exposed" property to geometry class. Added some "airfoil types" to excel sheet wing geometry section.
</commit_message>
<xml_diff>
--- a/examples/F-16A B Block 10 and 15/Operator/F-16A Block 50.xlsx
+++ b/examples/F-16A B Block 10 and 15/Operator/F-16A Block 50.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\John Freeman\Desktop\Academics\VRMastersProgram\code\air-vehicle-design\examples\F-16A B Block 10 and 15\Operator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4134956E-C43D-4079-B6CB-CAFF0D9292AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D15AE803-AEC2-471B-B915-6B8E15C4F50E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="384" windowWidth="23256" windowHeight="12720" activeTab="6" xr2:uid="{5F5D00AF-8D4A-4BC4-9FDA-F17071C88D94}"/>
+    <workbookView xWindow="22932" yWindow="384" windowWidth="23256" windowHeight="12720" activeTab="2" xr2:uid="{5F5D00AF-8D4A-4BC4-9FDA-F17071C88D94}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="179">
   <si>
     <t>THIS IS FOR THE END USER</t>
   </si>
@@ -571,6 +571,15 @@
   </si>
   <si>
     <t>Exposed  pilot - prone</t>
+  </si>
+  <si>
+    <t>Airfoil type</t>
+  </si>
+  <si>
+    <t>cambered</t>
+  </si>
+  <si>
+    <t>uncambered</t>
   </si>
 </sst>
 </file>
@@ -2420,10 +2429,10 @@
         <v>1</v>
       </c>
       <c r="D36" s="10">
-        <v>1</v>
+        <v>1.05</v>
       </c>
       <c r="E36" s="10">
-        <v>1</v>
+        <v>1.05</v>
       </c>
       <c r="F36" s="10">
         <v>1</v>
@@ -2437,12 +2446,22 @@
       <c r="M36" s="10"/>
       <c r="N36" s="10"/>
     </row>
-    <row r="37" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B37" s="5"/>
-      <c r="C37" s="12"/>
-      <c r="D37" s="10"/>
-      <c r="E37" s="10"/>
-      <c r="F37" s="10"/>
+    <row r="37" spans="2:14" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B37" s="5" t="s">
+        <v>176</v>
+      </c>
+      <c r="C37" s="12" t="s">
+        <v>177</v>
+      </c>
+      <c r="D37" s="10" t="s">
+        <v>178</v>
+      </c>
+      <c r="E37" s="10" t="s">
+        <v>178</v>
+      </c>
+      <c r="F37" s="10" t="s">
+        <v>178</v>
+      </c>
       <c r="G37" s="10"/>
       <c r="H37" s="10"/>
       <c r="I37" s="10"/>

</xml_diff>

<commit_message>
Removed duplicate "sizing" class.
</commit_message>
<xml_diff>
--- a/examples/F-16A B Block 10 and 15/Operator/F-16A Block 50.xlsx
+++ b/examples/F-16A B Block 10 and 15/Operator/F-16A Block 50.xlsx
@@ -8,19 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\John Freeman\Desktop\Academics\VRMastersProgram\code\air-vehicle-design\examples\F-16A B Block 10 and 15\Operator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D15AE803-AEC2-471B-B915-6B8E15C4F50E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CD4089D-D1F3-45C8-AE47-66A44FEBA7F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="384" windowWidth="23256" windowHeight="12720" activeTab="2" xr2:uid="{5F5D00AF-8D4A-4BC4-9FDA-F17071C88D94}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="FORMAT" sheetId="6" r:id="rId2"/>
-    <sheet name="Wings" sheetId="2" r:id="rId3"/>
-    <sheet name="Fuselage" sheetId="5" r:id="rId4"/>
-    <sheet name="Propulsion" sheetId="7" r:id="rId5"/>
-    <sheet name="Weights" sheetId="8" r:id="rId6"/>
-    <sheet name="Protuberances" sheetId="9" r:id="rId7"/>
-    <sheet name="Skin roughness" sheetId="10" r:id="rId8"/>
+    <sheet name="General" sheetId="11" r:id="rId3"/>
+    <sheet name="Wings" sheetId="2" r:id="rId4"/>
+    <sheet name="Fuselage" sheetId="5" r:id="rId5"/>
+    <sheet name="Propulsion" sheetId="7" r:id="rId6"/>
+    <sheet name="Weights" sheetId="8" r:id="rId7"/>
+    <sheet name="Protuberances" sheetId="9" r:id="rId8"/>
+    <sheet name="Skin roughness" sheetId="10" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="191">
   <si>
     <t>THIS IS FOR THE END USER</t>
   </si>
@@ -531,6 +532,9 @@
     <t>Cannon port</t>
   </si>
   <si>
+    <t>Pilot</t>
+  </si>
+  <si>
     <t>N</t>
   </si>
   <si>
@@ -580,6 +584,39 @@
   </si>
   <si>
     <t>uncambered</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Fighter</t>
+  </si>
+  <si>
+    <t>Wing config</t>
+  </si>
+  <si>
+    <t>Delta</t>
+  </si>
+  <si>
+    <t>Engine count</t>
+  </si>
+  <si>
+    <t>General design choices</t>
+  </si>
+  <si>
+    <t>Aerodynamic</t>
+  </si>
+  <si>
+    <t>Propulsion</t>
+  </si>
+  <si>
+    <t>Weight</t>
+  </si>
+  <si>
+    <t>Sub/supersonic</t>
+  </si>
+  <si>
+    <t>Supersonic</t>
   </si>
 </sst>
 </file>
@@ -889,7 +926,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="20">
+  <dxfs count="25">
     <dxf>
       <fill>
         <patternFill>
@@ -1013,6 +1050,41 @@
       <fill>
         <patternFill>
           <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1791,15 +1863,15 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="C14:N37">
-    <cfRule type="expression" dxfId="19" priority="2">
+    <cfRule type="expression" dxfId="22" priority="2">
       <formula>_xlfn.ISFORMULA(C14)</formula>
     </cfRule>
-    <cfRule type="containsBlanks" dxfId="18" priority="3">
+    <cfRule type="containsBlanks" dxfId="21" priority="3">
       <formula>LEN(TRIM(C14))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F23">
-    <cfRule type="expression" dxfId="17" priority="1">
+    <cfRule type="expression" dxfId="20" priority="1">
       <formula>ISNOTFORMULA(C14)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1808,8 +1880,435 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09A3520D-A7E0-44C0-B29B-0A2440D0EA5F}">
+  <dimension ref="C4:O29"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="4" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="5" spans="3:15" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C5" s="1"/>
+      <c r="D5" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>186</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>187</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>188</v>
+      </c>
+      <c r="H5" s="7"/>
+      <c r="I5" s="7"/>
+      <c r="J5" s="7"/>
+      <c r="K5" s="7"/>
+      <c r="L5" s="7"/>
+      <c r="M5" s="7"/>
+      <c r="N5" s="7"/>
+      <c r="O5" s="8"/>
+    </row>
+    <row r="6" spans="3:15" x14ac:dyDescent="0.25">
+      <c r="C6" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>181</v>
+      </c>
+      <c r="E6" s="9"/>
+      <c r="F6" s="9"/>
+      <c r="G6" s="9"/>
+      <c r="H6" s="11"/>
+      <c r="I6" s="11"/>
+      <c r="J6" s="11"/>
+      <c r="K6" s="11"/>
+      <c r="L6" s="11"/>
+      <c r="M6" s="11"/>
+      <c r="N6" s="10"/>
+      <c r="O6" s="10"/>
+    </row>
+    <row r="7" spans="3:15" ht="30" x14ac:dyDescent="0.25">
+      <c r="C7" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="D7" s="12" t="s">
+        <v>183</v>
+      </c>
+      <c r="E7" s="12"/>
+      <c r="F7" s="12"/>
+      <c r="G7" s="12"/>
+      <c r="H7" s="12"/>
+      <c r="I7" s="12"/>
+      <c r="J7" s="12"/>
+      <c r="K7" s="10"/>
+      <c r="L7" s="10"/>
+      <c r="M7" s="10"/>
+      <c r="N7" s="10"/>
+      <c r="O7" s="10"/>
+    </row>
+    <row r="8" spans="3:15" ht="30" x14ac:dyDescent="0.25">
+      <c r="C8" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="D8" s="12">
+        <v>1</v>
+      </c>
+      <c r="E8" s="12"/>
+      <c r="F8" s="12"/>
+      <c r="G8" s="12"/>
+      <c r="H8" s="12"/>
+      <c r="I8" s="12"/>
+      <c r="J8" s="12"/>
+      <c r="K8" s="10"/>
+      <c r="L8" s="10"/>
+      <c r="M8" s="10"/>
+      <c r="N8" s="10"/>
+      <c r="O8" s="10"/>
+    </row>
+    <row r="9" spans="3:15" x14ac:dyDescent="0.25">
+      <c r="C9" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="D9" s="12">
+        <v>1</v>
+      </c>
+      <c r="E9" s="12"/>
+      <c r="F9" s="12"/>
+      <c r="G9" s="12"/>
+      <c r="H9" s="10"/>
+      <c r="I9" s="10"/>
+      <c r="J9" s="10"/>
+      <c r="K9" s="10"/>
+      <c r="L9" s="10"/>
+      <c r="M9" s="10"/>
+      <c r="N9" s="10"/>
+      <c r="O9" s="10"/>
+    </row>
+    <row r="10" spans="3:15" ht="30" x14ac:dyDescent="0.25">
+      <c r="C10" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="D10" s="12" t="s">
+        <v>190</v>
+      </c>
+      <c r="E10" s="12"/>
+      <c r="F10" s="12"/>
+      <c r="G10" s="12"/>
+      <c r="H10" s="10"/>
+      <c r="I10" s="10"/>
+      <c r="J10" s="10"/>
+      <c r="K10" s="10"/>
+      <c r="L10" s="10"/>
+      <c r="M10" s="10"/>
+      <c r="N10" s="10"/>
+      <c r="O10" s="10"/>
+    </row>
+    <row r="11" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C11" s="5"/>
+      <c r="D11" s="12"/>
+      <c r="E11" s="12"/>
+      <c r="F11" s="12"/>
+      <c r="G11" s="12"/>
+      <c r="H11" s="10"/>
+      <c r="I11" s="10"/>
+      <c r="J11" s="10"/>
+      <c r="K11" s="10"/>
+      <c r="L11" s="10"/>
+      <c r="M11" s="10"/>
+      <c r="N11" s="10"/>
+      <c r="O11" s="10"/>
+    </row>
+    <row r="12" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C12" s="5"/>
+      <c r="D12" s="12"/>
+      <c r="E12" s="12"/>
+      <c r="F12" s="12"/>
+      <c r="G12" s="12"/>
+      <c r="H12" s="10"/>
+      <c r="I12" s="10"/>
+      <c r="J12" s="10"/>
+      <c r="K12" s="10"/>
+      <c r="L12" s="10"/>
+      <c r="M12" s="10"/>
+      <c r="N12" s="10"/>
+      <c r="O12" s="10"/>
+    </row>
+    <row r="13" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C13" s="5"/>
+      <c r="D13" s="12"/>
+      <c r="E13" s="12"/>
+      <c r="F13" s="12"/>
+      <c r="G13" s="12"/>
+      <c r="H13" s="10"/>
+      <c r="I13" s="10"/>
+      <c r="J13" s="10"/>
+      <c r="K13" s="10"/>
+      <c r="L13" s="10"/>
+      <c r="M13" s="10"/>
+      <c r="N13" s="10"/>
+      <c r="O13" s="10"/>
+    </row>
+    <row r="14" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C14" s="5"/>
+      <c r="D14" s="12"/>
+      <c r="E14" s="12"/>
+      <c r="F14" s="12"/>
+      <c r="G14" s="12"/>
+      <c r="H14" s="10"/>
+      <c r="I14" s="10"/>
+      <c r="J14" s="10"/>
+      <c r="K14" s="10"/>
+      <c r="L14" s="10"/>
+      <c r="M14" s="10"/>
+      <c r="N14" s="10"/>
+      <c r="O14" s="10"/>
+    </row>
+    <row r="15" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C15" s="5"/>
+      <c r="D15" s="12"/>
+      <c r="E15" s="12"/>
+      <c r="F15" s="12"/>
+      <c r="G15" s="12"/>
+      <c r="H15" s="10"/>
+      <c r="I15" s="10"/>
+      <c r="J15" s="10"/>
+      <c r="K15" s="10"/>
+      <c r="L15" s="10"/>
+      <c r="M15" s="10"/>
+      <c r="N15" s="10"/>
+      <c r="O15" s="10"/>
+    </row>
+    <row r="16" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C16" s="5"/>
+      <c r="D16" s="12"/>
+      <c r="E16" s="12"/>
+      <c r="F16" s="12"/>
+      <c r="G16" s="12"/>
+      <c r="H16" s="10"/>
+      <c r="I16" s="10"/>
+      <c r="J16" s="10"/>
+      <c r="K16" s="10"/>
+      <c r="L16" s="10"/>
+      <c r="M16" s="10"/>
+      <c r="N16" s="10"/>
+      <c r="O16" s="10"/>
+    </row>
+    <row r="17" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C17" s="5"/>
+      <c r="D17" s="12"/>
+      <c r="E17" s="12"/>
+      <c r="F17" s="12"/>
+      <c r="G17" s="12"/>
+      <c r="H17" s="10"/>
+      <c r="I17" s="10"/>
+      <c r="J17" s="10"/>
+      <c r="K17" s="10"/>
+      <c r="L17" s="10"/>
+      <c r="M17" s="10"/>
+      <c r="N17" s="10"/>
+      <c r="O17" s="10"/>
+    </row>
+    <row r="18" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C18" s="5"/>
+      <c r="D18" s="12"/>
+      <c r="E18" s="12"/>
+      <c r="F18" s="12"/>
+      <c r="G18" s="12"/>
+      <c r="H18" s="10"/>
+      <c r="I18" s="10"/>
+      <c r="J18" s="10"/>
+      <c r="K18" s="10"/>
+      <c r="L18" s="10"/>
+      <c r="M18" s="10"/>
+      <c r="N18" s="10"/>
+      <c r="O18" s="10"/>
+    </row>
+    <row r="19" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C19" s="5"/>
+      <c r="D19" s="12"/>
+      <c r="E19" s="12"/>
+      <c r="F19" s="12"/>
+      <c r="G19" s="12"/>
+      <c r="H19" s="10"/>
+      <c r="I19" s="10"/>
+      <c r="J19" s="10"/>
+      <c r="K19" s="10"/>
+      <c r="L19" s="10"/>
+      <c r="M19" s="10"/>
+      <c r="N19" s="10"/>
+      <c r="O19" s="10"/>
+    </row>
+    <row r="20" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C20" s="5"/>
+      <c r="D20" s="12"/>
+      <c r="E20" s="12"/>
+      <c r="F20" s="12"/>
+      <c r="G20" s="12"/>
+      <c r="H20" s="10"/>
+      <c r="I20" s="10"/>
+      <c r="J20" s="10"/>
+      <c r="K20" s="10"/>
+      <c r="L20" s="10"/>
+      <c r="M20" s="10"/>
+      <c r="N20" s="10"/>
+      <c r="O20" s="10"/>
+    </row>
+    <row r="21" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C21" s="5"/>
+      <c r="D21" s="12"/>
+      <c r="E21" s="12"/>
+      <c r="F21" s="12"/>
+      <c r="G21" s="12"/>
+      <c r="H21" s="10"/>
+      <c r="I21" s="10"/>
+      <c r="J21" s="10"/>
+      <c r="K21" s="10"/>
+      <c r="L21" s="10"/>
+      <c r="M21" s="10"/>
+      <c r="N21" s="10"/>
+      <c r="O21" s="10"/>
+    </row>
+    <row r="22" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C22" s="5"/>
+      <c r="D22" s="12"/>
+      <c r="E22" s="10"/>
+      <c r="F22" s="10"/>
+      <c r="G22" s="10"/>
+      <c r="H22" s="10"/>
+      <c r="I22" s="10"/>
+      <c r="J22" s="10"/>
+      <c r="K22" s="10"/>
+      <c r="L22" s="10"/>
+      <c r="M22" s="10"/>
+      <c r="N22" s="10"/>
+      <c r="O22" s="10"/>
+    </row>
+    <row r="23" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C23" s="5"/>
+      <c r="D23" s="12"/>
+      <c r="E23" s="10"/>
+      <c r="F23" s="10"/>
+      <c r="G23" s="10"/>
+      <c r="H23" s="10"/>
+      <c r="I23" s="10"/>
+      <c r="J23" s="10"/>
+      <c r="K23" s="10"/>
+      <c r="L23" s="10"/>
+      <c r="M23" s="10"/>
+      <c r="N23" s="10"/>
+      <c r="O23" s="10"/>
+    </row>
+    <row r="24" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C24" s="5"/>
+      <c r="D24" s="12"/>
+      <c r="E24" s="10"/>
+      <c r="F24" s="10"/>
+      <c r="G24" s="10"/>
+      <c r="H24" s="10"/>
+      <c r="I24" s="10"/>
+      <c r="J24" s="10"/>
+      <c r="K24" s="10"/>
+      <c r="L24" s="10"/>
+      <c r="M24" s="10"/>
+      <c r="N24" s="10"/>
+      <c r="O24" s="10"/>
+    </row>
+    <row r="25" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C25" s="5"/>
+      <c r="D25" s="12"/>
+      <c r="E25" s="10"/>
+      <c r="F25" s="10"/>
+      <c r="G25" s="10"/>
+      <c r="H25" s="10"/>
+      <c r="I25" s="10"/>
+      <c r="J25" s="10"/>
+      <c r="K25" s="10"/>
+      <c r="L25" s="10"/>
+      <c r="M25" s="10"/>
+      <c r="N25" s="10"/>
+      <c r="O25" s="10"/>
+    </row>
+    <row r="26" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C26" s="5"/>
+      <c r="D26" s="12"/>
+      <c r="E26" s="10"/>
+      <c r="F26" s="10"/>
+      <c r="G26" s="10"/>
+      <c r="H26" s="10"/>
+      <c r="I26" s="10"/>
+      <c r="J26" s="10"/>
+      <c r="K26" s="10"/>
+      <c r="L26" s="10"/>
+      <c r="M26" s="10"/>
+      <c r="N26" s="10"/>
+      <c r="O26" s="10"/>
+    </row>
+    <row r="27" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C27" s="5"/>
+      <c r="D27" s="12"/>
+      <c r="E27" s="10"/>
+      <c r="F27" s="10"/>
+      <c r="G27" s="10"/>
+      <c r="H27" s="10"/>
+      <c r="I27" s="10"/>
+      <c r="J27" s="10"/>
+      <c r="K27" s="10"/>
+      <c r="L27" s="10"/>
+      <c r="M27" s="10"/>
+      <c r="N27" s="10"/>
+      <c r="O27" s="10"/>
+    </row>
+    <row r="28" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C28" s="5"/>
+      <c r="D28" s="12"/>
+      <c r="E28" s="10"/>
+      <c r="F28" s="10"/>
+      <c r="G28" s="10"/>
+      <c r="H28" s="10"/>
+      <c r="I28" s="10"/>
+      <c r="J28" s="10"/>
+      <c r="K28" s="10"/>
+      <c r="L28" s="10"/>
+      <c r="M28" s="10"/>
+      <c r="N28" s="10"/>
+      <c r="O28" s="10"/>
+    </row>
+    <row r="29" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C29" s="5"/>
+      <c r="D29" s="12"/>
+      <c r="E29" s="10"/>
+      <c r="F29" s="10"/>
+      <c r="G29" s="10"/>
+      <c r="H29" s="10"/>
+      <c r="I29" s="10"/>
+      <c r="J29" s="10"/>
+      <c r="K29" s="10"/>
+      <c r="L29" s="10"/>
+      <c r="M29" s="10"/>
+      <c r="N29" s="10"/>
+      <c r="O29" s="10"/>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="D6:O29">
+    <cfRule type="expression" dxfId="19" priority="2">
+      <formula>_xlfn.ISFORMULA(D6)</formula>
+    </cfRule>
+    <cfRule type="containsBlanks" dxfId="18" priority="3">
+      <formula>LEN(TRIM(D6))=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G15">
+    <cfRule type="expression" dxfId="17" priority="1">
+      <formula>ISNOTFORMULA(D6)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E23C0A35-DD33-4388-8FA3-25D5F19A7937}">
-  <dimension ref="B8:N37"/>
+  <dimension ref="B8:N40"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="19.7109375" customWidth="1"/>
@@ -2237,7 +2736,8 @@
         <v>13</v>
       </c>
       <c r="C28" s="12">
-        <v>0</v>
+        <f>-1.0469</f>
+        <v>-1.0468999999999999</v>
       </c>
       <c r="D28" s="12">
         <v>0</v>
@@ -2448,19 +2948,19 @@
     </row>
     <row r="37" spans="2:14" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B37" s="5" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C37" s="12" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="D37" s="10" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="E37" s="10" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="F37" s="10" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="G37" s="10"/>
       <c r="H37" s="10"/>
@@ -2471,8 +2971,53 @@
       <c r="M37" s="10"/>
       <c r="N37" s="10"/>
     </row>
+    <row r="38" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B38" s="5"/>
+      <c r="C38" s="12"/>
+      <c r="D38" s="10"/>
+      <c r="E38" s="10"/>
+      <c r="F38" s="10"/>
+      <c r="G38" s="10"/>
+      <c r="H38" s="10"/>
+      <c r="I38" s="10"/>
+      <c r="J38" s="10"/>
+      <c r="K38" s="10"/>
+      <c r="L38" s="10"/>
+      <c r="M38" s="10"/>
+      <c r="N38" s="10"/>
+    </row>
+    <row r="39" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B39" s="5"/>
+      <c r="C39" s="12"/>
+      <c r="D39" s="10"/>
+      <c r="E39" s="10"/>
+      <c r="F39" s="10"/>
+      <c r="G39" s="10"/>
+      <c r="H39" s="10"/>
+      <c r="I39" s="10"/>
+      <c r="J39" s="10"/>
+      <c r="K39" s="10"/>
+      <c r="L39" s="10"/>
+      <c r="M39" s="10"/>
+      <c r="N39" s="10"/>
+    </row>
+    <row r="40" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B40" s="5"/>
+      <c r="C40" s="12"/>
+      <c r="D40" s="10"/>
+      <c r="E40" s="10"/>
+      <c r="F40" s="10"/>
+      <c r="G40" s="10"/>
+      <c r="H40" s="10"/>
+      <c r="I40" s="10"/>
+      <c r="J40" s="10"/>
+      <c r="K40" s="10"/>
+      <c r="L40" s="10"/>
+      <c r="M40" s="10"/>
+      <c r="N40" s="10"/>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="C14:N37">
+  <conditionalFormatting sqref="C14:N40">
     <cfRule type="expression" dxfId="16" priority="1">
       <formula>ISNOTFORMULA(C14)</formula>
     </cfRule>
@@ -2490,7 +3035,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22430FBE-B769-4986-BB7E-BD6C15EED0AA}">
   <dimension ref="B8:N37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2958,7 +3503,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2BA581E-9024-402F-8C3F-057AD5928920}">
   <dimension ref="B8:N37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3391,7 +3936,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4AB1411D-9791-41D9-8EB0-13E6C33885B9}">
   <dimension ref="B2:N106"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -5436,7 +5981,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{41AFF542-1B93-43EB-9BE7-8E21B1D3B06C}">
   <dimension ref="D5:P34"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -5464,10 +6009,10 @@
         <v>160</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="H10" s="7" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="I10" s="7"/>
       <c r="J10" s="7"/>
@@ -5505,10 +6050,10 @@
     </row>
     <row r="12" spans="4:16" ht="45" x14ac:dyDescent="0.25">
       <c r="D12" s="4" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="E12" s="12" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="F12" s="12"/>
       <c r="G12" s="12"/>
@@ -5547,10 +6092,10 @@
     </row>
     <row r="14" spans="4:16" ht="45" x14ac:dyDescent="0.25">
       <c r="D14" s="4" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="E14" s="12" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="F14" s="12"/>
       <c r="G14" s="12"/>
@@ -5566,10 +6111,10 @@
     </row>
     <row r="15" spans="4:16" ht="45" x14ac:dyDescent="0.25">
       <c r="D15" s="4" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="E15" s="12" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="F15" s="12"/>
       <c r="G15" s="12"/>
@@ -5585,10 +6130,10 @@
     </row>
     <row r="16" spans="4:16" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D16" s="5" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="E16" s="12" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="F16" s="12"/>
       <c r="G16" s="12"/>
@@ -5890,7 +6435,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B886CA18-31EA-4ECA-BF44-35433BB56EEA}">
   <dimension ref="C5:O30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -5903,10 +6448,10 @@
     <row r="6" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C6" s="1"/>
       <c r="D6" s="6" t="s">
+        <v>165</v>
+      </c>
+      <c r="E6" s="7" t="s">
         <v>164</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>163</v>
       </c>
       <c r="F6" s="7"/>
       <c r="G6" s="7"/>
@@ -5921,7 +6466,7 @@
     </row>
     <row r="7" spans="3:15" ht="60" x14ac:dyDescent="0.25">
       <c r="C7" s="2" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D7" s="9">
         <f>3.33*10^(-5)</f>
@@ -5944,7 +6489,7 @@
     </row>
     <row r="8" spans="3:15" ht="30" x14ac:dyDescent="0.25">
       <c r="C8" s="4" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D8" s="12">
         <f>2.08*10^(-5)</f>
@@ -5967,7 +6512,7 @@
     </row>
     <row r="9" spans="3:15" ht="45" x14ac:dyDescent="0.25">
       <c r="C9" s="4" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D9" s="12">
         <f>1.33*10^(-5)</f>
@@ -5990,7 +6535,7 @@
     </row>
     <row r="10" spans="3:15" ht="45" x14ac:dyDescent="0.25">
       <c r="C10" s="4" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D10" s="12">
         <f>0.5*10^(-5)</f>
@@ -6013,7 +6558,7 @@
     </row>
     <row r="11" spans="3:15" ht="60" x14ac:dyDescent="0.25">
       <c r="C11" s="4" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D11" s="12">
         <f>0.7*10^(-5)</f>

</xml_diff>

<commit_message>
Consulted the dark lords regarding importing geometry (ChatGPT).
</commit_message>
<xml_diff>
--- a/examples/F-16A B Block 10 and 15/Operator/F-16A Block 50.xlsx
+++ b/examples/F-16A B Block 10 and 15/Operator/F-16A Block 50.xlsx
@@ -926,7 +926,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="25">
+  <dxfs count="23">
     <dxf>
       <fill>
         <patternFill>
@@ -1071,20 +1071,6 @@
       <fill>
         <patternFill>
           <bgColor theme="2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>

</xml_diff>

<commit_message>
Added function for computing S_exposed.
</commit_message>
<xml_diff>
--- a/examples/F-16A B Block 10 and 15/Operator/F-16A Block 50.xlsx
+++ b/examples/F-16A B Block 10 and 15/Operator/F-16A Block 50.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\John Freeman\Desktop\Academics\VRMastersProgram\code\air-vehicle-design\examples\F-16A B Block 10 and 15\Operator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CD4089D-D1F3-45C8-AE47-66A44FEBA7F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C331854-FB2E-4BD6-9589-0D70D2898147}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="384" windowWidth="23256" windowHeight="12720" activeTab="2" xr2:uid="{5F5D00AF-8D4A-4BC4-9FDA-F17071C88D94}"/>
+    <workbookView xWindow="22932" yWindow="384" windowWidth="23256" windowHeight="12720" activeTab="3" xr2:uid="{5F5D00AF-8D4A-4BC4-9FDA-F17071C88D94}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="193">
   <si>
     <t>THIS IS FOR THE END USER</t>
   </si>
@@ -617,6 +617,12 @@
   </si>
   <si>
     <t>Supersonic</t>
+  </si>
+  <si>
+    <t>Exposed root chord</t>
+  </si>
+  <si>
+    <t>Exposed half-span</t>
   </si>
 </sst>
 </file>
@@ -878,7 +884,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -921,7 +927,13 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1090,6 +1102,74 @@
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1106,10 +1186,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
+        <a:sysClr val="windowText" lastClr="0A0A0A"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
+        <a:sysClr val="window" lastClr="FAFAFA"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="0E2841"/>
@@ -2936,16 +3016,16 @@
       <c r="B37" s="5" t="s">
         <v>177</v>
       </c>
-      <c r="C37" s="12" t="s">
+      <c r="C37" s="19" t="s">
         <v>178</v>
       </c>
-      <c r="D37" s="10" t="s">
+      <c r="D37" s="20" t="s">
         <v>179</v>
       </c>
-      <c r="E37" s="10" t="s">
+      <c r="E37" s="20" t="s">
         <v>179</v>
       </c>
-      <c r="F37" s="10" t="s">
+      <c r="F37" s="20" t="s">
         <v>179</v>
       </c>
       <c r="G37" s="10"/>
@@ -2958,11 +3038,21 @@
       <c r="N37" s="10"/>
     </row>
     <row r="38" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B38" s="5"/>
-      <c r="C38" s="12"/>
-      <c r="D38" s="10"/>
-      <c r="E38" s="10"/>
-      <c r="F38" s="10"/>
+      <c r="B38" s="5" t="s">
+        <v>191</v>
+      </c>
+      <c r="C38" s="12">
+        <v>13.36</v>
+      </c>
+      <c r="D38" s="10">
+        <v>6.84</v>
+      </c>
+      <c r="E38" s="10">
+        <v>7.12</v>
+      </c>
+      <c r="F38" s="10">
+        <v>7.3</v>
+      </c>
       <c r="G38" s="10"/>
       <c r="H38" s="10"/>
       <c r="I38" s="10"/>
@@ -2973,11 +3063,21 @@
       <c r="N38" s="10"/>
     </row>
     <row r="39" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B39" s="5"/>
-      <c r="C39" s="12"/>
-      <c r="D39" s="10"/>
-      <c r="E39" s="10"/>
-      <c r="F39" s="10"/>
+      <c r="B39" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="C39" s="12">
+        <v>11.5</v>
+      </c>
+      <c r="D39" s="10">
+        <v>5.5</v>
+      </c>
+      <c r="E39" s="10">
+        <v>7.3</v>
+      </c>
+      <c r="F39" s="10">
+        <v>2.74</v>
+      </c>
       <c r="G39" s="10"/>
       <c r="H39" s="10"/>
       <c r="I39" s="10"/>

</xml_diff>

<commit_message>
Added constructors. Corrected S_wet and S_exposed computations.
</commit_message>
<xml_diff>
--- a/examples/F-16A B Block 10 and 15/Operator/F-16A Block 50.xlsx
+++ b/examples/F-16A B Block 10 and 15/Operator/F-16A Block 50.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\John Freeman\Desktop\Academics\VRMastersProgram\code\air-vehicle-design\examples\F-16A B Block 10 and 15\Operator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C331854-FB2E-4BD6-9589-0D70D2898147}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BEDC0E0-2383-4D43-B018-F698A043D518}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="384" windowWidth="23256" windowHeight="12720" activeTab="3" xr2:uid="{5F5D00AF-8D4A-4BC4-9FDA-F17071C88D94}"/>
+    <workbookView xWindow="22932" yWindow="384" windowWidth="23256" windowHeight="12720" firstSheet="1" activeTab="4" xr2:uid="{5F5D00AF-8D4A-4BC4-9FDA-F17071C88D94}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -178,9 +178,6 @@
     <t>Diameter (ft)</t>
   </si>
   <si>
-    <t>Structural depth (ft)</t>
-  </si>
-  <si>
     <t>Fw (ft)</t>
   </si>
   <si>
@@ -623,6 +620,9 @@
   </si>
   <si>
     <t>Exposed half-span</t>
+  </si>
+  <si>
+    <t>Max height (ft)</t>
   </si>
 </sst>
 </file>
@@ -1954,16 +1954,16 @@
     <row r="5" spans="3:15" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C5" s="1"/>
       <c r="D5" s="6" t="s">
+        <v>184</v>
+      </c>
+      <c r="E5" s="7" t="s">
         <v>185</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="F5" s="7" t="s">
         <v>186</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="G5" s="7" t="s">
         <v>187</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>188</v>
       </c>
       <c r="H5" s="7"/>
       <c r="I5" s="7"/>
@@ -1976,10 +1976,10 @@
     </row>
     <row r="6" spans="3:15" x14ac:dyDescent="0.25">
       <c r="C6" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="D6" s="9" t="s">
         <v>180</v>
-      </c>
-      <c r="D6" s="9" t="s">
-        <v>181</v>
       </c>
       <c r="E6" s="9"/>
       <c r="F6" s="9"/>
@@ -1995,10 +1995,10 @@
     </row>
     <row r="7" spans="3:15" ht="30" x14ac:dyDescent="0.25">
       <c r="C7" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="D7" s="12" t="s">
         <v>182</v>
-      </c>
-      <c r="D7" s="12" t="s">
-        <v>183</v>
       </c>
       <c r="E7" s="12"/>
       <c r="F7" s="12"/>
@@ -2014,7 +2014,7 @@
     </row>
     <row r="8" spans="3:15" ht="30" x14ac:dyDescent="0.25">
       <c r="C8" s="4" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D8" s="12">
         <v>1</v>
@@ -2033,7 +2033,7 @@
     </row>
     <row r="9" spans="3:15" x14ac:dyDescent="0.25">
       <c r="C9" s="4" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D9" s="12">
         <v>1</v>
@@ -2052,10 +2052,10 @@
     </row>
     <row r="10" spans="3:15" ht="30" x14ac:dyDescent="0.25">
       <c r="C10" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="D10" s="12" t="s">
         <v>189</v>
-      </c>
-      <c r="D10" s="12" t="s">
-        <v>190</v>
       </c>
       <c r="E10" s="12"/>
       <c r="F10" s="12"/>
@@ -2908,7 +2908,7 @@
     </row>
     <row r="33" spans="2:14" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B33" s="5" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C33" s="12">
         <f>(1/6)*((1+2*C18)/(1+C18))</f>
@@ -2937,7 +2937,7 @@
     </row>
     <row r="34" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B34" s="5" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C34" s="12">
         <f>C33*C14</f>
@@ -2966,7 +2966,7 @@
     </row>
     <row r="35" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B35" s="5" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C35" s="12">
         <v>0.5</v>
@@ -2989,7 +2989,7 @@
     </row>
     <row r="36" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B36" s="5" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C36" s="12">
         <v>1</v>
@@ -3014,19 +3014,19 @@
     </row>
     <row r="37" spans="2:14" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B37" s="5" t="s">
+        <v>176</v>
+      </c>
+      <c r="C37" s="19" t="s">
         <v>177</v>
       </c>
-      <c r="C37" s="19" t="s">
+      <c r="D37" s="20" t="s">
         <v>178</v>
       </c>
-      <c r="D37" s="20" t="s">
-        <v>179</v>
-      </c>
       <c r="E37" s="20" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="F37" s="20" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="G37" s="10"/>
       <c r="H37" s="10"/>
@@ -3039,7 +3039,7 @@
     </row>
     <row r="38" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B38" s="5" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C38" s="12">
         <v>13.36</v>
@@ -3064,7 +3064,7 @@
     </row>
     <row r="39" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B39" s="5" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C39" s="12">
         <v>11.5</v>
@@ -3149,13 +3149,13 @@
     <row r="13" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B13" s="1"/>
       <c r="C13" s="6" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D13" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F13" s="7"/>
       <c r="G13" s="7"/>
@@ -3217,10 +3217,12 @@
     </row>
     <row r="16" spans="2:14" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="4" t="s">
-        <v>44</v>
+        <v>192</v>
       </c>
       <c r="C16" s="12"/>
-      <c r="D16" s="12"/>
+      <c r="D16" s="12">
+        <v>5</v>
+      </c>
       <c r="E16" s="12"/>
       <c r="F16" s="12"/>
       <c r="G16" s="12"/>
@@ -3234,7 +3236,7 @@
     </row>
     <row r="17" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B17" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C17" s="12"/>
       <c r="D17" s="12"/>
@@ -3251,7 +3253,7 @@
     </row>
     <row r="18" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B18" s="4" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C18" s="12"/>
       <c r="D18" s="12"/>
@@ -3268,7 +3270,7 @@
     </row>
     <row r="19" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B19" s="5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C19" s="12"/>
       <c r="D19" s="12">
@@ -3291,7 +3293,7 @@
     </row>
     <row r="20" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B20" s="5" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C20" s="12"/>
       <c r="D20" s="12">
@@ -3314,7 +3316,7 @@
     </row>
     <row r="21" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B21" s="5" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C21" s="12"/>
       <c r="D21" s="12">
@@ -3627,7 +3629,7 @@
         <v>42</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="H13" s="7"/>
       <c r="I13" s="7"/>
@@ -3722,7 +3724,7 @@
     </row>
     <row r="19" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B19" s="5" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C19" s="12"/>
       <c r="D19" s="12"/>
@@ -4038,10 +4040,10 @@
         <v>34</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F3" s="7"/>
       <c r="G3" s="7"/>
@@ -4112,7 +4114,7 @@
     </row>
     <row r="7" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B7" s="4" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C7" s="12"/>
       <c r="D7" s="12">
@@ -4131,7 +4133,7 @@
     </row>
     <row r="8" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B8" s="4" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C8" s="12"/>
       <c r="D8" s="12">
@@ -4150,7 +4152,7 @@
     </row>
     <row r="9" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B9" s="4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C9" s="12"/>
       <c r="D9" s="12">
@@ -4169,7 +4171,7 @@
     </row>
     <row r="10" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B10" s="4" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C10" s="12"/>
       <c r="D10" s="12">
@@ -4189,7 +4191,7 @@
     </row>
     <row r="11" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B11" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C11" s="12"/>
       <c r="D11" s="12">
@@ -4209,7 +4211,7 @@
     </row>
     <row r="12" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B12" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C12" s="12"/>
       <c r="D12" s="12">
@@ -4228,7 +4230,7 @@
     </row>
     <row r="13" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B13" s="5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C13" s="12"/>
       <c r="D13" s="12">
@@ -4247,7 +4249,7 @@
     </row>
     <row r="14" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B14" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C14" s="12"/>
       <c r="D14" s="12">
@@ -4266,7 +4268,7 @@
     </row>
     <row r="15" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B15" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C15" s="12"/>
       <c r="D15" s="12">
@@ -4286,7 +4288,7 @@
     </row>
     <row r="16" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B16" s="5" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C16" s="12"/>
       <c r="D16" s="12">
@@ -4306,7 +4308,7 @@
     </row>
     <row r="17" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B17" s="5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C17" s="12"/>
       <c r="D17" s="12">
@@ -4326,7 +4328,7 @@
     </row>
     <row r="18" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B18" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C18" s="12"/>
       <c r="D18" s="12">
@@ -4346,7 +4348,7 @@
     </row>
     <row r="19" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B19" s="5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C19" s="12"/>
       <c r="D19" s="12">
@@ -4365,7 +4367,7 @@
     </row>
     <row r="20" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B20" s="5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C20" s="12"/>
       <c r="D20" s="12">
@@ -4384,7 +4386,7 @@
     </row>
     <row r="21" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B21" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C21" s="12"/>
       <c r="D21" s="12">
@@ -4403,7 +4405,7 @@
     </row>
     <row r="22" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B22" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C22" s="12"/>
       <c r="D22" s="12">
@@ -4422,7 +4424,7 @@
     </row>
     <row r="23" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B23" s="5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C23" s="12"/>
       <c r="D23" s="12">
@@ -4441,7 +4443,7 @@
     </row>
     <row r="24" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B24" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C24" s="12"/>
       <c r="D24" s="12">
@@ -4460,7 +4462,7 @@
     </row>
     <row r="25" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B25" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C25" s="12"/>
       <c r="D25" s="10">
@@ -4479,7 +4481,7 @@
     </row>
     <row r="26" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B26" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C26" s="12"/>
       <c r="D26" s="10">
@@ -4498,7 +4500,7 @@
     </row>
     <row r="27" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B27" s="5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C27" s="12"/>
       <c r="D27" s="10">
@@ -4517,7 +4519,7 @@
     </row>
     <row r="28" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B28" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C28" s="12"/>
       <c r="D28" s="10">
@@ -4536,7 +4538,7 @@
     </row>
     <row r="29" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B29" s="5" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C29" s="12"/>
       <c r="D29" s="10">
@@ -4555,7 +4557,7 @@
     </row>
     <row r="30" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B30" s="5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C30" s="12"/>
       <c r="D30" s="10">
@@ -4574,7 +4576,7 @@
     </row>
     <row r="31" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B31" s="5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C31" s="12"/>
       <c r="D31" s="10">
@@ -4593,7 +4595,7 @@
     </row>
     <row r="32" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B32" s="17" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C32" s="12"/>
       <c r="D32" s="10">
@@ -4612,7 +4614,7 @@
     </row>
     <row r="33" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B33" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C33" s="12"/>
       <c r="D33" s="10">
@@ -4631,7 +4633,7 @@
     </row>
     <row r="34" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B34" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C34" s="12"/>
       <c r="D34" s="10">
@@ -4650,7 +4652,7 @@
     </row>
     <row r="35" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B35" s="4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C35" s="12"/>
       <c r="D35" s="10">
@@ -4669,7 +4671,7 @@
     </row>
     <row r="36" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B36" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C36" s="12"/>
       <c r="D36" s="10">
@@ -4688,7 +4690,7 @@
     </row>
     <row r="37" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B37" s="4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C37" s="12"/>
       <c r="D37" s="10">
@@ -4707,7 +4709,7 @@
     </row>
     <row r="38" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B38" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C38" s="12"/>
       <c r="D38" s="10">
@@ -4726,7 +4728,7 @@
     </row>
     <row r="39" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B39" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C39" s="12"/>
       <c r="D39" s="10">
@@ -4745,7 +4747,7 @@
     </row>
     <row r="40" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B40" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C40" s="12"/>
       <c r="D40" s="10">
@@ -4765,7 +4767,7 @@
     </row>
     <row r="41" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B41" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C41" s="12"/>
       <c r="D41" s="10">
@@ -4785,7 +4787,7 @@
     </row>
     <row r="42" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B42" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C42" s="12"/>
       <c r="D42" s="10">
@@ -4805,7 +4807,7 @@
     </row>
     <row r="43" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B43" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C43" s="12"/>
       <c r="D43" s="10">
@@ -4825,7 +4827,7 @@
     </row>
     <row r="44" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B44" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C44" s="12"/>
       <c r="D44" s="10">
@@ -4845,7 +4847,7 @@
     </row>
     <row r="45" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B45" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C45" s="12"/>
       <c r="D45" s="10">
@@ -4864,7 +4866,7 @@
     </row>
     <row r="46" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B46" s="4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C46" s="12"/>
       <c r="D46" s="10">
@@ -4883,7 +4885,7 @@
     </row>
     <row r="47" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B47" s="4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C47" s="12"/>
       <c r="D47" s="10">
@@ -4903,7 +4905,7 @@
     </row>
     <row r="48" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B48" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C48" s="12"/>
       <c r="D48" s="10">
@@ -4923,7 +4925,7 @@
     </row>
     <row r="49" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B49" s="4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C49" s="12"/>
       <c r="D49" s="10">
@@ -4943,7 +4945,7 @@
     </row>
     <row r="50" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B50" s="4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C50" s="12"/>
       <c r="D50" s="10">
@@ -4963,7 +4965,7 @@
     </row>
     <row r="51" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B51" s="4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C51" s="12"/>
       <c r="D51" s="10">
@@ -4982,7 +4984,7 @@
     </row>
     <row r="52" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B52" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C52" s="12"/>
       <c r="D52" s="10">
@@ -5002,7 +5004,7 @@
     </row>
     <row r="53" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B53" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C53" s="12"/>
       <c r="D53" s="10">
@@ -5022,7 +5024,7 @@
     </row>
     <row r="54" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B54" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C54" s="12"/>
       <c r="D54" s="10">
@@ -5041,7 +5043,7 @@
     </row>
     <row r="55" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B55" s="4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C55" s="12"/>
       <c r="D55" s="10">
@@ -5060,7 +5062,7 @@
     </row>
     <row r="56" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B56" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C56" s="12"/>
       <c r="D56" s="10">
@@ -5079,7 +5081,7 @@
     </row>
     <row r="57" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B57" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C57" s="12"/>
       <c r="D57" s="10">
@@ -5098,7 +5100,7 @@
     </row>
     <row r="58" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B58" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C58" s="12"/>
       <c r="D58" s="10">
@@ -5117,7 +5119,7 @@
     </row>
     <row r="59" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B59" s="4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C59" s="12"/>
       <c r="D59" s="10">
@@ -5136,7 +5138,7 @@
     </row>
     <row r="60" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B60" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C60" s="12"/>
       <c r="D60" s="10">
@@ -5155,7 +5157,7 @@
     </row>
     <row r="61" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B61" s="4" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C61" s="12"/>
       <c r="D61" s="10">
@@ -5175,7 +5177,7 @@
     </row>
     <row r="62" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B62" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C62" s="12"/>
       <c r="D62" s="10">
@@ -5194,7 +5196,7 @@
     </row>
     <row r="63" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B63" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C63" s="12"/>
       <c r="D63" s="10">
@@ -5213,7 +5215,7 @@
     </row>
     <row r="64" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B64" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C64" s="12"/>
       <c r="D64" s="10">
@@ -5232,7 +5234,7 @@
     </row>
     <row r="65" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B65" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C65" s="12"/>
       <c r="D65" s="10">
@@ -5251,7 +5253,7 @@
     </row>
     <row r="66" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B66" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C66" s="12"/>
       <c r="D66" s="10">
@@ -5270,7 +5272,7 @@
     </row>
     <row r="67" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B67" s="4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C67" s="12"/>
       <c r="D67" s="10">
@@ -5289,7 +5291,7 @@
     </row>
     <row r="68" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B68" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C68" s="12"/>
       <c r="D68" s="10">
@@ -5308,7 +5310,7 @@
     </row>
     <row r="69" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B69" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C69" s="12"/>
       <c r="D69" s="10">
@@ -5327,7 +5329,7 @@
     </row>
     <row r="70" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B70" s="4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C70" s="12"/>
       <c r="D70" s="10">
@@ -5346,7 +5348,7 @@
     </row>
     <row r="71" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B71" s="4" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C71" s="12"/>
       <c r="D71" s="10">
@@ -5366,7 +5368,7 @@
     </row>
     <row r="72" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B72" s="4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C72" s="12"/>
       <c r="D72" s="10">
@@ -5386,7 +5388,7 @@
     </row>
     <row r="73" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B73" s="4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C73" s="12"/>
       <c r="D73" s="10">
@@ -5405,7 +5407,7 @@
     </row>
     <row r="74" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B74" s="4" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C74" s="12"/>
       <c r="D74" s="10">
@@ -5425,7 +5427,7 @@
     </row>
     <row r="75" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B75" s="4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C75" s="12"/>
       <c r="D75" s="10">
@@ -5445,7 +5447,7 @@
     </row>
     <row r="76" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B76" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C76" s="12"/>
       <c r="D76" s="10">
@@ -5464,7 +5466,7 @@
     </row>
     <row r="77" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B77" s="4" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C77" s="12"/>
       <c r="D77" s="10">
@@ -5483,7 +5485,7 @@
     </row>
     <row r="78" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B78" s="4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C78" s="12"/>
       <c r="D78" s="10">
@@ -5502,7 +5504,7 @@
     </row>
     <row r="79" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B79" s="4" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C79" s="12"/>
       <c r="D79" s="10">
@@ -5522,7 +5524,7 @@
     </row>
     <row r="80" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B80" s="4" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C80" s="12"/>
       <c r="D80" s="10">
@@ -5541,7 +5543,7 @@
     </row>
     <row r="81" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B81" s="4" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C81" s="12"/>
       <c r="D81" s="10">
@@ -5560,7 +5562,7 @@
     </row>
     <row r="82" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B82" s="4" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C82" s="12"/>
       <c r="D82" s="10">
@@ -5579,7 +5581,7 @@
     </row>
     <row r="83" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B83" s="4" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C83" s="12"/>
       <c r="D83" s="10">
@@ -5598,7 +5600,7 @@
     </row>
     <row r="84" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B84" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C84" s="12"/>
       <c r="D84" s="10">
@@ -5617,7 +5619,7 @@
     </row>
     <row r="85" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B85" s="4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C85" s="12"/>
       <c r="D85" s="10">
@@ -5637,7 +5639,7 @@
     </row>
     <row r="86" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B86" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C86" s="12"/>
       <c r="D86" s="10">
@@ -5656,7 +5658,7 @@
     </row>
     <row r="87" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B87" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C87" s="12"/>
       <c r="D87" s="10">
@@ -5695,7 +5697,7 @@
     </row>
     <row r="89" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B89" s="4" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C89" s="12"/>
       <c r="D89" s="10">
@@ -5715,7 +5717,7 @@
     </row>
     <row r="90" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B90" s="4" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C90" s="12"/>
       <c r="D90" s="10">
@@ -5734,7 +5736,7 @@
     </row>
     <row r="91" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B91" s="4" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C91" s="12"/>
       <c r="D91" s="10">
@@ -5753,7 +5755,7 @@
     </row>
     <row r="92" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B92" s="4" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C92" s="12"/>
       <c r="D92" s="10">
@@ -5773,7 +5775,7 @@
     </row>
     <row r="93" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B93" s="4" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C93" s="12"/>
       <c r="D93" s="10">
@@ -5793,7 +5795,7 @@
     </row>
     <row r="94" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B94" s="4" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C94" s="12"/>
       <c r="D94" s="10">
@@ -5812,7 +5814,7 @@
     </row>
     <row r="95" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B95" s="4" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C95" s="12"/>
       <c r="D95" s="10">
@@ -5832,7 +5834,7 @@
     </row>
     <row r="96" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B96" s="4" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C96" s="12"/>
       <c r="D96" s="10">
@@ -5852,7 +5854,7 @@
     </row>
     <row r="97" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B97" s="4" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C97" s="12"/>
       <c r="D97" s="10">
@@ -5871,7 +5873,7 @@
     </row>
     <row r="98" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B98" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C98" s="12"/>
       <c r="D98" s="10">
@@ -5891,7 +5893,7 @@
     </row>
     <row r="99" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B99" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C99" s="12"/>
       <c r="D99" s="10">
@@ -5911,7 +5913,7 @@
     </row>
     <row r="100" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B100" s="4" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C100" s="12"/>
       <c r="D100" s="10">
@@ -5931,7 +5933,7 @@
     </row>
     <row r="101" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B101" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C101" s="12"/>
       <c r="D101" s="10">
@@ -5951,7 +5953,7 @@
     </row>
     <row r="102" spans="2:14" ht="30" x14ac:dyDescent="0.25">
       <c r="B102" s="4" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C102" s="12"/>
       <c r="D102" s="10">
@@ -5971,7 +5973,7 @@
     </row>
     <row r="103" spans="2:14" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B103" s="5" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C103" s="12"/>
       <c r="D103" s="10">
@@ -5991,7 +5993,7 @@
     </row>
     <row r="104" spans="2:14" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B104" s="5" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C104" s="12"/>
       <c r="D104" s="10">
@@ -6011,7 +6013,7 @@
     </row>
     <row r="105" spans="2:14" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B105" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C105" s="12"/>
       <c r="D105" s="10">
@@ -6031,7 +6033,7 @@
     </row>
     <row r="106" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B106" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C106" s="12"/>
       <c r="D106" s="10"/>
@@ -6089,16 +6091,16 @@
     <row r="10" spans="4:16" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D10" s="1"/>
       <c r="E10" s="6" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="G10" s="7" t="s">
+        <v>173</v>
+      </c>
+      <c r="H10" s="7" t="s">
         <v>174</v>
-      </c>
-      <c r="H10" s="7" t="s">
-        <v>175</v>
       </c>
       <c r="I10" s="7"/>
       <c r="J10" s="7"/>
@@ -6111,13 +6113,13 @@
     </row>
     <row r="11" spans="4:16" ht="30" x14ac:dyDescent="0.25">
       <c r="D11" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>156</v>
+      </c>
+      <c r="F11" s="9" t="s">
         <v>158</v>
-      </c>
-      <c r="E11" s="9" t="s">
-        <v>157</v>
-      </c>
-      <c r="F11" s="9" t="s">
-        <v>159</v>
       </c>
       <c r="G11" s="9">
         <v>0.1</v>
@@ -6136,10 +6138,10 @@
     </row>
     <row r="12" spans="4:16" ht="45" x14ac:dyDescent="0.25">
       <c r="D12" s="4" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E12" s="12" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F12" s="12"/>
       <c r="G12" s="12"/>
@@ -6155,10 +6157,10 @@
     </row>
     <row r="13" spans="4:16" ht="30" x14ac:dyDescent="0.25">
       <c r="D13" s="4" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="E13" s="12" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="F13" s="12"/>
       <c r="G13" s="12">
@@ -6178,10 +6180,10 @@
     </row>
     <row r="14" spans="4:16" ht="45" x14ac:dyDescent="0.25">
       <c r="D14" s="4" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E14" s="12" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F14" s="12"/>
       <c r="G14" s="12"/>
@@ -6197,10 +6199,10 @@
     </row>
     <row r="15" spans="4:16" ht="45" x14ac:dyDescent="0.25">
       <c r="D15" s="4" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="E15" s="12" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F15" s="12"/>
       <c r="G15" s="12"/>
@@ -6216,10 +6218,10 @@
     </row>
     <row r="16" spans="4:16" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D16" s="5" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="E16" s="12" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F16" s="12"/>
       <c r="G16" s="12"/>
@@ -6534,10 +6536,10 @@
     <row r="6" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C6" s="1"/>
       <c r="D6" s="6" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F6" s="7"/>
       <c r="G6" s="7"/>
@@ -6552,7 +6554,7 @@
     </row>
     <row r="7" spans="3:15" ht="60" x14ac:dyDescent="0.25">
       <c r="C7" s="2" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D7" s="9">
         <f>3.33*10^(-5)</f>
@@ -6575,7 +6577,7 @@
     </row>
     <row r="8" spans="3:15" ht="30" x14ac:dyDescent="0.25">
       <c r="C8" s="4" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D8" s="12">
         <f>2.08*10^(-5)</f>
@@ -6598,7 +6600,7 @@
     </row>
     <row r="9" spans="3:15" ht="45" x14ac:dyDescent="0.25">
       <c r="C9" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D9" s="12">
         <f>1.33*10^(-5)</f>
@@ -6621,7 +6623,7 @@
     </row>
     <row r="10" spans="3:15" ht="45" x14ac:dyDescent="0.25">
       <c r="C10" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D10" s="12">
         <f>0.5*10^(-5)</f>
@@ -6644,7 +6646,7 @@
     </row>
     <row r="11" spans="3:15" ht="60" x14ac:dyDescent="0.25">
       <c r="C11" s="4" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D11" s="12">
         <f>0.7*10^(-5)</f>

</xml_diff>

<commit_message>
Added extraction for design type.
</commit_message>
<xml_diff>
--- a/examples/F-16A B Block 10 and 15/Operator/F-16A Block 50.xlsx
+++ b/examples/F-16A B Block 10 and 15/Operator/F-16A Block 50.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\John Freeman\Desktop\Academics\VRMastersProgram\code\air-vehicle-design\examples\F-16A B Block 10 and 15\Operator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BEDC0E0-2383-4D43-B018-F698A043D518}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C894285B-56CE-4448-B59E-725D39AEE1EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="384" windowWidth="23256" windowHeight="12720" firstSheet="1" activeTab="4" xr2:uid="{5F5D00AF-8D4A-4BC4-9FDA-F17071C88D94}"/>
+    <workbookView xWindow="22932" yWindow="384" windowWidth="23256" windowHeight="12720" firstSheet="1" activeTab="2" xr2:uid="{5F5D00AF-8D4A-4BC4-9FDA-F17071C88D94}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -586,9 +586,6 @@
     <t>Type</t>
   </si>
   <si>
-    <t>Fighter</t>
-  </si>
-  <si>
     <t>Wing config</t>
   </si>
   <si>
@@ -623,6 +620,9 @@
   </si>
   <si>
     <t>Max height (ft)</t>
+  </si>
+  <si>
+    <t>"Jet fighter"</t>
   </si>
 </sst>
 </file>
@@ -1186,10 +1186,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="0A0A0A"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FAFAFA"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="0E2841"/>
@@ -1954,16 +1954,16 @@
     <row r="5" spans="3:15" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C5" s="1"/>
       <c r="D5" s="6" t="s">
+        <v>183</v>
+      </c>
+      <c r="E5" s="7" t="s">
         <v>184</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="F5" s="7" t="s">
         <v>185</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="G5" s="7" t="s">
         <v>186</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>187</v>
       </c>
       <c r="H5" s="7"/>
       <c r="I5" s="7"/>
@@ -1974,12 +1974,12 @@
       <c r="N5" s="7"/>
       <c r="O5" s="8"/>
     </row>
-    <row r="6" spans="3:15" x14ac:dyDescent="0.25">
+    <row r="6" spans="3:15" ht="30" x14ac:dyDescent="0.25">
       <c r="C6" s="2" t="s">
         <v>179</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>180</v>
+        <v>192</v>
       </c>
       <c r="E6" s="9"/>
       <c r="F6" s="9"/>
@@ -1995,10 +1995,10 @@
     </row>
     <row r="7" spans="3:15" ht="30" x14ac:dyDescent="0.25">
       <c r="C7" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="D7" s="12" t="s">
         <v>181</v>
-      </c>
-      <c r="D7" s="12" t="s">
-        <v>182</v>
       </c>
       <c r="E7" s="12"/>
       <c r="F7" s="12"/>
@@ -2014,7 +2014,7 @@
     </row>
     <row r="8" spans="3:15" ht="30" x14ac:dyDescent="0.25">
       <c r="C8" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D8" s="12">
         <v>1</v>
@@ -2052,10 +2052,10 @@
     </row>
     <row r="10" spans="3:15" ht="30" x14ac:dyDescent="0.25">
       <c r="C10" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="D10" s="12" t="s">
         <v>188</v>
-      </c>
-      <c r="D10" s="12" t="s">
-        <v>189</v>
       </c>
       <c r="E10" s="12"/>
       <c r="F10" s="12"/>
@@ -3039,7 +3039,7 @@
     </row>
     <row r="38" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B38" s="5" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C38" s="12">
         <v>13.36</v>
@@ -3064,7 +3064,7 @@
     </row>
     <row r="39" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B39" s="5" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C39" s="12">
         <v>11.5</v>
@@ -3172,15 +3172,15 @@
         <v>10</v>
       </c>
       <c r="C14" s="9">
-        <v>48.43</v>
+        <v>46.5</v>
       </c>
       <c r="D14" s="9">
         <f>C14*(2/3)</f>
-        <v>32.286666666666662</v>
+        <v>31</v>
       </c>
       <c r="E14" s="9">
         <f>C14/3</f>
-        <v>16.143333333333334</v>
+        <v>15.5</v>
       </c>
       <c r="F14" s="9"/>
       <c r="G14" s="11"/>
@@ -3217,9 +3217,11 @@
     </row>
     <row r="16" spans="2:14" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="4" t="s">
-        <v>192</v>
-      </c>
-      <c r="C16" s="12"/>
+        <v>191</v>
+      </c>
+      <c r="C16" s="12">
+        <v>5</v>
+      </c>
       <c r="D16" s="12">
         <v>5</v>
       </c>
@@ -3275,11 +3277,11 @@
       <c r="C19" s="12"/>
       <c r="D19" s="12">
         <f>D14*D15</f>
-        <v>242.14999999999998</v>
+        <v>232.5</v>
       </c>
       <c r="E19" s="12">
         <f>(1/2)*E15*E14</f>
-        <v>56.501666666666672</v>
+        <v>54.25</v>
       </c>
       <c r="F19" s="12"/>
       <c r="G19" s="10"/>
@@ -3298,11 +3300,11 @@
       <c r="C20" s="12"/>
       <c r="D20" s="12">
         <f>D19</f>
-        <v>242.14999999999998</v>
+        <v>232.5</v>
       </c>
       <c r="E20" s="12">
         <f>E19</f>
-        <v>56.501666666666672</v>
+        <v>54.25</v>
       </c>
       <c r="F20" s="12"/>
       <c r="G20" s="10"/>
@@ -4333,7 +4335,7 @@
       <c r="C18" s="12"/>
       <c r="D18" s="12">
         <f>E106</f>
-        <v>104.90516395377779</v>
+        <v>100.61584000000002</v>
       </c>
       <c r="E18" s="12"/>
       <c r="F18" s="12"/>
@@ -4752,7 +4754,7 @@
       <c r="C40" s="12"/>
       <c r="D40" s="10">
         <f>0.75*((1+2*Wings!C18)/(1+Wings!C18))*(Wings!C14/D47)*(TAN(Wings!C15*PI()/180))</f>
-        <v>0.69322528764551838</v>
+        <v>0.72199786410048283</v>
       </c>
       <c r="E40" s="10"/>
       <c r="F40" s="10"/>
@@ -4812,7 +4814,7 @@
       <c r="C43" s="12"/>
       <c r="D43" s="10">
         <f>Fuselage!D14</f>
-        <v>32.286666666666662</v>
+        <v>31</v>
       </c>
       <c r="E43" s="10"/>
       <c r="F43" s="10"/>
@@ -4890,7 +4892,7 @@
       <c r="C47" s="12"/>
       <c r="D47" s="10">
         <f>Fuselage!D14</f>
-        <v>32.286666666666662</v>
+        <v>31</v>
       </c>
       <c r="E47" s="10"/>
       <c r="F47" s="10"/>
@@ -6039,7 +6041,7 @@
       <c r="D106" s="10"/>
       <c r="E106" s="10">
         <f>((D11+D47)/2)^2 * ((D54*0.52^2)/4)</f>
-        <v>104.90516395377779</v>
+        <v>100.61584000000002</v>
       </c>
       <c r="F106" s="10"/>
       <c r="G106" s="10"/>

</xml_diff>

<commit_message>
Incorporated "design type" into geometry estimations.
</commit_message>
<xml_diff>
--- a/examples/F-16A B Block 10 and 15/Operator/F-16A Block 50.xlsx
+++ b/examples/F-16A B Block 10 and 15/Operator/F-16A Block 50.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\John Freeman\Desktop\Academics\VRMastersProgram\code\air-vehicle-design\examples\F-16A B Block 10 and 15\Operator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C894285B-56CE-4448-B59E-725D39AEE1EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{553A142F-2700-4EF3-834A-8CD677FD10FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="384" windowWidth="23256" windowHeight="12720" firstSheet="1" activeTab="2" xr2:uid="{5F5D00AF-8D4A-4BC4-9FDA-F17071C88D94}"/>
+    <workbookView xWindow="22932" yWindow="384" windowWidth="23256" windowHeight="12720" firstSheet="1" activeTab="6" xr2:uid="{5F5D00AF-8D4A-4BC4-9FDA-F17071C88D94}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="194">
   <si>
     <t>THIS IS FOR THE END USER</t>
   </si>
@@ -623,6 +623,9 @@
   </si>
   <si>
     <t>"Jet fighter"</t>
+  </si>
+  <si>
+    <t>WTO_guess</t>
   </si>
 </sst>
 </file>
@@ -4028,7 +4031,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4AB1411D-9791-41D9-8EB0-13E6C33885B9}">
-  <dimension ref="B2:N106"/>
+  <dimension ref="B2:N107"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="11.5703125" bestFit="1" customWidth="1"/>
@@ -4114,14 +4117,14 @@
       <c r="M6" s="10"/>
       <c r="N6" s="10"/>
     </row>
-    <row r="7" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:14" ht="30" x14ac:dyDescent="0.25">
       <c r="B7" s="4" t="s">
-        <v>134</v>
-      </c>
-      <c r="C7" s="12"/>
-      <c r="D7" s="12">
-        <v>3</v>
-      </c>
+        <v>193</v>
+      </c>
+      <c r="C7" s="12">
+        <v>45000</v>
+      </c>
+      <c r="D7" s="12"/>
       <c r="E7" s="12"/>
       <c r="F7" s="12"/>
       <c r="G7" s="12"/>
@@ -4135,7 +4138,7 @@
     </row>
     <row r="8" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B8" s="4" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C8" s="12"/>
       <c r="D8" s="12">
@@ -4154,11 +4157,11 @@
     </row>
     <row r="9" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B9" s="4" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C9" s="12"/>
       <c r="D9" s="12">
-        <v>1.6</v>
+        <v>3</v>
       </c>
       <c r="E9" s="12"/>
       <c r="F9" s="12"/>
@@ -4173,12 +4176,11 @@
     </row>
     <row r="10" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B10" s="4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C10" s="12"/>
       <c r="D10" s="12">
-        <f>Wings!D14</f>
-        <v>18</v>
+        <v>1.6</v>
       </c>
       <c r="E10" s="12"/>
       <c r="F10" s="12"/>
@@ -4193,12 +4195,12 @@
     </row>
     <row r="11" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B11" s="4" t="s">
-        <v>45</v>
+        <v>137</v>
       </c>
       <c r="C11" s="12"/>
       <c r="D11" s="12">
-        <f>Wings!C14</f>
-        <v>30</v>
+        <f>Wings!D14</f>
+        <v>18</v>
       </c>
       <c r="E11" s="12"/>
       <c r="F11" s="12"/>
@@ -4213,11 +4215,12 @@
     </row>
     <row r="12" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B12" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C12" s="12"/>
       <c r="D12" s="12">
-        <v>7.5</v>
+        <f>Wings!C14</f>
+        <v>30</v>
       </c>
       <c r="E12" s="12"/>
       <c r="F12" s="12"/>
@@ -4230,13 +4233,13 @@
       <c r="M12" s="10"/>
       <c r="N12" s="10"/>
     </row>
-    <row r="13" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="5" t="s">
-        <v>47</v>
+    <row r="13" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B13" s="4" t="s">
+        <v>46</v>
       </c>
       <c r="C13" s="12"/>
       <c r="D13" s="12">
-        <v>3.45</v>
+        <v>7.5</v>
       </c>
       <c r="E13" s="12"/>
       <c r="F13" s="12"/>
@@ -4251,11 +4254,11 @@
     </row>
     <row r="14" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B14" s="5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C14" s="12"/>
       <c r="D14" s="12">
-        <v>7</v>
+        <v>3.45</v>
       </c>
       <c r="E14" s="12"/>
       <c r="F14" s="12"/>
@@ -4270,12 +4273,11 @@
     </row>
     <row r="15" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B15" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C15" s="12"/>
       <c r="D15" s="12">
-        <f>Wings!D31</f>
-        <v>0.4</v>
+        <v>7</v>
       </c>
       <c r="E15" s="12"/>
       <c r="F15" s="12"/>
@@ -4290,12 +4292,12 @@
     </row>
     <row r="16" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B16" s="5" t="s">
-        <v>138</v>
+        <v>49</v>
       </c>
       <c r="C16" s="12"/>
       <c r="D16" s="12">
-        <f>D15/D17</f>
-        <v>5.7142857142857144</v>
+        <f>Wings!D31</f>
+        <v>0.4</v>
       </c>
       <c r="E16" s="12"/>
       <c r="F16" s="12"/>
@@ -4310,12 +4312,12 @@
     </row>
     <row r="17" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B17" s="5" t="s">
-        <v>50</v>
+        <v>138</v>
       </c>
       <c r="C17" s="12"/>
       <c r="D17" s="12">
-        <f>Wings!E30</f>
-        <v>7.0000000000000007E-2</v>
+        <f>D16/D18</f>
+        <v>5.7142857142857144</v>
       </c>
       <c r="E17" s="12"/>
       <c r="F17" s="12"/>
@@ -4330,12 +4332,12 @@
     </row>
     <row r="18" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B18" s="5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C18" s="12"/>
       <c r="D18" s="12">
-        <f>E106</f>
-        <v>100.61584000000002</v>
+        <f>Wings!E30</f>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="E18" s="12"/>
       <c r="F18" s="12"/>
@@ -4350,11 +4352,12 @@
     </row>
     <row r="19" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B19" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C19" s="12"/>
       <c r="D19" s="12">
-        <v>1</v>
+        <f>E107</f>
+        <v>100.61584000000002</v>
       </c>
       <c r="E19" s="12"/>
       <c r="F19" s="12"/>
@@ -4369,11 +4372,11 @@
     </row>
     <row r="20" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B20" s="5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C20" s="12"/>
       <c r="D20" s="12">
-        <v>3.43</v>
+        <v>1</v>
       </c>
       <c r="E20" s="12"/>
       <c r="F20" s="12"/>
@@ -4388,11 +4391,11 @@
     </row>
     <row r="21" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B21" s="5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C21" s="12"/>
       <c r="D21" s="12">
-        <v>1</v>
+        <v>3.43</v>
       </c>
       <c r="E21" s="12"/>
       <c r="F21" s="12"/>
@@ -4407,11 +4410,11 @@
     </row>
     <row r="22" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B22" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C22" s="12"/>
       <c r="D22" s="12">
-        <v>0.76800000000000002</v>
+        <v>1</v>
       </c>
       <c r="E22" s="12"/>
       <c r="F22" s="12"/>
@@ -4426,11 +4429,11 @@
     </row>
     <row r="23" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B23" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C23" s="12"/>
       <c r="D23" s="12">
-        <v>0.77400000000000002</v>
+        <v>0.76800000000000002</v>
       </c>
       <c r="E23" s="12"/>
       <c r="F23" s="12"/>
@@ -4445,13 +4448,13 @@
     </row>
     <row r="24" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B24" s="5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C24" s="12"/>
       <c r="D24" s="12">
-        <v>0.12</v>
-      </c>
-      <c r="E24" s="10"/>
+        <v>0.77400000000000002</v>
+      </c>
+      <c r="E24" s="12"/>
       <c r="F24" s="10"/>
       <c r="G24" s="10"/>
       <c r="H24" s="10"/>
@@ -4464,11 +4467,11 @@
     </row>
     <row r="25" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B25" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C25" s="12"/>
-      <c r="D25" s="10">
-        <v>1.1200000000000001</v>
+      <c r="D25" s="12">
+        <v>0.12</v>
       </c>
       <c r="E25" s="10"/>
       <c r="F25" s="10"/>
@@ -4483,11 +4486,11 @@
     </row>
     <row r="26" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B26" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C26" s="12"/>
       <c r="D26" s="10">
-        <v>1</v>
+        <v>1.1200000000000001</v>
       </c>
       <c r="E26" s="10"/>
       <c r="F26" s="10"/>
@@ -4502,7 +4505,7 @@
     </row>
     <row r="27" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B27" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C27" s="12"/>
       <c r="D27" s="10">
@@ -4521,7 +4524,7 @@
     </row>
     <row r="28" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B28" s="5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C28" s="12"/>
       <c r="D28" s="10">
@@ -4540,7 +4543,7 @@
     </row>
     <row r="29" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B29" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C29" s="12"/>
       <c r="D29" s="10">
@@ -4559,7 +4562,7 @@
     </row>
     <row r="30" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B30" s="5" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C30" s="12"/>
       <c r="D30" s="10">
@@ -4578,7 +4581,7 @@
     </row>
     <row r="31" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B31" s="5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C31" s="12"/>
       <c r="D31" s="10">
@@ -4596,8 +4599,8 @@
       <c r="N31" s="10"/>
     </row>
     <row r="32" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="17" t="s">
-        <v>65</v>
+      <c r="B32" s="5" t="s">
+        <v>64</v>
       </c>
       <c r="C32" s="12"/>
       <c r="D32" s="10">
@@ -4614,9 +4617,9 @@
       <c r="M32" s="10"/>
       <c r="N32" s="10"/>
     </row>
-    <row r="33" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B33" s="2" t="s">
-        <v>66</v>
+    <row r="33" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B33" s="17" t="s">
+        <v>65</v>
       </c>
       <c r="C33" s="12"/>
       <c r="D33" s="10">
@@ -4634,12 +4637,12 @@
       <c r="N33" s="10"/>
     </row>
     <row r="34" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B34" s="4" t="s">
-        <v>67</v>
+      <c r="B34" s="2" t="s">
+        <v>66</v>
       </c>
       <c r="C34" s="12"/>
       <c r="D34" s="10">
-        <v>0.82599999999999996</v>
+        <v>1</v>
       </c>
       <c r="E34" s="10"/>
       <c r="F34" s="10"/>
@@ -4654,11 +4657,11 @@
     </row>
     <row r="35" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B35" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C35" s="12"/>
       <c r="D35" s="10">
-        <v>1</v>
+        <v>0.82599999999999996</v>
       </c>
       <c r="E35" s="10"/>
       <c r="F35" s="10"/>
@@ -4673,11 +4676,11 @@
     </row>
     <row r="36" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B36" s="4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C36" s="12"/>
       <c r="D36" s="10">
-        <v>1.143</v>
+        <v>1</v>
       </c>
       <c r="E36" s="10"/>
       <c r="F36" s="10"/>
@@ -4692,11 +4695,11 @@
     </row>
     <row r="37" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B37" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C37" s="12"/>
       <c r="D37" s="10">
-        <v>1</v>
+        <v>1.143</v>
       </c>
       <c r="E37" s="10"/>
       <c r="F37" s="10"/>
@@ -4711,7 +4714,7 @@
     </row>
     <row r="38" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B38" s="4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C38" s="12"/>
       <c r="D38" s="10">
@@ -4730,7 +4733,7 @@
     </row>
     <row r="39" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B39" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C39" s="12"/>
       <c r="D39" s="10">
@@ -4749,12 +4752,11 @@
     </row>
     <row r="40" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B40" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C40" s="12"/>
       <c r="D40" s="10">
-        <f>0.75*((1+2*Wings!C18)/(1+Wings!C18))*(Wings!C14/D47)*(TAN(Wings!C15*PI()/180))</f>
-        <v>0.72199786410048283</v>
+        <v>1</v>
       </c>
       <c r="E40" s="10"/>
       <c r="F40" s="10"/>
@@ -4769,12 +4771,12 @@
     </row>
     <row r="41" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B41" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C41" s="12"/>
       <c r="D41" s="10">
-        <f>0.3*D52</f>
-        <v>0.71174999999999999</v>
+        <f>0.75*((1+2*Wings!C18)/(1+Wings!C18))*(Wings!C14/D48)*(TAN(Wings!C15*PI()/180))</f>
+        <v>0.72199786410048283</v>
       </c>
       <c r="E41" s="10"/>
       <c r="F41" s="10"/>
@@ -4789,12 +4791,12 @@
     </row>
     <row r="42" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B42" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C42" s="12"/>
       <c r="D42" s="10">
-        <f>D52</f>
-        <v>2.3725000000000001</v>
+        <f>0.3*D53</f>
+        <v>0.71174999999999999</v>
       </c>
       <c r="E42" s="10"/>
       <c r="F42" s="10"/>
@@ -4809,12 +4811,12 @@
     </row>
     <row r="43" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B43" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C43" s="12"/>
       <c r="D43" s="10">
-        <f>Fuselage!D14</f>
-        <v>31</v>
+        <f>D53</f>
+        <v>2.3725000000000001</v>
       </c>
       <c r="E43" s="10"/>
       <c r="F43" s="10"/>
@@ -4829,12 +4831,12 @@
     </row>
     <row r="44" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B44" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C44" s="12"/>
       <c r="D44" s="10">
-        <f>15*5280</f>
-        <v>79200</v>
+        <f>Fuselage!D14</f>
+        <v>31</v>
       </c>
       <c r="E44" s="10"/>
       <c r="F44" s="10"/>
@@ -4849,11 +4851,12 @@
     </row>
     <row r="45" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B45" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C45" s="12"/>
       <c r="D45" s="10">
-        <v>15.92</v>
+        <f>15*5280</f>
+        <v>79200</v>
       </c>
       <c r="E45" s="10"/>
       <c r="F45" s="10"/>
@@ -4868,11 +4871,11 @@
     </row>
     <row r="46" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B46" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C46" s="12"/>
       <c r="D46" s="10">
-        <v>0</v>
+        <v>15.92</v>
       </c>
       <c r="E46" s="10"/>
       <c r="F46" s="10"/>
@@ -4887,12 +4890,11 @@
     </row>
     <row r="47" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B47" s="4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C47" s="12"/>
       <c r="D47" s="10">
-        <f>Fuselage!D14</f>
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="E47" s="10"/>
       <c r="F47" s="10"/>
@@ -4907,12 +4909,12 @@
     </row>
     <row r="48" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B48" s="4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C48" s="12"/>
       <c r="D48" s="10">
-        <f>5.3*12</f>
-        <v>63.599999999999994</v>
+        <f>Fuselage!D14</f>
+        <v>31</v>
       </c>
       <c r="E48" s="10"/>
       <c r="F48" s="10"/>
@@ -4927,7 +4929,7 @@
     </row>
     <row r="49" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B49" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C49" s="12"/>
       <c r="D49" s="10">
@@ -4947,12 +4949,12 @@
     </row>
     <row r="50" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B50" s="4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C50" s="12"/>
       <c r="D50" s="10">
-        <f>D45</f>
-        <v>15.92</v>
+        <f>5.3*12</f>
+        <v>63.599999999999994</v>
       </c>
       <c r="E50" s="10"/>
       <c r="F50" s="10"/>
@@ -4967,11 +4969,12 @@
     </row>
     <row r="51" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B51" s="4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C51" s="12"/>
       <c r="D51" s="10">
-        <v>1</v>
+        <f>D46</f>
+        <v>15.92</v>
       </c>
       <c r="E51" s="10"/>
       <c r="F51" s="10"/>
@@ -4986,12 +4989,11 @@
     </row>
     <row r="52" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B52" s="4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C52" s="12"/>
       <c r="D52" s="10">
-        <f>Wings!C34-Wings!D34</f>
-        <v>2.3725000000000001</v>
+        <v>1</v>
       </c>
       <c r="E52" s="10"/>
       <c r="F52" s="10"/>
@@ -5006,12 +5008,12 @@
     </row>
     <row r="53" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B53" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C53" s="12"/>
       <c r="D53" s="10">
-        <f>36-17.79</f>
-        <v>18.21</v>
+        <f>Wings!C34-Wings!D34</f>
+        <v>2.3725000000000001</v>
       </c>
       <c r="E53" s="10"/>
       <c r="F53" s="10"/>
@@ -5026,11 +5028,12 @@
     </row>
     <row r="54" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B54" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C54" s="12"/>
       <c r="D54" s="10">
-        <v>1.6</v>
+        <f>36-17.79</f>
+        <v>18.21</v>
       </c>
       <c r="E54" s="10"/>
       <c r="F54" s="10"/>
@@ -5045,11 +5048,11 @@
     </row>
     <row r="55" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B55" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C55" s="12"/>
       <c r="D55" s="10">
-        <v>1</v>
+        <v>1.6</v>
       </c>
       <c r="E55" s="10"/>
       <c r="F55" s="10"/>
@@ -5064,7 +5067,7 @@
     </row>
     <row r="56" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B56" s="4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C56" s="12"/>
       <c r="D56" s="10">
@@ -5083,7 +5086,7 @@
     </row>
     <row r="57" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B57" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C57" s="12"/>
       <c r="D57" s="10">
@@ -5102,11 +5105,11 @@
     </row>
     <row r="58" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B58" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C58" s="12"/>
       <c r="D58" s="10">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E58" s="10"/>
       <c r="F58" s="10"/>
@@ -5121,11 +5124,11 @@
     </row>
     <row r="59" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B59" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C59" s="12"/>
       <c r="D59" s="10">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E59" s="10"/>
       <c r="F59" s="10"/>
@@ -5140,11 +5143,11 @@
     </row>
     <row r="60" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B60" s="4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C60" s="12"/>
       <c r="D60" s="10">
-        <v>15.69</v>
+        <v>1</v>
       </c>
       <c r="E60" s="10"/>
       <c r="F60" s="10"/>
@@ -5159,12 +5162,11 @@
     </row>
     <row r="61" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B61" s="4" t="s">
-        <v>144</v>
+        <v>93</v>
       </c>
       <c r="C61" s="12"/>
       <c r="D61" s="10">
-        <f>3*1.5</f>
-        <v>4.5</v>
+        <v>15.69</v>
       </c>
       <c r="E61" s="10"/>
       <c r="F61" s="10"/>
@@ -5179,11 +5181,12 @@
     </row>
     <row r="62" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B62" s="4" t="s">
-        <v>94</v>
+        <v>144</v>
       </c>
       <c r="C62" s="12"/>
       <c r="D62" s="10">
-        <v>3</v>
+        <f>3*1.5</f>
+        <v>4.5</v>
       </c>
       <c r="E62" s="10"/>
       <c r="F62" s="10"/>
@@ -5198,11 +5201,11 @@
     </row>
     <row r="63" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B63" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C63" s="12"/>
       <c r="D63" s="10">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E63" s="10"/>
       <c r="F63" s="10"/>
@@ -5217,11 +5220,11 @@
     </row>
     <row r="64" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B64" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C64" s="12"/>
       <c r="D64" s="10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E64" s="10"/>
       <c r="F64" s="10"/>
@@ -5236,7 +5239,7 @@
     </row>
     <row r="65" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B65" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C65" s="12"/>
       <c r="D65" s="10">
@@ -5255,7 +5258,7 @@
     </row>
     <row r="66" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B66" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C66" s="12"/>
       <c r="D66" s="10">
@@ -5274,11 +5277,11 @@
     </row>
     <row r="67" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B67" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C67" s="12"/>
       <c r="D67" s="10">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E67" s="10"/>
       <c r="F67" s="10"/>
@@ -5293,11 +5296,11 @@
     </row>
     <row r="68" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B68" s="4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C68" s="12"/>
       <c r="D68" s="10">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E68" s="10"/>
       <c r="F68" s="10"/>
@@ -5312,11 +5315,11 @@
     </row>
     <row r="69" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B69" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C69" s="12"/>
       <c r="D69" s="10">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E69" s="10"/>
       <c r="F69" s="10"/>
@@ -5331,11 +5334,11 @@
     </row>
     <row r="70" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B70" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C70" s="12"/>
       <c r="D70" s="10">
-        <v>3.69</v>
+        <v>5</v>
       </c>
       <c r="E70" s="10"/>
       <c r="F70" s="10"/>
@@ -5350,12 +5353,11 @@
     </row>
     <row r="71" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B71" s="4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C71" s="12"/>
       <c r="D71" s="10">
-        <f>1.5*9.5</f>
-        <v>14.25</v>
+        <v>3.69</v>
       </c>
       <c r="E71" s="10"/>
       <c r="F71" s="10"/>
@@ -5370,12 +5372,12 @@
     </row>
     <row r="72" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B72" s="4" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C72" s="12"/>
       <c r="D72" s="10">
-        <f>208</f>
-        <v>208</v>
+        <f>1.5*9.5</f>
+        <v>14.25</v>
       </c>
       <c r="E72" s="10"/>
       <c r="F72" s="10"/>
@@ -5390,11 +5392,12 @@
     </row>
     <row r="73" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B73" s="4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C73" s="12"/>
       <c r="D73" s="10">
-        <v>110</v>
+        <f>208</f>
+        <v>208</v>
       </c>
       <c r="E73" s="10"/>
       <c r="F73" s="10"/>
@@ -5409,12 +5412,11 @@
     </row>
     <row r="74" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B74" s="4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C74" s="12"/>
       <c r="D74" s="10">
-        <f>108+24+21.31+24+60</f>
-        <v>237.31</v>
+        <v>110</v>
       </c>
       <c r="E74" s="10"/>
       <c r="F74" s="10"/>
@@ -5429,12 +5431,12 @@
     </row>
     <row r="75" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B75" s="4" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C75" s="12"/>
       <c r="D75" s="10">
-        <f>108</f>
-        <v>108</v>
+        <f>108+24+21.31+24+60</f>
+        <v>237.31</v>
       </c>
       <c r="E75" s="10"/>
       <c r="F75" s="10"/>
@@ -5449,10 +5451,11 @@
     </row>
     <row r="76" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B76" s="4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C76" s="12"/>
       <c r="D76" s="10">
+        <f>108</f>
         <v>108</v>
       </c>
       <c r="E76" s="10"/>
@@ -5468,11 +5471,11 @@
     </row>
     <row r="77" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B77" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C77" s="12"/>
       <c r="D77" s="10">
-        <v>730.42200000000003</v>
+        <v>108</v>
       </c>
       <c r="E77" s="10"/>
       <c r="F77" s="10"/>
@@ -5487,11 +5490,11 @@
     </row>
     <row r="78" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B78" s="4" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C78" s="12"/>
       <c r="D78" s="10">
-        <v>0</v>
+        <v>730.42200000000003</v>
       </c>
       <c r="E78" s="10"/>
       <c r="F78" s="10"/>
@@ -5506,12 +5509,11 @@
     </row>
     <row r="79" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B79" s="4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C79" s="12"/>
       <c r="D79" s="10">
-        <f>D76</f>
-        <v>108</v>
+        <v>0</v>
       </c>
       <c r="E79" s="10"/>
       <c r="F79" s="10"/>
@@ -5526,11 +5528,12 @@
     </row>
     <row r="80" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B80" s="4" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C80" s="12"/>
       <c r="D80" s="10">
-        <v>41.515000000000001</v>
+        <f>D77</f>
+        <v>108</v>
       </c>
       <c r="E80" s="10"/>
       <c r="F80" s="10"/>
@@ -5545,11 +5548,11 @@
     </row>
     <row r="81" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B81" s="4" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C81" s="12"/>
       <c r="D81" s="10">
-        <v>60</v>
+        <v>41.515000000000001</v>
       </c>
       <c r="E81" s="10"/>
       <c r="F81" s="10"/>
@@ -5564,11 +5567,11 @@
     </row>
     <row r="82" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B82" s="4" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C82" s="12"/>
       <c r="D82" s="10">
-        <v>200</v>
+        <v>60</v>
       </c>
       <c r="E82" s="10"/>
       <c r="F82" s="10"/>
@@ -5583,11 +5586,11 @@
     </row>
     <row r="83" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B83" s="4" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C83" s="12"/>
       <c r="D83" s="10">
-        <v>60</v>
+        <v>200</v>
       </c>
       <c r="E83" s="10"/>
       <c r="F83" s="10"/>
@@ -5602,11 +5605,11 @@
     </row>
     <row r="84" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B84" s="4" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C84" s="12"/>
       <c r="D84" s="10">
-        <v>300</v>
+        <v>60</v>
       </c>
       <c r="E84" s="10"/>
       <c r="F84" s="10"/>
@@ -5621,12 +5624,11 @@
     </row>
     <row r="85" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B85" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C85" s="12"/>
       <c r="D85" s="10">
-        <f>1.708</f>
-        <v>1.708</v>
+        <v>300</v>
       </c>
       <c r="E85" s="10"/>
       <c r="F85" s="10"/>
@@ -5641,11 +5643,12 @@
     </row>
     <row r="86" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B86" s="4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C86" s="12"/>
       <c r="D86" s="10">
-        <v>23770</v>
+        <f>1.708</f>
+        <v>1.708</v>
       </c>
       <c r="E86" s="10"/>
       <c r="F86" s="10"/>
@@ -5660,11 +5663,10 @@
     </row>
     <row r="87" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B87" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C87" s="12"/>
       <c r="D87" s="10">
-        <f>D86*D57</f>
         <v>23770</v>
       </c>
       <c r="E87" s="10"/>
@@ -5680,11 +5682,12 @@
     </row>
     <row r="88" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B88" s="4" t="s">
-        <v>12</v>
+        <v>119</v>
       </c>
       <c r="C88" s="12"/>
       <c r="D88" s="10">
-        <v>0.04</v>
+        <f>D87*D58</f>
+        <v>23770</v>
       </c>
       <c r="E88" s="10"/>
       <c r="F88" s="10"/>
@@ -5699,12 +5702,11 @@
     </row>
     <row r="89" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B89" s="4" t="s">
-        <v>120</v>
+        <v>12</v>
       </c>
       <c r="C89" s="12"/>
       <c r="D89" s="10">
-        <f>(6950-2300*2)*(1/6.8)</f>
-        <v>345.58823529411768</v>
+        <v>0.04</v>
       </c>
       <c r="E89" s="10"/>
       <c r="F89" s="10"/>
@@ -5719,11 +5721,12 @@
     </row>
     <row r="90" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B90" s="4" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C90" s="12"/>
       <c r="D90" s="10">
-        <v>0</v>
+        <f>(6950-2300*2)*(1/6.8)</f>
+        <v>345.58823529411768</v>
       </c>
       <c r="E90" s="10"/>
       <c r="F90" s="10"/>
@@ -5738,11 +5741,11 @@
     </row>
     <row r="91" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B91" s="4" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C91" s="12"/>
       <c r="D91" s="10">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="E91" s="10"/>
       <c r="F91" s="10"/>
@@ -5757,12 +5760,11 @@
     </row>
     <row r="92" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B92" s="4" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C92" s="12"/>
       <c r="D92" s="10">
-        <f>6950*(1/6.8)</f>
-        <v>1022.0588235294118</v>
+        <v>300</v>
       </c>
       <c r="E92" s="10"/>
       <c r="F92" s="10"/>
@@ -5777,12 +5779,12 @@
     </row>
     <row r="93" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B93" s="4" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C93" s="12"/>
       <c r="D93" s="10">
-        <f>Fuselage!D15</f>
-        <v>7.5</v>
+        <f>6950*(1/6.8)</f>
+        <v>1022.0588235294118</v>
       </c>
       <c r="E93" s="10"/>
       <c r="F93" s="10"/>
@@ -5797,11 +5799,12 @@
     </row>
     <row r="94" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B94" s="4" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C94" s="12"/>
       <c r="D94" s="10">
-        <v>5100</v>
+        <f>Fuselage!D15</f>
+        <v>7.5</v>
       </c>
       <c r="E94" s="10"/>
       <c r="F94" s="10"/>
@@ -5816,12 +5819,11 @@
     </row>
     <row r="95" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B95" s="4" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C95" s="12"/>
       <c r="D95" s="10">
-        <f>0.6*D89*6.8</f>
-        <v>1410</v>
+        <v>5100</v>
       </c>
       <c r="E95" s="10"/>
       <c r="F95" s="10"/>
@@ -5836,12 +5838,12 @@
     </row>
     <row r="96" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B96" s="4" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C96" s="12"/>
       <c r="D96" s="10">
-        <f>2.331*(4730.23)^(0.901) *D30*D35</f>
-        <v>4771.0194615715218</v>
+        <f>0.6*D90*6.8</f>
+        <v>1410</v>
       </c>
       <c r="E96" s="10"/>
       <c r="F96" s="10"/>
@@ -5856,11 +5858,12 @@
     </row>
     <row r="97" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B97" s="4" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C97" s="12"/>
       <c r="D97" s="10">
-        <v>4730.2299999999996</v>
+        <f>2.331*(4730.23)^(0.901) *D31*D36</f>
+        <v>4771.0194615715218</v>
       </c>
       <c r="E97" s="10"/>
       <c r="F97" s="10"/>
@@ -5875,12 +5878,11 @@
     </row>
     <row r="98" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B98" s="4" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C98" s="12"/>
       <c r="D98" s="10">
-        <f>1050</f>
-        <v>1050</v>
+        <v>4730.2299999999996</v>
       </c>
       <c r="E98" s="10"/>
       <c r="F98" s="10"/>
@@ -5895,12 +5897,12 @@
     </row>
     <row r="99" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B99" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C99" s="12"/>
       <c r="D99" s="10">
-        <f>0.6688*30000</f>
-        <v>20064</v>
+        <f>1050</f>
+        <v>1050</v>
       </c>
       <c r="E99" s="10"/>
       <c r="F99" s="10"/>
@@ -5915,12 +5917,12 @@
     </row>
     <row r="100" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B100" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C100" s="12"/>
       <c r="D100" s="10">
-        <f>11.9*(D91*8*12^2)^(0.271)</f>
-        <v>377.13812992987448</v>
+        <f>0.6688*30000</f>
+        <v>20064</v>
       </c>
       <c r="E100" s="10"/>
       <c r="F100" s="10"/>
@@ -5935,12 +5937,12 @@
     </row>
     <row r="101" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B101" s="4" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C101" s="12"/>
       <c r="D101" s="10">
-        <f>700</f>
-        <v>700</v>
+        <f>11.9*(D92*8*12^2)^(0.271)</f>
+        <v>377.13812992987448</v>
       </c>
       <c r="E101" s="10"/>
       <c r="F101" s="10"/>
@@ -5953,14 +5955,14 @@
       <c r="M101" s="10"/>
       <c r="N101" s="10"/>
     </row>
-    <row r="102" spans="2:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="102" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B102" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C102" s="12"/>
       <c r="D102" s="10">
-        <f>Wings!C15</f>
-        <v>40</v>
+        <f>700</f>
+        <v>700</v>
       </c>
       <c r="E102" s="10"/>
       <c r="F102" s="10"/>
@@ -5973,14 +5975,14 @@
       <c r="M102" s="10"/>
       <c r="N102" s="10"/>
     </row>
-    <row r="103" spans="2:14" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B103" s="5" t="s">
-        <v>141</v>
+    <row r="103" spans="2:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="B103" s="4" t="s">
+        <v>133</v>
       </c>
       <c r="C103" s="12"/>
       <c r="D103" s="10">
-        <f>Wings!C18</f>
-        <v>0.22774708410067526</v>
+        <f>Wings!C15</f>
+        <v>40</v>
       </c>
       <c r="E103" s="10"/>
       <c r="F103" s="10"/>
@@ -5995,12 +5997,12 @@
     </row>
     <row r="104" spans="2:14" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B104" s="5" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C104" s="12"/>
       <c r="D104" s="10">
-        <f>Wings!D18</f>
-        <v>0.22699386503067487</v>
+        <f>Wings!C18</f>
+        <v>0.22774708410067526</v>
       </c>
       <c r="E104" s="10"/>
       <c r="F104" s="10"/>
@@ -6015,12 +6017,12 @@
     </row>
     <row r="105" spans="2:14" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B105" s="5" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C105" s="12"/>
       <c r="D105" s="10">
-        <f>Wings!E18</f>
-        <v>0.5</v>
+        <f>Wings!D18</f>
+        <v>0.22699386503067487</v>
       </c>
       <c r="E105" s="10"/>
       <c r="F105" s="10"/>
@@ -6033,16 +6035,16 @@
       <c r="M105" s="10"/>
       <c r="N105" s="10"/>
     </row>
-    <row r="106" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="2:14" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B106" s="5" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="C106" s="12"/>
-      <c r="D106" s="10"/>
-      <c r="E106" s="10">
-        <f>((D11+D47)/2)^2 * ((D54*0.52^2)/4)</f>
-        <v>100.61584000000002</v>
-      </c>
+      <c r="D106" s="10">
+        <f>Wings!E18</f>
+        <v>0.5</v>
+      </c>
+      <c r="E106" s="10"/>
       <c r="F106" s="10"/>
       <c r="G106" s="10"/>
       <c r="H106" s="10"/>
@@ -6053,8 +6055,28 @@
       <c r="M106" s="10"/>
       <c r="N106" s="10"/>
     </row>
+    <row r="107" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B107" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="C107" s="12"/>
+      <c r="D107" s="10"/>
+      <c r="E107" s="10">
+        <f>((D12+D48)/2)^2 * ((D55*0.52^2)/4)</f>
+        <v>100.61584000000002</v>
+      </c>
+      <c r="F107" s="10"/>
+      <c r="G107" s="10"/>
+      <c r="H107" s="10"/>
+      <c r="I107" s="10"/>
+      <c r="J107" s="10"/>
+      <c r="K107" s="10"/>
+      <c r="L107" s="10"/>
+      <c r="M107" s="10"/>
+      <c r="N107" s="10"/>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="C4:N106">
+  <conditionalFormatting sqref="C4:N107">
     <cfRule type="expression" dxfId="8" priority="2">
       <formula>_xlfn.ISFORMULA(C4)</formula>
     </cfRule>

</xml_diff>

<commit_message>
Added helper function for normalizing engine type input.
</commit_message>
<xml_diff>
--- a/examples/F-16A B Block 10 and 15/Operator/F-16A Block 50.xlsx
+++ b/examples/F-16A B Block 10 and 15/Operator/F-16A Block 50.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\John Freeman\Desktop\Academics\VRMastersProgram\code\air-vehicle-design\examples\F-16A B Block 10 and 15\Operator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E3135B5-E29A-4D17-A26A-50B918589A51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{236CF331-A4A6-40EE-8DAF-94C92C43FE5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="384" windowWidth="23256" windowHeight="12720" firstSheet="1" activeTab="2" xr2:uid="{5F5D00AF-8D4A-4BC4-9FDA-F17071C88D94}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="197">
   <si>
     <t>THIS IS FOR THE END USER</t>
   </si>
@@ -632,6 +632,9 @@
   </si>
   <si>
     <t>Tail config</t>
+  </si>
+  <si>
+    <t>turbofan</t>
   </si>
 </sst>
 </file>
@@ -1991,7 +1994,9 @@
         <v>193</v>
       </c>
       <c r="E6" s="9"/>
-      <c r="F6" s="9"/>
+      <c r="F6" s="9" t="s">
+        <v>196</v>
+      </c>
       <c r="G6" s="9"/>
       <c r="H6" s="11"/>
       <c r="I6" s="11"/>

</xml_diff>

<commit_message>
Added variable for "engine type".
</commit_message>
<xml_diff>
--- a/examples/F-16A B Block 10 and 15/Operator/F-16A Block 50.xlsx
+++ b/examples/F-16A B Block 10 and 15/Operator/F-16A Block 50.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\John Freeman\Desktop\Academics\VRMastersProgram\code\air-vehicle-design\examples\F-16A B Block 10 and 15\Operator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{236CF331-A4A6-40EE-8DAF-94C92C43FE5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC62EE07-BB43-4726-9635-AF8D798844FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="384" windowWidth="23256" windowHeight="12720" firstSheet="1" activeTab="2" xr2:uid="{5F5D00AF-8D4A-4BC4-9FDA-F17071C88D94}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="197">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="198">
   <si>
     <t>THIS IS FOR THE END USER</t>
   </si>
@@ -634,7 +634,10 @@
     <t>Tail config</t>
   </si>
   <si>
-    <t>turbofan</t>
+    <t>engine type</t>
+  </si>
+  <si>
+    <t>"low bpr turbofan"</t>
   </si>
 </sst>
 </file>
@@ -1994,9 +1997,7 @@
         <v>193</v>
       </c>
       <c r="E6" s="9"/>
-      <c r="F6" s="9" t="s">
-        <v>196</v>
-      </c>
+      <c r="F6" s="9"/>
       <c r="G6" s="9"/>
       <c r="H6" s="11"/>
       <c r="I6" s="11"/>
@@ -2102,9 +2103,13 @@
       <c r="N11" s="10"/>
       <c r="O11" s="10"/>
     </row>
-    <row r="12" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C12" s="5"/>
-      <c r="D12" s="12"/>
+    <row r="12" spans="3:15" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C12" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>197</v>
+      </c>
       <c r="E12" s="12"/>
       <c r="F12" s="12"/>
       <c r="G12" s="12"/>

</xml_diff>

<commit_message>
Added "requirements" class and "isafterburning" to design input arguments.
</commit_message>
<xml_diff>
--- a/examples/F-16A B Block 10 and 15/Operator/F-16A Block 50.xlsx
+++ b/examples/F-16A B Block 10 and 15/Operator/F-16A Block 50.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\John Freeman\Desktop\Academics\VRMastersProgram\code\air-vehicle-design\examples\F-16A B Block 10 and 15\Operator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC62EE07-BB43-4726-9635-AF8D798844FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{547F5B16-0483-4619-8C5C-11CFAE0C35D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="384" windowWidth="23256" windowHeight="12720" firstSheet="1" activeTab="2" xr2:uid="{5F5D00AF-8D4A-4BC4-9FDA-F17071C88D94}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="198">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="199">
   <si>
     <t>THIS IS FOR THE END USER</t>
   </si>
@@ -638,6 +638,9 @@
   </si>
   <si>
     <t>"low bpr turbofan"</t>
+  </si>
+  <si>
+    <t>isafterburning</t>
   </si>
 </sst>
 </file>
@@ -2122,9 +2125,13 @@
       <c r="N12" s="10"/>
       <c r="O12" s="10"/>
     </row>
-    <row r="13" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C13" s="5"/>
-      <c r="D13" s="12"/>
+    <row r="13" spans="3:15" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C13" s="5" t="s">
+        <v>198</v>
+      </c>
+      <c r="D13" s="12" t="s">
+        <v>156</v>
+      </c>
       <c r="E13" s="12"/>
       <c r="F13" s="12"/>
       <c r="G13" s="12"/>

</xml_diff>

<commit_message>
Added propulsion coefficients E, F1, F2. Constants. Unknown definitions.
</commit_message>
<xml_diff>
--- a/examples/F-16A B Block 10 and 15/Operator/F-16A Block 50.xlsx
+++ b/examples/F-16A B Block 10 and 15/Operator/F-16A Block 50.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\John Freeman\Desktop\Academics\VRMastersProgram\code\air-vehicle-design\examples\F-16A B Block 10 and 15\Operator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{547F5B16-0483-4619-8C5C-11CFAE0C35D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39D3A9D8-0F17-4DB5-85D7-2636FCC830AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="384" windowWidth="23256" windowHeight="12720" firstSheet="1" activeTab="2" xr2:uid="{5F5D00AF-8D4A-4BC4-9FDA-F17071C88D94}"/>
+    <workbookView xWindow="22932" yWindow="384" windowWidth="23256" windowHeight="12720" firstSheet="1" activeTab="5" xr2:uid="{5F5D00AF-8D4A-4BC4-9FDA-F17071C88D94}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="202">
   <si>
     <t>THIS IS FOR THE END USER</t>
   </si>
@@ -641,6 +641,15 @@
   </si>
   <si>
     <t>isafterburning</t>
+  </si>
+  <si>
+    <t>E</t>
+  </si>
+  <si>
+    <t>F1</t>
+  </si>
+  <si>
+    <t>F2</t>
   </si>
 </sst>
 </file>
@@ -1204,10 +1213,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
+        <a:sysClr val="windowText" lastClr="0A0A0A"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
+        <a:sysClr val="window" lastClr="FAFAFA"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="0E2841"/>
@@ -3690,13 +3699,15 @@
       <c r="M14" s="10"/>
       <c r="N14" s="10"/>
     </row>
-    <row r="15" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B15" s="4"/>
+    <row r="15" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="5" t="s">
+        <v>43</v>
+      </c>
       <c r="C15" s="12"/>
       <c r="D15" s="12"/>
       <c r="E15" s="12"/>
       <c r="F15" s="12"/>
-      <c r="G15" s="12"/>
+      <c r="G15" s="10"/>
       <c r="H15" s="12"/>
       <c r="I15" s="12"/>
       <c r="J15" s="10"/>
@@ -3705,13 +3716,15 @@
       <c r="M15" s="10"/>
       <c r="N15" s="10"/>
     </row>
-    <row r="16" spans="2:14" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="4"/>
+    <row r="16" spans="2:14" ht="24.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="5" t="s">
+        <v>10</v>
+      </c>
       <c r="C16" s="12"/>
       <c r="D16" s="12"/>
       <c r="E16" s="12"/>
       <c r="F16" s="12"/>
-      <c r="G16" s="12"/>
+      <c r="G16" s="10"/>
       <c r="H16" s="12"/>
       <c r="I16" s="12"/>
       <c r="J16" s="10"/>
@@ -3722,13 +3735,15 @@
     </row>
     <row r="17" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B17" s="5" t="s">
-        <v>43</v>
+        <v>146</v>
       </c>
       <c r="C17" s="12"/>
       <c r="D17" s="12"/>
       <c r="E17" s="12"/>
       <c r="F17" s="12"/>
-      <c r="G17" s="10"/>
+      <c r="G17" s="10">
+        <v>0.63</v>
+      </c>
       <c r="H17" s="10"/>
       <c r="I17" s="10"/>
       <c r="J17" s="10"/>
@@ -3739,11 +3754,15 @@
     </row>
     <row r="18" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B18" s="5" t="s">
-        <v>10</v>
+        <v>199</v>
       </c>
       <c r="C18" s="12"/>
-      <c r="D18" s="12"/>
-      <c r="E18" s="12"/>
+      <c r="D18" s="12">
+        <v>1</v>
+      </c>
+      <c r="E18" s="12">
+        <v>0.5</v>
+      </c>
       <c r="F18" s="12"/>
       <c r="G18" s="10"/>
       <c r="H18" s="10"/>
@@ -3756,15 +3775,17 @@
     </row>
     <row r="19" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B19" s="5" t="s">
-        <v>146</v>
+        <v>200</v>
       </c>
       <c r="C19" s="12"/>
-      <c r="D19" s="12"/>
-      <c r="E19" s="12"/>
+      <c r="D19" s="12">
+        <v>0.3</v>
+      </c>
+      <c r="E19" s="12">
+        <v>0.1</v>
+      </c>
       <c r="F19" s="12"/>
-      <c r="G19" s="10">
-        <v>0.63</v>
-      </c>
+      <c r="G19" s="10"/>
       <c r="H19" s="10"/>
       <c r="I19" s="10"/>
       <c r="J19" s="10"/>
@@ -3774,10 +3795,16 @@
       <c r="N19" s="10"/>
     </row>
     <row r="20" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="5"/>
+      <c r="B20" s="5" t="s">
+        <v>201</v>
+      </c>
       <c r="C20" s="12"/>
-      <c r="D20" s="12"/>
-      <c r="E20" s="12"/>
+      <c r="D20" s="12">
+        <v>1.7</v>
+      </c>
+      <c r="E20" s="12">
+        <v>2.2000000000000002</v>
+      </c>
       <c r="F20" s="12"/>
       <c r="G20" s="10"/>
       <c r="H20" s="10"/>

</xml_diff>

<commit_message>
Linked computations of TSFC and thrust for low bypass ratio engines (Brandt's work used).
</commit_message>
<xml_diff>
--- a/examples/F-16A B Block 10 and 15/Operator/F-16A Block 50.xlsx
+++ b/examples/F-16A B Block 10 and 15/Operator/F-16A Block 50.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\John Freeman\Desktop\Academics\VRMastersProgram\code\air-vehicle-design\examples\F-16A B Block 10 and 15\Operator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C3F67A9-BA2C-4844-823D-44A97F5F475B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BAB8AEA-AC53-416B-BD10-C61162362B6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="384" windowWidth="23256" windowHeight="12720" firstSheet="1" activeTab="5" xr2:uid="{5F5D00AF-8D4A-4BC4-9FDA-F17071C88D94}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="201">
   <si>
     <t>THIS IS FOR THE END USER</t>
   </si>
@@ -644,6 +644,9 @@
   </si>
   <si>
     <t>F2</t>
+  </si>
+  <si>
+    <t>TSFC (sea level) (per hour)</t>
   </si>
 </sst>
 </file>
@@ -3685,7 +3688,9 @@
       <c r="C14" s="9">
         <v>15000</v>
       </c>
-      <c r="D14" s="9"/>
+      <c r="D14" s="9">
+        <v>23770</v>
+      </c>
       <c r="E14" s="11"/>
       <c r="F14" s="10"/>
       <c r="G14" s="10"/>
@@ -3699,13 +3704,13 @@
     </row>
     <row r="15" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B15" s="5" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="C15" s="12">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="D15" s="12">
-        <v>0.5</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="E15" s="12"/>
       <c r="F15" s="10"/>
@@ -3720,13 +3725,13 @@
     </row>
     <row r="16" spans="2:14" ht="24.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B16" s="5" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C16" s="12">
-        <v>0.3</v>
+        <v>1</v>
       </c>
       <c r="D16" s="12">
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
       <c r="E16" s="12"/>
       <c r="F16" s="10"/>
@@ -3741,13 +3746,13 @@
     </row>
     <row r="17" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B17" s="5" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C17" s="12">
-        <v>1.7</v>
+        <v>0.3</v>
       </c>
       <c r="D17" s="12">
-        <v>2.2000000000000002</v>
+        <v>0.1</v>
       </c>
       <c r="E17" s="12"/>
       <c r="F17" s="10"/>
@@ -3762,13 +3767,15 @@
     </row>
     <row r="18" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B18" s="5" t="s">
-        <v>144</v>
-      </c>
-      <c r="C18" s="12"/>
-      <c r="D18" s="12"/>
-      <c r="E18" s="10">
-        <v>0.63</v>
-      </c>
+        <v>199</v>
+      </c>
+      <c r="C18" s="12">
+        <v>1.7</v>
+      </c>
+      <c r="D18" s="12">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="E18" s="12"/>
       <c r="F18" s="10"/>
       <c r="G18" s="10"/>
       <c r="H18" s="10"/>
@@ -3780,10 +3787,14 @@
       <c r="N18" s="10"/>
     </row>
     <row r="19" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="5"/>
+      <c r="B19" s="5" t="s">
+        <v>144</v>
+      </c>
       <c r="C19" s="12"/>
       <c r="D19" s="12"/>
-      <c r="E19" s="12"/>
+      <c r="E19" s="10">
+        <v>0.63</v>
+      </c>
       <c r="F19" s="10"/>
       <c r="G19" s="10"/>
       <c r="H19" s="10"/>

</xml_diff>

<commit_message>
Updated mission segments to use propulsion results.
</commit_message>
<xml_diff>
--- a/examples/F-16A B Block 10 and 15/Operator/F-16A Block 50.xlsx
+++ b/examples/F-16A B Block 10 and 15/Operator/F-16A Block 50.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BAB8AEA-AC53-416B-BD10-C61162362B6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="384" windowWidth="23256" windowHeight="12720" firstSheet="1" activeTab="5" xr2:uid="{5F5D00AF-8D4A-4BC4-9FDA-F17071C88D94}"/>
+    <workbookView xWindow="22932" yWindow="384" windowWidth="23256" windowHeight="12720" firstSheet="1" activeTab="6" xr2:uid="{5F5D00AF-8D4A-4BC4-9FDA-F17071C88D94}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1216,10 +1216,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="0A0A0A"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FAFAFA"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="0E2841"/>

</xml_diff>

<commit_message>
Added subsystem level 3. Fuel volume check, internal volume check functions.
</commit_message>
<xml_diff>
--- a/examples/F-16A B Block 10 and 15/Operator/F-16A Block 50.xlsx
+++ b/examples/F-16A B Block 10 and 15/Operator/F-16A Block 50.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\John Freeman\Desktop\Academics\VRMastersProgram\code\air-vehicle-design\examples\F-16A B Block 10 and 15\Operator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BAB8AEA-AC53-416B-BD10-C61162362B6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45EFEEB1-A096-4C28-9CC8-08BA870FFEF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="384" windowWidth="23256" windowHeight="12720" firstSheet="1" activeTab="2" xr2:uid="{5F5D00AF-8D4A-4BC4-9FDA-F17071C88D94}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="203">
   <si>
     <t>THIS IS FOR THE END USER</t>
   </si>
@@ -647,6 +647,12 @@
   </si>
   <si>
     <t>TSFC (sea level) (per hour)</t>
+  </si>
+  <si>
+    <t>fuel_type</t>
+  </si>
+  <si>
+    <t>JP-4</t>
   </si>
 </sst>
 </file>
@@ -2157,8 +2163,12 @@
       <c r="O13" s="10"/>
     </row>
     <row r="14" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C14" s="5"/>
-      <c r="D14" s="12"/>
+      <c r="C14" s="5" t="s">
+        <v>201</v>
+      </c>
+      <c r="D14" s="12" t="s">
+        <v>202</v>
+      </c>
       <c r="E14" s="12"/>
       <c r="F14" s="12"/>
       <c r="G14" s="12"/>

</xml_diff>

<commit_message>
Added functions to compute MAC.
</commit_message>
<xml_diff>
--- a/examples/F-16A B Block 10 and 15/Operator/F-16A Block 50.xlsx
+++ b/examples/F-16A B Block 10 and 15/Operator/F-16A Block 50.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\John Freeman\Desktop\Academics\VRMastersProgram\code\air-vehicle-design\examples\F-16A B Block 10 and 15\Operator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45EFEEB1-A096-4C28-9CC8-08BA870FFEF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E139D14-E043-4B54-9E32-9642F65CB0D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="384" windowWidth="23256" windowHeight="12720" firstSheet="1" activeTab="2" xr2:uid="{5F5D00AF-8D4A-4BC4-9FDA-F17071C88D94}"/>
+    <workbookView xWindow="22932" yWindow="384" windowWidth="23256" windowHeight="12720" firstSheet="1" activeTab="7" xr2:uid="{5F5D00AF-8D4A-4BC4-9FDA-F17071C88D94}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,8 +20,9 @@
     <sheet name="Fuselage" sheetId="5" r:id="rId5"/>
     <sheet name="Propulsion" sheetId="7" r:id="rId6"/>
     <sheet name="Weights" sheetId="8" r:id="rId7"/>
-    <sheet name="Protuberances" sheetId="9" r:id="rId8"/>
-    <sheet name="Skin roughness" sheetId="10" r:id="rId9"/>
+    <sheet name="Stability&amp;Control" sheetId="12" r:id="rId8"/>
+    <sheet name="Protuberances" sheetId="9" r:id="rId9"/>
+    <sheet name="Skin roughness" sheetId="10" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -44,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="226">
   <si>
     <t>THIS IS FOR THE END USER</t>
   </si>
@@ -653,6 +654,75 @@
   </si>
   <si>
     <t>JP-4</t>
+  </si>
+  <si>
+    <t>Wing</t>
+  </si>
+  <si>
+    <t>HT</t>
+  </si>
+  <si>
+    <t>VT</t>
+  </si>
+  <si>
+    <t>Nacelles</t>
+  </si>
+  <si>
+    <t>Engine</t>
+  </si>
+  <si>
+    <t>Gear</t>
+  </si>
+  <si>
+    <t>Inlet duct</t>
+  </si>
+  <si>
+    <t>Controls</t>
+  </si>
+  <si>
+    <t>Electrical</t>
+  </si>
+  <si>
+    <t>Hydraulics</t>
+  </si>
+  <si>
+    <t>ECS</t>
+  </si>
+  <si>
+    <t>Other</t>
+  </si>
+  <si>
+    <t>Avionics</t>
+  </si>
+  <si>
+    <t>Fixed Payload</t>
+  </si>
+  <si>
+    <t>Exp Payload 1</t>
+  </si>
+  <si>
+    <t>Exp Payload 2</t>
+  </si>
+  <si>
+    <t>Fuel 1</t>
+  </si>
+  <si>
+    <t>Fuel 2</t>
+  </si>
+  <si>
+    <t>Fuel 3</t>
+  </si>
+  <si>
+    <t>Weight (lbf)</t>
+  </si>
+  <si>
+    <t>CG X-Location (fT)</t>
+  </si>
+  <si>
+    <t>X-MAC</t>
+  </si>
+  <si>
+    <t>Y-MAC</t>
   </si>
 </sst>
 </file>
@@ -974,7 +1044,28 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="23">
+  <dxfs count="26">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -1552,6 +1643,453 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B886CA18-31EA-4ECA-BF44-35433BB56EEA}">
+  <dimension ref="C5:O30"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="4" max="4" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="5" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="6" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C6" s="1"/>
+      <c r="D6" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="F6" s="7"/>
+      <c r="G6" s="7"/>
+      <c r="H6" s="7"/>
+      <c r="I6" s="7"/>
+      <c r="J6" s="7"/>
+      <c r="K6" s="7"/>
+      <c r="L6" s="7"/>
+      <c r="M6" s="7"/>
+      <c r="N6" s="7"/>
+      <c r="O6" s="8"/>
+    </row>
+    <row r="7" spans="3:15" ht="60" x14ac:dyDescent="0.25">
+      <c r="C7" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="D7" s="9">
+        <f>3.33*10^(-5)</f>
+        <v>3.3300000000000003E-5</v>
+      </c>
+      <c r="E7" s="9">
+        <f>1.015*10^(-5)</f>
+        <v>1.0149999999999999E-5</v>
+      </c>
+      <c r="F7" s="9"/>
+      <c r="G7" s="9"/>
+      <c r="H7" s="11"/>
+      <c r="I7" s="11"/>
+      <c r="J7" s="11"/>
+      <c r="K7" s="11"/>
+      <c r="L7" s="11"/>
+      <c r="M7" s="11"/>
+      <c r="N7" s="10"/>
+      <c r="O7" s="10"/>
+    </row>
+    <row r="8" spans="3:15" ht="30" x14ac:dyDescent="0.25">
+      <c r="C8" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="D8" s="12">
+        <f>2.08*10^(-5)</f>
+        <v>2.0800000000000001E-5</v>
+      </c>
+      <c r="E8" s="12">
+        <f>0.634*10^(-5)</f>
+        <v>6.3400000000000003E-6</v>
+      </c>
+      <c r="F8" s="12"/>
+      <c r="G8" s="12"/>
+      <c r="H8" s="12"/>
+      <c r="I8" s="12"/>
+      <c r="J8" s="12"/>
+      <c r="K8" s="10"/>
+      <c r="L8" s="10"/>
+      <c r="M8" s="10"/>
+      <c r="N8" s="10"/>
+      <c r="O8" s="10"/>
+    </row>
+    <row r="9" spans="3:15" ht="45" x14ac:dyDescent="0.25">
+      <c r="C9" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="D9" s="12">
+        <f>1.33*10^(-5)</f>
+        <v>1.3300000000000001E-5</v>
+      </c>
+      <c r="E9" s="12">
+        <f>0.405*10^(-5)</f>
+        <v>4.0500000000000002E-6</v>
+      </c>
+      <c r="F9" s="12"/>
+      <c r="G9" s="12"/>
+      <c r="H9" s="12"/>
+      <c r="I9" s="12"/>
+      <c r="J9" s="12"/>
+      <c r="K9" s="10"/>
+      <c r="L9" s="10"/>
+      <c r="M9" s="10"/>
+      <c r="N9" s="10"/>
+      <c r="O9" s="10"/>
+    </row>
+    <row r="10" spans="3:15" ht="45" x14ac:dyDescent="0.25">
+      <c r="C10" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="D10" s="12">
+        <f>0.5*10^(-5)</f>
+        <v>5.0000000000000004E-6</v>
+      </c>
+      <c r="E10" s="12">
+        <f>0.152*10^(-5)</f>
+        <v>1.5200000000000001E-6</v>
+      </c>
+      <c r="F10" s="12"/>
+      <c r="G10" s="12"/>
+      <c r="H10" s="10"/>
+      <c r="I10" s="10"/>
+      <c r="J10" s="10"/>
+      <c r="K10" s="10"/>
+      <c r="L10" s="10"/>
+      <c r="M10" s="10"/>
+      <c r="N10" s="10"/>
+      <c r="O10" s="10"/>
+    </row>
+    <row r="11" spans="3:15" ht="60" x14ac:dyDescent="0.25">
+      <c r="C11" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="D11" s="12">
+        <f>0.7*10^(-5)</f>
+        <v>6.9999999999999999E-6</v>
+      </c>
+      <c r="E11" s="12">
+        <f>0.052*10^(-5)</f>
+        <v>5.2E-7</v>
+      </c>
+      <c r="F11" s="12"/>
+      <c r="G11" s="12"/>
+      <c r="H11" s="10"/>
+      <c r="I11" s="10"/>
+      <c r="J11" s="10"/>
+      <c r="K11" s="10"/>
+      <c r="L11" s="10"/>
+      <c r="M11" s="10"/>
+      <c r="N11" s="10"/>
+      <c r="O11" s="10"/>
+    </row>
+    <row r="12" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C12" s="5"/>
+      <c r="D12" s="12"/>
+      <c r="E12" s="12"/>
+      <c r="F12" s="12"/>
+      <c r="G12" s="12"/>
+      <c r="H12" s="10"/>
+      <c r="I12" s="10"/>
+      <c r="J12" s="10"/>
+      <c r="K12" s="10"/>
+      <c r="L12" s="10"/>
+      <c r="M12" s="10"/>
+      <c r="N12" s="10"/>
+      <c r="O12" s="10"/>
+    </row>
+    <row r="13" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C13" s="5"/>
+      <c r="D13" s="12"/>
+      <c r="E13" s="12"/>
+      <c r="F13" s="12"/>
+      <c r="G13" s="12"/>
+      <c r="H13" s="10"/>
+      <c r="I13" s="10"/>
+      <c r="J13" s="10"/>
+      <c r="K13" s="10"/>
+      <c r="L13" s="10"/>
+      <c r="M13" s="10"/>
+      <c r="N13" s="10"/>
+      <c r="O13" s="10"/>
+    </row>
+    <row r="14" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C14" s="5"/>
+      <c r="D14" s="12"/>
+      <c r="E14" s="12"/>
+      <c r="F14" s="12"/>
+      <c r="G14" s="12"/>
+      <c r="H14" s="10"/>
+      <c r="I14" s="10"/>
+      <c r="J14" s="10"/>
+      <c r="K14" s="10"/>
+      <c r="L14" s="10"/>
+      <c r="M14" s="10"/>
+      <c r="N14" s="10"/>
+      <c r="O14" s="10"/>
+    </row>
+    <row r="15" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C15" s="5"/>
+      <c r="D15" s="12"/>
+      <c r="E15" s="12"/>
+      <c r="F15" s="12"/>
+      <c r="G15" s="12"/>
+      <c r="H15" s="10"/>
+      <c r="I15" s="10"/>
+      <c r="J15" s="10"/>
+      <c r="K15" s="10"/>
+      <c r="L15" s="10"/>
+      <c r="M15" s="10"/>
+      <c r="N15" s="10"/>
+      <c r="O15" s="10"/>
+    </row>
+    <row r="16" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C16" s="5"/>
+      <c r="D16" s="12"/>
+      <c r="E16" s="12"/>
+      <c r="F16" s="12"/>
+      <c r="G16" s="12"/>
+      <c r="H16" s="10"/>
+      <c r="I16" s="10"/>
+      <c r="J16" s="10"/>
+      <c r="K16" s="10"/>
+      <c r="L16" s="10"/>
+      <c r="M16" s="10"/>
+      <c r="N16" s="10"/>
+      <c r="O16" s="10"/>
+    </row>
+    <row r="17" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C17" s="5"/>
+      <c r="D17" s="12"/>
+      <c r="E17" s="12"/>
+      <c r="F17" s="12"/>
+      <c r="G17" s="12"/>
+      <c r="H17" s="10"/>
+      <c r="I17" s="10"/>
+      <c r="J17" s="10"/>
+      <c r="K17" s="10"/>
+      <c r="L17" s="10"/>
+      <c r="M17" s="10"/>
+      <c r="N17" s="10"/>
+      <c r="O17" s="10"/>
+    </row>
+    <row r="18" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C18" s="5"/>
+      <c r="D18" s="12"/>
+      <c r="E18" s="12"/>
+      <c r="F18" s="12"/>
+      <c r="G18" s="12"/>
+      <c r="H18" s="10"/>
+      <c r="I18" s="10"/>
+      <c r="J18" s="10"/>
+      <c r="K18" s="10"/>
+      <c r="L18" s="10"/>
+      <c r="M18" s="10"/>
+      <c r="N18" s="10"/>
+      <c r="O18" s="10"/>
+    </row>
+    <row r="19" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C19" s="5"/>
+      <c r="D19" s="12"/>
+      <c r="E19" s="12"/>
+      <c r="F19" s="12"/>
+      <c r="G19" s="12"/>
+      <c r="H19" s="10"/>
+      <c r="I19" s="10"/>
+      <c r="J19" s="10"/>
+      <c r="K19" s="10"/>
+      <c r="L19" s="10"/>
+      <c r="M19" s="10"/>
+      <c r="N19" s="10"/>
+      <c r="O19" s="10"/>
+    </row>
+    <row r="20" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C20" s="5"/>
+      <c r="D20" s="12"/>
+      <c r="E20" s="12"/>
+      <c r="F20" s="12"/>
+      <c r="G20" s="12"/>
+      <c r="H20" s="10"/>
+      <c r="I20" s="10"/>
+      <c r="J20" s="10"/>
+      <c r="K20" s="10"/>
+      <c r="L20" s="10"/>
+      <c r="M20" s="10"/>
+      <c r="N20" s="10"/>
+      <c r="O20" s="10"/>
+    </row>
+    <row r="21" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C21" s="5"/>
+      <c r="D21" s="12"/>
+      <c r="E21" s="12"/>
+      <c r="F21" s="12"/>
+      <c r="G21" s="12"/>
+      <c r="H21" s="10"/>
+      <c r="I21" s="10"/>
+      <c r="J21" s="10"/>
+      <c r="K21" s="10"/>
+      <c r="L21" s="10"/>
+      <c r="M21" s="10"/>
+      <c r="N21" s="10"/>
+      <c r="O21" s="10"/>
+    </row>
+    <row r="22" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C22" s="5"/>
+      <c r="D22" s="12"/>
+      <c r="E22" s="12"/>
+      <c r="F22" s="12"/>
+      <c r="G22" s="12"/>
+      <c r="H22" s="10"/>
+      <c r="I22" s="10"/>
+      <c r="J22" s="10"/>
+      <c r="K22" s="10"/>
+      <c r="L22" s="10"/>
+      <c r="M22" s="10"/>
+      <c r="N22" s="10"/>
+      <c r="O22" s="10"/>
+    </row>
+    <row r="23" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C23" s="5"/>
+      <c r="D23" s="12"/>
+      <c r="E23" s="10"/>
+      <c r="F23" s="10"/>
+      <c r="G23" s="10"/>
+      <c r="H23" s="10"/>
+      <c r="I23" s="10"/>
+      <c r="J23" s="10"/>
+      <c r="K23" s="10"/>
+      <c r="L23" s="10"/>
+      <c r="M23" s="10"/>
+      <c r="N23" s="10"/>
+      <c r="O23" s="10"/>
+    </row>
+    <row r="24" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C24" s="5"/>
+      <c r="D24" s="12"/>
+      <c r="E24" s="10"/>
+      <c r="F24" s="10"/>
+      <c r="G24" s="10"/>
+      <c r="H24" s="10"/>
+      <c r="I24" s="10"/>
+      <c r="J24" s="10"/>
+      <c r="K24" s="10"/>
+      <c r="L24" s="10"/>
+      <c r="M24" s="10"/>
+      <c r="N24" s="10"/>
+      <c r="O24" s="10"/>
+    </row>
+    <row r="25" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C25" s="5"/>
+      <c r="D25" s="12"/>
+      <c r="E25" s="10"/>
+      <c r="F25" s="10"/>
+      <c r="G25" s="10"/>
+      <c r="H25" s="10"/>
+      <c r="I25" s="10"/>
+      <c r="J25" s="10"/>
+      <c r="K25" s="10"/>
+      <c r="L25" s="10"/>
+      <c r="M25" s="10"/>
+      <c r="N25" s="10"/>
+      <c r="O25" s="10"/>
+    </row>
+    <row r="26" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C26" s="5"/>
+      <c r="D26" s="12"/>
+      <c r="E26" s="10"/>
+      <c r="F26" s="10"/>
+      <c r="G26" s="10"/>
+      <c r="H26" s="10"/>
+      <c r="I26" s="10"/>
+      <c r="J26" s="10"/>
+      <c r="K26" s="10"/>
+      <c r="L26" s="10"/>
+      <c r="M26" s="10"/>
+      <c r="N26" s="10"/>
+      <c r="O26" s="10"/>
+    </row>
+    <row r="27" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C27" s="5"/>
+      <c r="D27" s="12"/>
+      <c r="E27" s="10"/>
+      <c r="F27" s="10"/>
+      <c r="G27" s="10"/>
+      <c r="H27" s="10"/>
+      <c r="I27" s="10"/>
+      <c r="J27" s="10"/>
+      <c r="K27" s="10"/>
+      <c r="L27" s="10"/>
+      <c r="M27" s="10"/>
+      <c r="N27" s="10"/>
+      <c r="O27" s="10"/>
+    </row>
+    <row r="28" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C28" s="5"/>
+      <c r="D28" s="12"/>
+      <c r="E28" s="10"/>
+      <c r="F28" s="10"/>
+      <c r="G28" s="10"/>
+      <c r="H28" s="10"/>
+      <c r="I28" s="10"/>
+      <c r="J28" s="10"/>
+      <c r="K28" s="10"/>
+      <c r="L28" s="10"/>
+      <c r="M28" s="10"/>
+      <c r="N28" s="10"/>
+      <c r="O28" s="10"/>
+    </row>
+    <row r="29" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C29" s="5"/>
+      <c r="D29" s="12"/>
+      <c r="E29" s="10"/>
+      <c r="F29" s="10"/>
+      <c r="G29" s="10"/>
+      <c r="H29" s="10"/>
+      <c r="I29" s="10"/>
+      <c r="J29" s="10"/>
+      <c r="K29" s="10"/>
+      <c r="L29" s="10"/>
+      <c r="M29" s="10"/>
+      <c r="N29" s="10"/>
+      <c r="O29" s="10"/>
+    </row>
+    <row r="30" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C30" s="5"/>
+      <c r="D30" s="12"/>
+      <c r="E30" s="10"/>
+      <c r="F30" s="10"/>
+      <c r="G30" s="10"/>
+      <c r="H30" s="10"/>
+      <c r="I30" s="10"/>
+      <c r="J30" s="10"/>
+      <c r="K30" s="10"/>
+      <c r="L30" s="10"/>
+      <c r="M30" s="10"/>
+      <c r="N30" s="10"/>
+      <c r="O30" s="10"/>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="D7:O30">
+    <cfRule type="expression" dxfId="5" priority="2">
+      <formula>_xlfn.ISFORMULA(D7)</formula>
+    </cfRule>
+    <cfRule type="containsBlanks" dxfId="4" priority="3">
+      <formula>LEN(TRIM(D7))=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G16">
+    <cfRule type="expression" dxfId="3" priority="1">
+      <formula>ISNOTFORMULA(D7)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5A6F23B-4C6A-46FF-A5EA-3CA7645F338A}">
   <dimension ref="B8:N37"/>
@@ -1965,15 +2503,15 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="C14:N37">
-    <cfRule type="expression" dxfId="22" priority="2">
+    <cfRule type="expression" dxfId="25" priority="2">
       <formula>_xlfn.ISFORMULA(C14)</formula>
     </cfRule>
-    <cfRule type="containsBlanks" dxfId="21" priority="3">
+    <cfRule type="containsBlanks" dxfId="24" priority="3">
       <formula>LEN(TRIM(C14))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F23">
-    <cfRule type="expression" dxfId="20" priority="1">
+    <cfRule type="expression" dxfId="23" priority="1">
       <formula>ISNOTFORMULA(C14)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2408,15 +2946,15 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="D6:O29">
-    <cfRule type="expression" dxfId="19" priority="2">
+    <cfRule type="expression" dxfId="22" priority="2">
       <formula>_xlfn.ISFORMULA(D6)</formula>
     </cfRule>
-    <cfRule type="containsBlanks" dxfId="18" priority="3">
+    <cfRule type="containsBlanks" dxfId="21" priority="3">
       <formula>LEN(TRIM(D6))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G15">
-    <cfRule type="expression" dxfId="17" priority="1">
+    <cfRule type="expression" dxfId="20" priority="1">
       <formula>ISNOTFORMULA(D6)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3156,13 +3694,13 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="C14:N40">
-    <cfRule type="expression" dxfId="16" priority="1">
+    <cfRule type="expression" dxfId="19" priority="1">
       <formula>ISNOTFORMULA(C14)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="15" priority="2">
+    <cfRule type="expression" dxfId="18" priority="2">
       <formula>_xlfn.ISFORMULA(C14)</formula>
     </cfRule>
-    <cfRule type="containsBlanks" dxfId="14" priority="3">
+    <cfRule type="containsBlanks" dxfId="17" priority="3">
       <formula>LEN(TRIM(C14))=0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3631,13 +4169,13 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="C14:N37">
-    <cfRule type="expression" dxfId="13" priority="1">
+    <cfRule type="expression" dxfId="16" priority="1">
       <formula>ISNOTFORMULA(C14)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="12" priority="2">
+    <cfRule type="expression" dxfId="15" priority="2">
       <formula>_xlfn.ISFORMULA(C14)</formula>
     </cfRule>
-    <cfRule type="containsBlanks" dxfId="11" priority="3">
+    <cfRule type="containsBlanks" dxfId="14" priority="3">
       <formula>LEN(TRIM(C14))=0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4088,10 +4626,10 @@
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
   <conditionalFormatting sqref="C14:N37">
-    <cfRule type="expression" dxfId="10" priority="2">
+    <cfRule type="expression" dxfId="13" priority="2">
       <formula>_xlfn.ISFORMULA(C14)</formula>
     </cfRule>
-    <cfRule type="containsBlanks" dxfId="9" priority="3">
+    <cfRule type="containsBlanks" dxfId="12" priority="3">
       <formula>LEN(TRIM(C14))=0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6147,15 +6685,15 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="C4:N107">
-    <cfRule type="expression" dxfId="8" priority="2">
+    <cfRule type="expression" dxfId="11" priority="2">
       <formula>_xlfn.ISFORMULA(C4)</formula>
     </cfRule>
-    <cfRule type="containsBlanks" dxfId="7" priority="3">
+    <cfRule type="containsBlanks" dxfId="10" priority="3">
       <formula>LEN(TRIM(C4))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F16:F17">
-    <cfRule type="expression" dxfId="6" priority="1">
+    <cfRule type="expression" dxfId="9" priority="1">
       <formula>ISNOTFORMULA(C3)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6164,6 +6702,459 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F4989AF-198A-4CC1-9095-07C71A58C4DB}">
+  <dimension ref="D6:P31"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="6" spans="4:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="7" spans="4:16" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D7" s="1"/>
+      <c r="E7" s="6" t="s">
+        <v>222</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>223</v>
+      </c>
+      <c r="G7" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="H7" s="7" t="s">
+        <v>225</v>
+      </c>
+      <c r="I7" s="7"/>
+      <c r="J7" s="7"/>
+      <c r="K7" s="7"/>
+      <c r="L7" s="7"/>
+      <c r="M7" s="7"/>
+      <c r="N7" s="7"/>
+      <c r="O7" s="7"/>
+      <c r="P7" s="8"/>
+    </row>
+    <row r="8" spans="4:16" x14ac:dyDescent="0.25">
+      <c r="D8" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="E8" s="9">
+        <v>0</v>
+      </c>
+      <c r="F8" s="9">
+        <v>27.28</v>
+      </c>
+      <c r="G8" s="9"/>
+      <c r="H8" s="9"/>
+      <c r="I8" s="11"/>
+      <c r="J8" s="11"/>
+      <c r="K8" s="11"/>
+      <c r="L8" s="11"/>
+      <c r="M8" s="11"/>
+      <c r="N8" s="11"/>
+      <c r="O8" s="10"/>
+      <c r="P8" s="10"/>
+    </row>
+    <row r="9" spans="4:16" x14ac:dyDescent="0.25">
+      <c r="D9" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E9" s="12"/>
+      <c r="F9" s="12"/>
+      <c r="G9" s="12"/>
+      <c r="H9" s="12"/>
+      <c r="I9" s="12"/>
+      <c r="J9" s="12"/>
+      <c r="K9" s="12"/>
+      <c r="L9" s="10"/>
+      <c r="M9" s="10"/>
+      <c r="N9" s="10"/>
+      <c r="O9" s="10"/>
+      <c r="P9" s="10"/>
+    </row>
+    <row r="10" spans="4:16" x14ac:dyDescent="0.25">
+      <c r="D10" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="E10" s="12"/>
+      <c r="F10" s="12"/>
+      <c r="G10" s="12"/>
+      <c r="H10" s="12"/>
+      <c r="I10" s="12"/>
+      <c r="J10" s="12"/>
+      <c r="K10" s="12"/>
+      <c r="L10" s="10"/>
+      <c r="M10" s="10"/>
+      <c r="N10" s="10"/>
+      <c r="O10" s="10"/>
+      <c r="P10" s="10"/>
+    </row>
+    <row r="11" spans="4:16" x14ac:dyDescent="0.25">
+      <c r="D11" s="4" t="s">
+        <v>205</v>
+      </c>
+      <c r="E11" s="12"/>
+      <c r="F11" s="12"/>
+      <c r="G11" s="12"/>
+      <c r="H11" s="12"/>
+      <c r="I11" s="10"/>
+      <c r="J11" s="10"/>
+      <c r="K11" s="10"/>
+      <c r="L11" s="10"/>
+      <c r="M11" s="10"/>
+      <c r="N11" s="10"/>
+      <c r="O11" s="10"/>
+      <c r="P11" s="10"/>
+    </row>
+    <row r="12" spans="4:16" x14ac:dyDescent="0.25">
+      <c r="D12" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="E12" s="12"/>
+      <c r="F12" s="12"/>
+      <c r="G12" s="12"/>
+      <c r="H12" s="12"/>
+      <c r="I12" s="10"/>
+      <c r="J12" s="10"/>
+      <c r="K12" s="10"/>
+      <c r="L12" s="10"/>
+      <c r="M12" s="10"/>
+      <c r="N12" s="10"/>
+      <c r="O12" s="10"/>
+      <c r="P12" s="10"/>
+    </row>
+    <row r="13" spans="4:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D13" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E13" s="12"/>
+      <c r="F13" s="12"/>
+      <c r="G13" s="12"/>
+      <c r="H13" s="12"/>
+      <c r="I13" s="10"/>
+      <c r="J13" s="10"/>
+      <c r="K13" s="10"/>
+      <c r="L13" s="10"/>
+      <c r="M13" s="10"/>
+      <c r="N13" s="10"/>
+      <c r="O13" s="10"/>
+      <c r="P13" s="10"/>
+    </row>
+    <row r="14" spans="4:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D14" s="5" t="s">
+        <v>207</v>
+      </c>
+      <c r="E14" s="12"/>
+      <c r="F14" s="12"/>
+      <c r="G14" s="12"/>
+      <c r="H14" s="12"/>
+      <c r="I14" s="10"/>
+      <c r="J14" s="10"/>
+      <c r="K14" s="10"/>
+      <c r="L14" s="10"/>
+      <c r="M14" s="10"/>
+      <c r="N14" s="10"/>
+      <c r="O14" s="10"/>
+      <c r="P14" s="10"/>
+    </row>
+    <row r="15" spans="4:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D15" s="5" t="s">
+        <v>208</v>
+      </c>
+      <c r="E15" s="12"/>
+      <c r="F15" s="12"/>
+      <c r="G15" s="12"/>
+      <c r="H15" s="12"/>
+      <c r="I15" s="10"/>
+      <c r="J15" s="10"/>
+      <c r="K15" s="10"/>
+      <c r="L15" s="10"/>
+      <c r="M15" s="10"/>
+      <c r="N15" s="10"/>
+      <c r="O15" s="10"/>
+      <c r="P15" s="10"/>
+    </row>
+    <row r="16" spans="4:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D16" s="5" t="s">
+        <v>209</v>
+      </c>
+      <c r="E16" s="12"/>
+      <c r="F16" s="12"/>
+      <c r="G16" s="12"/>
+      <c r="H16" s="12"/>
+      <c r="I16" s="10"/>
+      <c r="J16" s="10"/>
+      <c r="K16" s="10"/>
+      <c r="L16" s="10"/>
+      <c r="M16" s="10"/>
+      <c r="N16" s="10"/>
+      <c r="O16" s="10"/>
+      <c r="P16" s="10"/>
+    </row>
+    <row r="17" spans="4:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D17" s="5" t="s">
+        <v>210</v>
+      </c>
+      <c r="E17" s="12"/>
+      <c r="F17" s="12"/>
+      <c r="G17" s="12"/>
+      <c r="H17" s="12"/>
+      <c r="I17" s="10"/>
+      <c r="J17" s="10"/>
+      <c r="K17" s="10"/>
+      <c r="L17" s="10"/>
+      <c r="M17" s="10"/>
+      <c r="N17" s="10"/>
+      <c r="O17" s="10"/>
+      <c r="P17" s="10"/>
+    </row>
+    <row r="18" spans="4:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D18" s="5" t="s">
+        <v>211</v>
+      </c>
+      <c r="E18" s="12"/>
+      <c r="F18" s="12"/>
+      <c r="G18" s="12"/>
+      <c r="H18" s="12"/>
+      <c r="I18" s="10"/>
+      <c r="J18" s="10"/>
+      <c r="K18" s="10"/>
+      <c r="L18" s="10"/>
+      <c r="M18" s="10"/>
+      <c r="N18" s="10"/>
+      <c r="O18" s="10"/>
+      <c r="P18" s="10"/>
+    </row>
+    <row r="19" spans="4:16" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D19" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="E19" s="12"/>
+      <c r="F19" s="12"/>
+      <c r="G19" s="12"/>
+      <c r="H19" s="12"/>
+      <c r="I19" s="10"/>
+      <c r="J19" s="10"/>
+      <c r="K19" s="10"/>
+      <c r="L19" s="10"/>
+      <c r="M19" s="10"/>
+      <c r="N19" s="10"/>
+      <c r="O19" s="10"/>
+      <c r="P19" s="10"/>
+    </row>
+    <row r="20" spans="4:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D20" s="5" t="s">
+        <v>213</v>
+      </c>
+      <c r="E20" s="12"/>
+      <c r="F20" s="12"/>
+      <c r="G20" s="12"/>
+      <c r="H20" s="12"/>
+      <c r="I20" s="10"/>
+      <c r="J20" s="10"/>
+      <c r="K20" s="10"/>
+      <c r="L20" s="10"/>
+      <c r="M20" s="10"/>
+      <c r="N20" s="10"/>
+      <c r="O20" s="10"/>
+      <c r="P20" s="10"/>
+    </row>
+    <row r="21" spans="4:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D21" s="5" t="s">
+        <v>214</v>
+      </c>
+      <c r="E21" s="12"/>
+      <c r="F21" s="12"/>
+      <c r="G21" s="12"/>
+      <c r="H21" s="12"/>
+      <c r="I21" s="10"/>
+      <c r="J21" s="10"/>
+      <c r="K21" s="10"/>
+      <c r="L21" s="10"/>
+      <c r="M21" s="10"/>
+      <c r="N21" s="10"/>
+      <c r="O21" s="10"/>
+      <c r="P21" s="10"/>
+    </row>
+    <row r="22" spans="4:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D22" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="E22" s="12"/>
+      <c r="F22" s="12"/>
+      <c r="G22" s="12"/>
+      <c r="H22" s="12"/>
+      <c r="I22" s="10"/>
+      <c r="J22" s="10"/>
+      <c r="K22" s="10"/>
+      <c r="L22" s="10"/>
+      <c r="M22" s="10"/>
+      <c r="N22" s="10"/>
+      <c r="O22" s="10"/>
+      <c r="P22" s="10"/>
+    </row>
+    <row r="23" spans="4:16" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D23" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="E23" s="12"/>
+      <c r="F23" s="12"/>
+      <c r="G23" s="12"/>
+      <c r="H23" s="12"/>
+      <c r="I23" s="10"/>
+      <c r="J23" s="10"/>
+      <c r="K23" s="10"/>
+      <c r="L23" s="10"/>
+      <c r="M23" s="10"/>
+      <c r="N23" s="10"/>
+      <c r="O23" s="10"/>
+      <c r="P23" s="10"/>
+    </row>
+    <row r="24" spans="4:16" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D24" s="5" t="s">
+        <v>217</v>
+      </c>
+      <c r="E24" s="12"/>
+      <c r="F24" s="10"/>
+      <c r="G24" s="10"/>
+      <c r="H24" s="10"/>
+      <c r="I24" s="10"/>
+      <c r="J24" s="10"/>
+      <c r="K24" s="10"/>
+      <c r="L24" s="10"/>
+      <c r="M24" s="10"/>
+      <c r="N24" s="10"/>
+      <c r="O24" s="10"/>
+      <c r="P24" s="10"/>
+    </row>
+    <row r="25" spans="4:16" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D25" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="E25" s="12"/>
+      <c r="F25" s="10"/>
+      <c r="G25" s="10"/>
+      <c r="H25" s="10"/>
+      <c r="I25" s="10"/>
+      <c r="J25" s="10"/>
+      <c r="K25" s="10"/>
+      <c r="L25" s="10"/>
+      <c r="M25" s="10"/>
+      <c r="N25" s="10"/>
+      <c r="O25" s="10"/>
+      <c r="P25" s="10"/>
+    </row>
+    <row r="26" spans="4:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D26" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="E26" s="12"/>
+      <c r="F26" s="10"/>
+      <c r="G26" s="10"/>
+      <c r="H26" s="10"/>
+      <c r="I26" s="10"/>
+      <c r="J26" s="10"/>
+      <c r="K26" s="10"/>
+      <c r="L26" s="10"/>
+      <c r="M26" s="10"/>
+      <c r="N26" s="10"/>
+      <c r="O26" s="10"/>
+      <c r="P26" s="10"/>
+    </row>
+    <row r="27" spans="4:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D27" s="5" t="s">
+        <v>220</v>
+      </c>
+      <c r="E27" s="12"/>
+      <c r="F27" s="10"/>
+      <c r="G27" s="10"/>
+      <c r="H27" s="10"/>
+      <c r="I27" s="10"/>
+      <c r="J27" s="10"/>
+      <c r="K27" s="10"/>
+      <c r="L27" s="10"/>
+      <c r="M27" s="10"/>
+      <c r="N27" s="10"/>
+      <c r="O27" s="10"/>
+      <c r="P27" s="10"/>
+    </row>
+    <row r="28" spans="4:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D28" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="E28" s="12"/>
+      <c r="F28" s="10"/>
+      <c r="G28" s="10"/>
+      <c r="H28" s="10"/>
+      <c r="I28" s="10"/>
+      <c r="J28" s="10"/>
+      <c r="K28" s="10"/>
+      <c r="L28" s="10"/>
+      <c r="M28" s="10"/>
+      <c r="N28" s="10"/>
+      <c r="O28" s="10"/>
+      <c r="P28" s="10"/>
+    </row>
+    <row r="29" spans="4:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D29" s="5"/>
+      <c r="E29" s="12"/>
+      <c r="F29" s="10"/>
+      <c r="G29" s="10"/>
+      <c r="H29" s="10"/>
+      <c r="I29" s="10"/>
+      <c r="J29" s="10"/>
+      <c r="K29" s="10"/>
+      <c r="L29" s="10"/>
+      <c r="M29" s="10"/>
+      <c r="N29" s="10"/>
+      <c r="O29" s="10"/>
+      <c r="P29" s="10"/>
+    </row>
+    <row r="30" spans="4:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D30" s="5"/>
+      <c r="E30" s="12"/>
+      <c r="F30" s="10"/>
+      <c r="G30" s="10"/>
+      <c r="H30" s="10"/>
+      <c r="I30" s="10"/>
+      <c r="J30" s="10"/>
+      <c r="K30" s="10"/>
+      <c r="L30" s="10"/>
+      <c r="M30" s="10"/>
+      <c r="N30" s="10"/>
+      <c r="O30" s="10"/>
+      <c r="P30" s="10"/>
+    </row>
+    <row r="31" spans="4:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D31" s="5"/>
+      <c r="E31" s="12"/>
+      <c r="F31" s="10"/>
+      <c r="G31" s="10"/>
+      <c r="H31" s="10"/>
+      <c r="I31" s="10"/>
+      <c r="J31" s="10"/>
+      <c r="K31" s="10"/>
+      <c r="L31" s="10"/>
+      <c r="M31" s="10"/>
+      <c r="N31" s="10"/>
+      <c r="O31" s="10"/>
+      <c r="P31" s="10"/>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="E8:P31">
+    <cfRule type="expression" dxfId="2" priority="2">
+      <formula>_xlfn.ISFORMULA(E8)</formula>
+    </cfRule>
+    <cfRule type="containsBlanks" dxfId="1" priority="3">
+      <formula>LEN(TRIM(E8))=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H17">
+    <cfRule type="expression" dxfId="0" priority="1">
+      <formula>ISNOTFORMULA(E8)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{41AFF542-1B93-43EB-9BE7-8E21B1D3B06C}">
   <dimension ref="D5:P34"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -6601,465 +7592,18 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="E11:P34">
-    <cfRule type="expression" dxfId="5" priority="2">
+    <cfRule type="expression" dxfId="8" priority="2">
       <formula>_xlfn.ISFORMULA(E11)</formula>
     </cfRule>
-    <cfRule type="containsBlanks" dxfId="4" priority="3">
+    <cfRule type="containsBlanks" dxfId="7" priority="3">
       <formula>LEN(TRIM(E11))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H20">
-    <cfRule type="expression" dxfId="3" priority="1">
+    <cfRule type="expression" dxfId="6" priority="1">
       <formula>ISNOTFORMULA(E11)</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B886CA18-31EA-4ECA-BF44-35433BB56EEA}">
-  <dimension ref="C5:O30"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="4" max="4" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.85546875" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="5" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="6" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C6" s="1"/>
-      <c r="D6" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>161</v>
-      </c>
-      <c r="F6" s="7"/>
-      <c r="G6" s="7"/>
-      <c r="H6" s="7"/>
-      <c r="I6" s="7"/>
-      <c r="J6" s="7"/>
-      <c r="K6" s="7"/>
-      <c r="L6" s="7"/>
-      <c r="M6" s="7"/>
-      <c r="N6" s="7"/>
-      <c r="O6" s="8"/>
-    </row>
-    <row r="7" spans="3:15" ht="60" x14ac:dyDescent="0.25">
-      <c r="C7" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="D7" s="9">
-        <f>3.33*10^(-5)</f>
-        <v>3.3300000000000003E-5</v>
-      </c>
-      <c r="E7" s="9">
-        <f>1.015*10^(-5)</f>
-        <v>1.0149999999999999E-5</v>
-      </c>
-      <c r="F7" s="9"/>
-      <c r="G7" s="9"/>
-      <c r="H7" s="11"/>
-      <c r="I7" s="11"/>
-      <c r="J7" s="11"/>
-      <c r="K7" s="11"/>
-      <c r="L7" s="11"/>
-      <c r="M7" s="11"/>
-      <c r="N7" s="10"/>
-      <c r="O7" s="10"/>
-    </row>
-    <row r="8" spans="3:15" ht="30" x14ac:dyDescent="0.25">
-      <c r="C8" s="4" t="s">
-        <v>164</v>
-      </c>
-      <c r="D8" s="12">
-        <f>2.08*10^(-5)</f>
-        <v>2.0800000000000001E-5</v>
-      </c>
-      <c r="E8" s="12">
-        <f>0.634*10^(-5)</f>
-        <v>6.3400000000000003E-6</v>
-      </c>
-      <c r="F8" s="12"/>
-      <c r="G8" s="12"/>
-      <c r="H8" s="12"/>
-      <c r="I8" s="12"/>
-      <c r="J8" s="12"/>
-      <c r="K8" s="10"/>
-      <c r="L8" s="10"/>
-      <c r="M8" s="10"/>
-      <c r="N8" s="10"/>
-      <c r="O8" s="10"/>
-    </row>
-    <row r="9" spans="3:15" ht="45" x14ac:dyDescent="0.25">
-      <c r="C9" s="4" t="s">
-        <v>165</v>
-      </c>
-      <c r="D9" s="12">
-        <f>1.33*10^(-5)</f>
-        <v>1.3300000000000001E-5</v>
-      </c>
-      <c r="E9" s="12">
-        <f>0.405*10^(-5)</f>
-        <v>4.0500000000000002E-6</v>
-      </c>
-      <c r="F9" s="12"/>
-      <c r="G9" s="12"/>
-      <c r="H9" s="12"/>
-      <c r="I9" s="12"/>
-      <c r="J9" s="12"/>
-      <c r="K9" s="10"/>
-      <c r="L9" s="10"/>
-      <c r="M9" s="10"/>
-      <c r="N9" s="10"/>
-      <c r="O9" s="10"/>
-    </row>
-    <row r="10" spans="3:15" ht="45" x14ac:dyDescent="0.25">
-      <c r="C10" s="4" t="s">
-        <v>166</v>
-      </c>
-      <c r="D10" s="12">
-        <f>0.5*10^(-5)</f>
-        <v>5.0000000000000004E-6</v>
-      </c>
-      <c r="E10" s="12">
-        <f>0.152*10^(-5)</f>
-        <v>1.5200000000000001E-6</v>
-      </c>
-      <c r="F10" s="12"/>
-      <c r="G10" s="12"/>
-      <c r="H10" s="10"/>
-      <c r="I10" s="10"/>
-      <c r="J10" s="10"/>
-      <c r="K10" s="10"/>
-      <c r="L10" s="10"/>
-      <c r="M10" s="10"/>
-      <c r="N10" s="10"/>
-      <c r="O10" s="10"/>
-    </row>
-    <row r="11" spans="3:15" ht="60" x14ac:dyDescent="0.25">
-      <c r="C11" s="4" t="s">
-        <v>167</v>
-      </c>
-      <c r="D11" s="12">
-        <f>0.7*10^(-5)</f>
-        <v>6.9999999999999999E-6</v>
-      </c>
-      <c r="E11" s="12">
-        <f>0.052*10^(-5)</f>
-        <v>5.2E-7</v>
-      </c>
-      <c r="F11" s="12"/>
-      <c r="G11" s="12"/>
-      <c r="H11" s="10"/>
-      <c r="I11" s="10"/>
-      <c r="J11" s="10"/>
-      <c r="K11" s="10"/>
-      <c r="L11" s="10"/>
-      <c r="M11" s="10"/>
-      <c r="N11" s="10"/>
-      <c r="O11" s="10"/>
-    </row>
-    <row r="12" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C12" s="5"/>
-      <c r="D12" s="12"/>
-      <c r="E12" s="12"/>
-      <c r="F12" s="12"/>
-      <c r="G12" s="12"/>
-      <c r="H12" s="10"/>
-      <c r="I12" s="10"/>
-      <c r="J12" s="10"/>
-      <c r="K12" s="10"/>
-      <c r="L12" s="10"/>
-      <c r="M12" s="10"/>
-      <c r="N12" s="10"/>
-      <c r="O12" s="10"/>
-    </row>
-    <row r="13" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C13" s="5"/>
-      <c r="D13" s="12"/>
-      <c r="E13" s="12"/>
-      <c r="F13" s="12"/>
-      <c r="G13" s="12"/>
-      <c r="H13" s="10"/>
-      <c r="I13" s="10"/>
-      <c r="J13" s="10"/>
-      <c r="K13" s="10"/>
-      <c r="L13" s="10"/>
-      <c r="M13" s="10"/>
-      <c r="N13" s="10"/>
-      <c r="O13" s="10"/>
-    </row>
-    <row r="14" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C14" s="5"/>
-      <c r="D14" s="12"/>
-      <c r="E14" s="12"/>
-      <c r="F14" s="12"/>
-      <c r="G14" s="12"/>
-      <c r="H14" s="10"/>
-      <c r="I14" s="10"/>
-      <c r="J14" s="10"/>
-      <c r="K14" s="10"/>
-      <c r="L14" s="10"/>
-      <c r="M14" s="10"/>
-      <c r="N14" s="10"/>
-      <c r="O14" s="10"/>
-    </row>
-    <row r="15" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C15" s="5"/>
-      <c r="D15" s="12"/>
-      <c r="E15" s="12"/>
-      <c r="F15" s="12"/>
-      <c r="G15" s="12"/>
-      <c r="H15" s="10"/>
-      <c r="I15" s="10"/>
-      <c r="J15" s="10"/>
-      <c r="K15" s="10"/>
-      <c r="L15" s="10"/>
-      <c r="M15" s="10"/>
-      <c r="N15" s="10"/>
-      <c r="O15" s="10"/>
-    </row>
-    <row r="16" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C16" s="5"/>
-      <c r="D16" s="12"/>
-      <c r="E16" s="12"/>
-      <c r="F16" s="12"/>
-      <c r="G16" s="12"/>
-      <c r="H16" s="10"/>
-      <c r="I16" s="10"/>
-      <c r="J16" s="10"/>
-      <c r="K16" s="10"/>
-      <c r="L16" s="10"/>
-      <c r="M16" s="10"/>
-      <c r="N16" s="10"/>
-      <c r="O16" s="10"/>
-    </row>
-    <row r="17" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C17" s="5"/>
-      <c r="D17" s="12"/>
-      <c r="E17" s="12"/>
-      <c r="F17" s="12"/>
-      <c r="G17" s="12"/>
-      <c r="H17" s="10"/>
-      <c r="I17" s="10"/>
-      <c r="J17" s="10"/>
-      <c r="K17" s="10"/>
-      <c r="L17" s="10"/>
-      <c r="M17" s="10"/>
-      <c r="N17" s="10"/>
-      <c r="O17" s="10"/>
-    </row>
-    <row r="18" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C18" s="5"/>
-      <c r="D18" s="12"/>
-      <c r="E18" s="12"/>
-      <c r="F18" s="12"/>
-      <c r="G18" s="12"/>
-      <c r="H18" s="10"/>
-      <c r="I18" s="10"/>
-      <c r="J18" s="10"/>
-      <c r="K18" s="10"/>
-      <c r="L18" s="10"/>
-      <c r="M18" s="10"/>
-      <c r="N18" s="10"/>
-      <c r="O18" s="10"/>
-    </row>
-    <row r="19" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C19" s="5"/>
-      <c r="D19" s="12"/>
-      <c r="E19" s="12"/>
-      <c r="F19" s="12"/>
-      <c r="G19" s="12"/>
-      <c r="H19" s="10"/>
-      <c r="I19" s="10"/>
-      <c r="J19" s="10"/>
-      <c r="K19" s="10"/>
-      <c r="L19" s="10"/>
-      <c r="M19" s="10"/>
-      <c r="N19" s="10"/>
-      <c r="O19" s="10"/>
-    </row>
-    <row r="20" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C20" s="5"/>
-      <c r="D20" s="12"/>
-      <c r="E20" s="12"/>
-      <c r="F20" s="12"/>
-      <c r="G20" s="12"/>
-      <c r="H20" s="10"/>
-      <c r="I20" s="10"/>
-      <c r="J20" s="10"/>
-      <c r="K20" s="10"/>
-      <c r="L20" s="10"/>
-      <c r="M20" s="10"/>
-      <c r="N20" s="10"/>
-      <c r="O20" s="10"/>
-    </row>
-    <row r="21" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C21" s="5"/>
-      <c r="D21" s="12"/>
-      <c r="E21" s="12"/>
-      <c r="F21" s="12"/>
-      <c r="G21" s="12"/>
-      <c r="H21" s="10"/>
-      <c r="I21" s="10"/>
-      <c r="J21" s="10"/>
-      <c r="K21" s="10"/>
-      <c r="L21" s="10"/>
-      <c r="M21" s="10"/>
-      <c r="N21" s="10"/>
-      <c r="O21" s="10"/>
-    </row>
-    <row r="22" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C22" s="5"/>
-      <c r="D22" s="12"/>
-      <c r="E22" s="12"/>
-      <c r="F22" s="12"/>
-      <c r="G22" s="12"/>
-      <c r="H22" s="10"/>
-      <c r="I22" s="10"/>
-      <c r="J22" s="10"/>
-      <c r="K22" s="10"/>
-      <c r="L22" s="10"/>
-      <c r="M22" s="10"/>
-      <c r="N22" s="10"/>
-      <c r="O22" s="10"/>
-    </row>
-    <row r="23" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C23" s="5"/>
-      <c r="D23" s="12"/>
-      <c r="E23" s="10"/>
-      <c r="F23" s="10"/>
-      <c r="G23" s="10"/>
-      <c r="H23" s="10"/>
-      <c r="I23" s="10"/>
-      <c r="J23" s="10"/>
-      <c r="K23" s="10"/>
-      <c r="L23" s="10"/>
-      <c r="M23" s="10"/>
-      <c r="N23" s="10"/>
-      <c r="O23" s="10"/>
-    </row>
-    <row r="24" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C24" s="5"/>
-      <c r="D24" s="12"/>
-      <c r="E24" s="10"/>
-      <c r="F24" s="10"/>
-      <c r="G24" s="10"/>
-      <c r="H24" s="10"/>
-      <c r="I24" s="10"/>
-      <c r="J24" s="10"/>
-      <c r="K24" s="10"/>
-      <c r="L24" s="10"/>
-      <c r="M24" s="10"/>
-      <c r="N24" s="10"/>
-      <c r="O24" s="10"/>
-    </row>
-    <row r="25" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C25" s="5"/>
-      <c r="D25" s="12"/>
-      <c r="E25" s="10"/>
-      <c r="F25" s="10"/>
-      <c r="G25" s="10"/>
-      <c r="H25" s="10"/>
-      <c r="I25" s="10"/>
-      <c r="J25" s="10"/>
-      <c r="K25" s="10"/>
-      <c r="L25" s="10"/>
-      <c r="M25" s="10"/>
-      <c r="N25" s="10"/>
-      <c r="O25" s="10"/>
-    </row>
-    <row r="26" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C26" s="5"/>
-      <c r="D26" s="12"/>
-      <c r="E26" s="10"/>
-      <c r="F26" s="10"/>
-      <c r="G26" s="10"/>
-      <c r="H26" s="10"/>
-      <c r="I26" s="10"/>
-      <c r="J26" s="10"/>
-      <c r="K26" s="10"/>
-      <c r="L26" s="10"/>
-      <c r="M26" s="10"/>
-      <c r="N26" s="10"/>
-      <c r="O26" s="10"/>
-    </row>
-    <row r="27" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C27" s="5"/>
-      <c r="D27" s="12"/>
-      <c r="E27" s="10"/>
-      <c r="F27" s="10"/>
-      <c r="G27" s="10"/>
-      <c r="H27" s="10"/>
-      <c r="I27" s="10"/>
-      <c r="J27" s="10"/>
-      <c r="K27" s="10"/>
-      <c r="L27" s="10"/>
-      <c r="M27" s="10"/>
-      <c r="N27" s="10"/>
-      <c r="O27" s="10"/>
-    </row>
-    <row r="28" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C28" s="5"/>
-      <c r="D28" s="12"/>
-      <c r="E28" s="10"/>
-      <c r="F28" s="10"/>
-      <c r="G28" s="10"/>
-      <c r="H28" s="10"/>
-      <c r="I28" s="10"/>
-      <c r="J28" s="10"/>
-      <c r="K28" s="10"/>
-      <c r="L28" s="10"/>
-      <c r="M28" s="10"/>
-      <c r="N28" s="10"/>
-      <c r="O28" s="10"/>
-    </row>
-    <row r="29" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C29" s="5"/>
-      <c r="D29" s="12"/>
-      <c r="E29" s="10"/>
-      <c r="F29" s="10"/>
-      <c r="G29" s="10"/>
-      <c r="H29" s="10"/>
-      <c r="I29" s="10"/>
-      <c r="J29" s="10"/>
-      <c r="K29" s="10"/>
-      <c r="L29" s="10"/>
-      <c r="M29" s="10"/>
-      <c r="N29" s="10"/>
-      <c r="O29" s="10"/>
-    </row>
-    <row r="30" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C30" s="5"/>
-      <c r="D30" s="12"/>
-      <c r="E30" s="10"/>
-      <c r="F30" s="10"/>
-      <c r="G30" s="10"/>
-      <c r="H30" s="10"/>
-      <c r="I30" s="10"/>
-      <c r="J30" s="10"/>
-      <c r="K30" s="10"/>
-      <c r="L30" s="10"/>
-      <c r="M30" s="10"/>
-      <c r="N30" s="10"/>
-      <c r="O30" s="10"/>
-    </row>
-  </sheetData>
-  <conditionalFormatting sqref="D7:O30">
-    <cfRule type="expression" dxfId="2" priority="2">
-      <formula>_xlfn.ISFORMULA(D7)</formula>
-    </cfRule>
-    <cfRule type="containsBlanks" dxfId="1" priority="3">
-      <formula>LEN(TRIM(D7))=0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G16">
-    <cfRule type="expression" dxfId="0" priority="1">
-      <formula>ISNOTFORMULA(D7)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Added architecture for K_fus.
</commit_message>
<xml_diff>
--- a/examples/F-16A B Block 10 and 15/Operator/F-16A Block 50.xlsx
+++ b/examples/F-16A B Block 10 and 15/Operator/F-16A Block 50.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\John Freeman\Desktop\Academics\VRMastersProgram\code\air-vehicle-design\examples\F-16A B Block 10 and 15\Operator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1C84802-EE5A-49AB-A9E8-F59A9780BC37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B838FC6B-90DB-411C-B3B4-C8E649BF7C29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="384" windowWidth="23256" windowHeight="12720" firstSheet="1" activeTab="5" xr2:uid="{5F5D00AF-8D4A-4BC4-9FDA-F17071C88D94}"/>
+    <workbookView xWindow="22932" yWindow="384" windowWidth="23256" windowHeight="12720" firstSheet="1" activeTab="7" xr2:uid="{5F5D00AF-8D4A-4BC4-9FDA-F17071C88D94}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="228">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="230">
   <si>
     <t>THIS IS FOR THE END USER</t>
   </si>
@@ -729,6 +729,12 @@
   </si>
   <si>
     <t>Inlet Area</t>
+  </si>
+  <si>
+    <t>Kfus</t>
+  </si>
+  <si>
+    <t>x location</t>
   </si>
 </sst>
 </file>
@@ -1319,10 +1325,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="0A0A0A"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FAFAFA"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="0E2841"/>
@@ -2970,7 +2976,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E23C0A35-DD33-4388-8FA3-25D5F19A7937}">
-  <dimension ref="B8:N40"/>
+  <dimension ref="B8:N42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="19.7109375" customWidth="1"/>
@@ -3684,11 +3690,21 @@
       <c r="N39" s="10"/>
     </row>
     <row r="40" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B40" s="5"/>
-      <c r="C40" s="12"/>
-      <c r="D40" s="10"/>
-      <c r="E40" s="10"/>
-      <c r="F40" s="10"/>
+      <c r="B40" s="5" t="s">
+        <v>229</v>
+      </c>
+      <c r="C40" s="12">
+        <v>17.79</v>
+      </c>
+      <c r="D40" s="10">
+        <v>36</v>
+      </c>
+      <c r="E40" s="10">
+        <v>36</v>
+      </c>
+      <c r="F40" s="10">
+        <v>12</v>
+      </c>
       <c r="G40" s="10"/>
       <c r="H40" s="10"/>
       <c r="I40" s="10"/>
@@ -3698,8 +3714,38 @@
       <c r="M40" s="10"/>
       <c r="N40" s="10"/>
     </row>
+    <row r="41" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B41" s="5"/>
+      <c r="C41" s="12"/>
+      <c r="D41" s="10"/>
+      <c r="E41" s="10"/>
+      <c r="F41" s="10"/>
+      <c r="G41" s="10"/>
+      <c r="H41" s="10"/>
+      <c r="I41" s="10"/>
+      <c r="J41" s="10"/>
+      <c r="K41" s="10"/>
+      <c r="L41" s="10"/>
+      <c r="M41" s="10"/>
+      <c r="N41" s="10"/>
+    </row>
+    <row r="42" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B42" s="5"/>
+      <c r="C42" s="12"/>
+      <c r="D42" s="10"/>
+      <c r="E42" s="10"/>
+      <c r="F42" s="10"/>
+      <c r="G42" s="10"/>
+      <c r="H42" s="10"/>
+      <c r="I42" s="10"/>
+      <c r="J42" s="10"/>
+      <c r="K42" s="10"/>
+      <c r="L42" s="10"/>
+      <c r="M42" s="10"/>
+      <c r="N42" s="10"/>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="C14:N40">
+  <conditionalFormatting sqref="C14:N42">
     <cfRule type="expression" dxfId="19" priority="1">
       <formula>ISNOTFORMULA(C14)</formula>
     </cfRule>
@@ -6734,7 +6780,9 @@
       <c r="H7" s="7" t="s">
         <v>225</v>
       </c>
-      <c r="I7" s="7"/>
+      <c r="I7" s="7" t="s">
+        <v>228</v>
+      </c>
       <c r="J7" s="7"/>
       <c r="K7" s="7"/>
       <c r="L7" s="7"/>
@@ -7105,12 +7153,16 @@
       <c r="P28" s="10"/>
     </row>
     <row r="29" spans="4:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D29" s="5"/>
+      <c r="D29" s="5" t="s">
+        <v>228</v>
+      </c>
       <c r="E29" s="12"/>
       <c r="F29" s="10"/>
       <c r="G29" s="10"/>
       <c r="H29" s="10"/>
-      <c r="I29" s="10"/>
+      <c r="I29" s="10">
+        <v>0.06</v>
+      </c>
       <c r="J29" s="10"/>
       <c r="K29" s="10"/>
       <c r="L29" s="10"/>

</xml_diff>

<commit_message>
Added more for computing the static margin.
</commit_message>
<xml_diff>
--- a/examples/F-16A B Block 10 and 15/Operator/F-16A Block 50.xlsx
+++ b/examples/F-16A B Block 10 and 15/Operator/F-16A Block 50.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\John Freeman\Desktop\Academics\VRMastersProgram\code\air-vehicle-design\examples\F-16A B Block 10 and 15\Operator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B838FC6B-90DB-411C-B3B4-C8E649BF7C29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90DDEDDF-7518-49DF-AA8D-7A1DD8FB17F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="384" windowWidth="23256" windowHeight="12720" firstSheet="1" activeTab="7" xr2:uid="{5F5D00AF-8D4A-4BC4-9FDA-F17071C88D94}"/>
   </bookViews>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="230">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="232">
   <si>
     <t>THIS IS FOR THE END USER</t>
   </si>
@@ -735,6 +735,12 @@
   </si>
   <si>
     <t>x location</t>
+  </si>
+  <si>
+    <t>Armaments</t>
+  </si>
+  <si>
+    <t/>
   </si>
 </sst>
 </file>
@@ -1002,7 +1008,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1050,6 +1056,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3715,8 +3724,12 @@
       <c r="N40" s="10"/>
     </row>
     <row r="41" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B41" s="5"/>
-      <c r="C41" s="12"/>
+      <c r="B41" s="5" t="s">
+        <v>228</v>
+      </c>
+      <c r="C41" s="12">
+        <v>0.06</v>
+      </c>
       <c r="D41" s="10"/>
       <c r="E41" s="10"/>
       <c r="F41" s="10"/>
@@ -6780,9 +6793,7 @@
       <c r="H7" s="7" t="s">
         <v>225</v>
       </c>
-      <c r="I7" s="7" t="s">
-        <v>228</v>
-      </c>
+      <c r="I7" s="7"/>
       <c r="J7" s="7"/>
       <c r="K7" s="7"/>
       <c r="L7" s="7"/>
@@ -6816,8 +6827,12 @@
       <c r="D9" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="E9" s="12"/>
-      <c r="F9" s="12"/>
+      <c r="E9" s="12">
+        <v>3652</v>
+      </c>
+      <c r="F9" s="12">
+        <v>26</v>
+      </c>
       <c r="G9" s="12"/>
       <c r="H9" s="12"/>
       <c r="I9" s="12"/>
@@ -6833,8 +6848,12 @@
       <c r="D10" s="4" t="s">
         <v>204</v>
       </c>
-      <c r="E10" s="12"/>
-      <c r="F10" s="12"/>
+      <c r="E10" s="12">
+        <v>648</v>
+      </c>
+      <c r="F10" s="12">
+        <v>41</v>
+      </c>
       <c r="G10" s="12"/>
       <c r="H10" s="12"/>
       <c r="I10" s="12"/>
@@ -6850,8 +6869,12 @@
       <c r="D11" s="4" t="s">
         <v>205</v>
       </c>
-      <c r="E11" s="12"/>
-      <c r="F11" s="12"/>
+      <c r="E11" s="12">
+        <v>360</v>
+      </c>
+      <c r="F11" s="12">
+        <v>40</v>
+      </c>
       <c r="G11" s="12"/>
       <c r="H11" s="12"/>
       <c r="I11" s="10"/>
@@ -6867,8 +6890,12 @@
       <c r="D12" s="4" t="s">
         <v>206</v>
       </c>
-      <c r="E12" s="12"/>
-      <c r="F12" s="12"/>
+      <c r="E12" s="12">
+        <v>186</v>
+      </c>
+      <c r="F12" s="12">
+        <v>29</v>
+      </c>
       <c r="G12" s="12"/>
       <c r="H12" s="12"/>
       <c r="I12" s="10"/>
@@ -6884,8 +6911,12 @@
       <c r="D13" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="E13" s="12"/>
-      <c r="F13" s="12"/>
+      <c r="E13" s="12">
+        <v>90</v>
+      </c>
+      <c r="F13" s="12">
+        <v>17</v>
+      </c>
       <c r="G13" s="12"/>
       <c r="H13" s="12"/>
       <c r="I13" s="10"/>
@@ -6901,8 +6932,12 @@
       <c r="D14" s="5" t="s">
         <v>207</v>
       </c>
-      <c r="E14" s="12"/>
-      <c r="F14" s="12"/>
+      <c r="E14" s="12">
+        <v>4730</v>
+      </c>
+      <c r="F14" s="12">
+        <v>33</v>
+      </c>
       <c r="G14" s="12"/>
       <c r="H14" s="12"/>
       <c r="I14" s="10"/>
@@ -6918,8 +6953,12 @@
       <c r="D15" s="5" t="s">
         <v>208</v>
       </c>
-      <c r="E15" s="12"/>
-      <c r="F15" s="12"/>
+      <c r="E15" s="12">
+        <v>1066</v>
+      </c>
+      <c r="F15" s="12">
+        <v>26</v>
+      </c>
       <c r="G15" s="12"/>
       <c r="H15" s="12"/>
       <c r="I15" s="10"/>
@@ -6935,8 +6974,12 @@
       <c r="D16" s="5" t="s">
         <v>209</v>
       </c>
-      <c r="E16" s="12"/>
-      <c r="F16" s="12"/>
+      <c r="E16" s="12">
+        <v>728</v>
+      </c>
+      <c r="F16" s="12">
+        <v>22</v>
+      </c>
       <c r="G16" s="12"/>
       <c r="H16" s="12"/>
       <c r="I16" s="10"/>
@@ -6952,8 +6995,12 @@
       <c r="D17" s="5" t="s">
         <v>210</v>
       </c>
-      <c r="E17" s="12"/>
-      <c r="F17" s="12"/>
+      <c r="E17" s="12">
+        <v>472</v>
+      </c>
+      <c r="F17" s="12">
+        <v>27</v>
+      </c>
       <c r="G17" s="12"/>
       <c r="H17" s="12"/>
       <c r="I17" s="10"/>
@@ -6969,8 +7016,12 @@
       <c r="D18" s="5" t="s">
         <v>211</v>
       </c>
-      <c r="E18" s="12"/>
-      <c r="F18" s="12"/>
+      <c r="E18" s="12">
+        <v>533</v>
+      </c>
+      <c r="F18" s="12">
+        <v>33</v>
+      </c>
       <c r="G18" s="12"/>
       <c r="H18" s="12"/>
       <c r="I18" s="10"/>
@@ -6986,8 +7037,12 @@
       <c r="D19" s="5" t="s">
         <v>212</v>
       </c>
-      <c r="E19" s="12"/>
-      <c r="F19" s="12"/>
+      <c r="E19" s="12">
+        <v>367</v>
+      </c>
+      <c r="F19" s="12">
+        <v>33</v>
+      </c>
       <c r="G19" s="12"/>
       <c r="H19" s="12"/>
       <c r="I19" s="10"/>
@@ -7003,8 +7058,12 @@
       <c r="D20" s="5" t="s">
         <v>213</v>
       </c>
-      <c r="E20" s="12"/>
-      <c r="F20" s="12"/>
+      <c r="E20" s="12">
+        <v>360</v>
+      </c>
+      <c r="F20" s="12">
+        <v>27</v>
+      </c>
       <c r="G20" s="12"/>
       <c r="H20" s="12"/>
       <c r="I20" s="10"/>
@@ -7020,8 +7079,12 @@
       <c r="D21" s="5" t="s">
         <v>214</v>
       </c>
-      <c r="E21" s="12"/>
-      <c r="F21" s="12"/>
+      <c r="E21" s="12">
+        <v>2016</v>
+      </c>
+      <c r="F21" s="12">
+        <v>20</v>
+      </c>
       <c r="G21" s="12"/>
       <c r="H21" s="12"/>
       <c r="I21" s="10"/>
@@ -7037,8 +7100,12 @@
       <c r="D22" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="E22" s="12"/>
-      <c r="F22" s="12"/>
+      <c r="E22" s="12">
+        <v>2541</v>
+      </c>
+      <c r="F22" s="12">
+        <v>15</v>
+      </c>
       <c r="G22" s="12"/>
       <c r="H22" s="12"/>
       <c r="I22" s="10"/>
@@ -7052,10 +7119,14 @@
     </row>
     <row r="23" spans="4:16" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D23" s="5" t="s">
-        <v>216</v>
-      </c>
-      <c r="E23" s="12"/>
-      <c r="F23" s="12"/>
+        <v>230</v>
+      </c>
+      <c r="E23" s="12">
+        <v>440</v>
+      </c>
+      <c r="F23" s="12">
+        <v>26</v>
+      </c>
       <c r="G23" s="12"/>
       <c r="H23" s="12"/>
       <c r="I23" s="10"/>
@@ -7067,14 +7138,18 @@
       <c r="O23" s="10"/>
       <c r="P23" s="10"/>
     </row>
-    <row r="24" spans="4:16" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="4:16" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D24" s="5" t="s">
-        <v>217</v>
-      </c>
-      <c r="E24" s="12"/>
-      <c r="F24" s="10"/>
-      <c r="G24" s="10"/>
-      <c r="H24" s="10"/>
+        <v>216</v>
+      </c>
+      <c r="E24" s="12">
+        <v>700</v>
+      </c>
+      <c r="F24" s="12">
+        <v>16</v>
+      </c>
+      <c r="G24" s="12"/>
+      <c r="H24" s="12"/>
       <c r="I24" s="10"/>
       <c r="J24" s="10"/>
       <c r="K24" s="10"/>
@@ -7086,10 +7161,14 @@
     </row>
     <row r="25" spans="4:16" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D25" s="5" t="s">
-        <v>218</v>
-      </c>
-      <c r="E25" s="12"/>
-      <c r="F25" s="10"/>
+        <v>217</v>
+      </c>
+      <c r="E25" s="12">
+        <v>2200</v>
+      </c>
+      <c r="F25" s="10">
+        <v>26</v>
+      </c>
       <c r="G25" s="10"/>
       <c r="H25" s="10"/>
       <c r="I25" s="10"/>
@@ -7101,12 +7180,16 @@
       <c r="O25" s="10"/>
       <c r="P25" s="10"/>
     </row>
-    <row r="26" spans="4:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="4:16" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D26" s="5" t="s">
-        <v>219</v>
-      </c>
-      <c r="E26" s="12"/>
-      <c r="F26" s="10"/>
+        <v>218</v>
+      </c>
+      <c r="E26" s="12">
+        <v>2200</v>
+      </c>
+      <c r="F26" s="10">
+        <v>26</v>
+      </c>
       <c r="G26" s="10"/>
       <c r="H26" s="10"/>
       <c r="I26" s="10"/>
@@ -7120,10 +7203,14 @@
     </row>
     <row r="27" spans="4:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D27" s="5" t="s">
-        <v>220</v>
-      </c>
-      <c r="E27" s="12"/>
-      <c r="F27" s="10"/>
+        <v>219</v>
+      </c>
+      <c r="E27" s="12">
+        <v>2098</v>
+      </c>
+      <c r="F27" s="10">
+        <v>24</v>
+      </c>
       <c r="G27" s="10"/>
       <c r="H27" s="10"/>
       <c r="I27" s="10"/>
@@ -7137,10 +7224,14 @@
     </row>
     <row r="28" spans="4:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D28" s="5" t="s">
-        <v>221</v>
-      </c>
-      <c r="E28" s="12"/>
-      <c r="F28" s="10"/>
+        <v>220</v>
+      </c>
+      <c r="E28" s="12">
+        <v>2098</v>
+      </c>
+      <c r="F28" s="10">
+        <v>26</v>
+      </c>
       <c r="G28" s="10"/>
       <c r="H28" s="10"/>
       <c r="I28" s="10"/>
@@ -7154,15 +7245,17 @@
     </row>
     <row r="29" spans="4:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D29" s="5" t="s">
-        <v>228</v>
-      </c>
-      <c r="E29" s="12"/>
-      <c r="F29" s="10"/>
+        <v>221</v>
+      </c>
+      <c r="E29" s="12">
+        <v>2098</v>
+      </c>
+      <c r="F29" s="10">
+        <v>28</v>
+      </c>
       <c r="G29" s="10"/>
       <c r="H29" s="10"/>
-      <c r="I29" s="10">
-        <v>0.06</v>
-      </c>
+      <c r="I29" s="10"/>
       <c r="J29" s="10"/>
       <c r="K29" s="10"/>
       <c r="L29" s="10"/>
@@ -7174,7 +7267,9 @@
     <row r="30" spans="4:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D30" s="5"/>
       <c r="E30" s="12"/>
-      <c r="F30" s="10"/>
+      <c r="F30" s="21" t="s">
+        <v>231</v>
+      </c>
       <c r="G30" s="10"/>
       <c r="H30" s="10"/>
       <c r="I30" s="10"/>

</xml_diff>

<commit_message>
Added SandCUtils. Added function to import both component weight and their cg locations.
</commit_message>
<xml_diff>
--- a/examples/F-16A B Block 10 and 15/Operator/F-16A Block 50.xlsx
+++ b/examples/F-16A B Block 10 and 15/Operator/F-16A Block 50.xlsx
@@ -1250,74 +1250,6 @@
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>

</xml_diff>

<commit_message>
Inconsistency fixes, bug fixes.
</commit_message>
<xml_diff>
--- a/examples/F-16A B Block 10 and 15/Operator/F-16A Block 50.xlsx
+++ b/examples/F-16A B Block 10 and 15/Operator/F-16A Block 50.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\John Freeman\Desktop\Academics\VRMastersProgram\code\air-vehicle-design\examples\F-16A B Block 10 and 15\Operator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90DDEDDF-7518-49DF-AA8D-7A1DD8FB17F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5C90E6B-BF10-485B-8608-97834C271CCA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="384" windowWidth="23256" windowHeight="12720" firstSheet="1" activeTab="7" xr2:uid="{5F5D00AF-8D4A-4BC4-9FDA-F17071C88D94}"/>
+    <workbookView xWindow="22932" yWindow="384" windowWidth="23256" windowHeight="12720" firstSheet="1" activeTab="6" xr2:uid="{5F5D00AF-8D4A-4BC4-9FDA-F17071C88D94}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -4928,8 +4928,7 @@
       </c>
       <c r="C17" s="12"/>
       <c r="D17" s="12">
-        <f>D16/D18</f>
-        <v>5.7142857142857144</v>
+        <v>0</v>
       </c>
       <c r="E17" s="12"/>
       <c r="F17" s="12"/>
@@ -4948,8 +4947,7 @@
       </c>
       <c r="C18" s="12"/>
       <c r="D18" s="12">
-        <f>Wings!E30</f>
-        <v>7.0000000000000007E-2</v>
+        <v>3.5</v>
       </c>
       <c r="E18" s="12"/>
       <c r="F18" s="12"/>

</xml_diff>

<commit_message>
Added control surface sizing.
</commit_message>
<xml_diff>
--- a/examples/F-16A B Block 10 and 15/Operator/F-16A Block 50.xlsx
+++ b/examples/F-16A B Block 10 and 15/Operator/F-16A Block 50.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\John Freeman\Desktop\Academics\VRMastersProgram\code\air-vehicle-design\examples\F-16A B Block 10 and 15\Operator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5C90E6B-BF10-485B-8608-97834C271CCA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EBFEBAD-02AB-4AFC-BB8F-E3ABA6C018E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="384" windowWidth="23256" windowHeight="12720" firstSheet="1" activeTab="6" xr2:uid="{5F5D00AF-8D4A-4BC4-9FDA-F17071C88D94}"/>
   </bookViews>
@@ -4928,7 +4928,8 @@
       </c>
       <c r="C17" s="12"/>
       <c r="D17" s="12">
-        <v>0</v>
+        <f>D16/D18</f>
+        <v>0.1142857142857143</v>
       </c>
       <c r="E17" s="12"/>
       <c r="F17" s="12"/>
@@ -5233,7 +5234,7 @@
       </c>
       <c r="C33" s="12"/>
       <c r="D33" s="10">
-        <v>1</v>
+        <v>1.0469999999999999</v>
       </c>
       <c r="E33" s="10"/>
       <c r="F33" s="10"/>

</xml_diff>

<commit_message>
Updated F16WeightLevel2 to actually do its job.
</commit_message>
<xml_diff>
--- a/examples/F-16A B Block 10 and 15/Operator/F-16A Block 50.xlsx
+++ b/examples/F-16A B Block 10 and 15/Operator/F-16A Block 50.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\John Freeman\Desktop\Academics\VRMastersProgram\code\air-vehicle-design\examples\F-16A B Block 10 and 15\Operator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19A2DDDB-6907-4616-B064-517782ED7816}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{901C11AA-C51A-4717-8CC7-DE513BA25844}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="384" windowWidth="23256" windowHeight="12720" firstSheet="1" activeTab="3" xr2:uid="{5F5D00AF-8D4A-4BC4-9FDA-F17071C88D94}"/>
+    <workbookView xWindow="22932" yWindow="384" windowWidth="23256" windowHeight="12720" firstSheet="1" activeTab="5" xr2:uid="{5F5D00AF-8D4A-4BC4-9FDA-F17071C88D94}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="232">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="232">
   <si>
     <t>THIS IS FOR THE END USER</t>
   </si>
@@ -4441,8 +4441,12 @@
       <c r="N20" s="10"/>
     </row>
     <row r="21" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="5"/>
-      <c r="C21" s="12"/>
+      <c r="B21" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="C21" s="12">
+        <v>3234</v>
+      </c>
       <c r="D21" s="12"/>
       <c r="E21" s="12"/>
       <c r="F21" s="12"/>

</xml_diff>